<commit_message>
Actualisation du 22/09/2026 10:11 UTC
</commit_message>
<xml_diff>
--- a/classeur/Analyse_football_paris_sportifs.xlsx
+++ b/classeur/Analyse_football_paris_sportifs.xlsx
@@ -452,7 +452,7 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Copie automatique du 2026-09-21T10:56+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
+          <t>Copie automatique du 2026-09-22T10:11+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fenetre : 2026-09-21 au 2026-09-28. Competitions : .</t>
+          <t>Fenetre : 2026-09-22 au 2026-09-29. Competitions : .</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualisation du 23/09/2026 10:13 UTC
</commit_message>
<xml_diff>
--- a/classeur/Analyse_football_paris_sportifs.xlsx
+++ b/classeur/Analyse_football_paris_sportifs.xlsx
@@ -452,7 +452,7 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Copie automatique du 2026-09-22T10:11+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
+          <t>Copie automatique du 2026-09-23T10:13+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fenetre : 2026-09-22 au 2026-09-29. Competitions : .</t>
+          <t>Fenetre : 2026-09-23 au 2026-09-30. Competitions : .</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualisation du 24/09/2026 10:20 UTC
</commit_message>
<xml_diff>
--- a/classeur/Analyse_football_paris_sportifs.xlsx
+++ b/classeur/Analyse_football_paris_sportifs.xlsx
@@ -452,7 +452,7 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Copie automatique du 2026-09-23T10:13+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
+          <t>Copie automatique du 2026-09-24T10:20+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fenetre : 2026-09-23 au 2026-09-30. Competitions : .</t>
+          <t>Fenetre : 2026-09-24 au 2026-10-01. Competitions : .</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualisation du 25/09/2026 10:23 UTC
</commit_message>
<xml_diff>
--- a/classeur/Analyse_football_paris_sportifs.xlsx
+++ b/classeur/Analyse_football_paris_sportifs.xlsx
@@ -452,7 +452,7 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Copie automatique du 2026-09-24T10:20+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
+          <t>Copie automatique du 2026-09-25T10:23+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fenetre : 2026-09-24 au 2026-10-01. Competitions : .</t>
+          <t>Fenetre : 2026-09-25 au 2026-10-02. Competitions : Brasileirao.</t>
         </is>
       </c>
     </row>
@@ -691,29 +691,29 @@
   <dimension ref="A1:X2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="9" customWidth="1" min="14" max="14"/>
-    <col width="9" customWidth="1" min="15" max="15"/>
-    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
     <col width="9" customWidth="1" min="17" max="17"/>
     <col width="9" customWidth="1" min="18" max="18"/>
     <col width="9" customWidth="1" min="19" max="19"/>
     <col width="9" customWidth="1" min="20" max="20"/>
-    <col width="9" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="21" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="15" customWidth="1" min="23" max="23"/>
     <col width="18" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
@@ -839,7 +839,102 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>2.165215499840775</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1.387745500189346</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.5108114321095949</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.2450462113718627</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.2441423565185424</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Victoire São Paulo</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Inter-champ.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2 - 1</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>0.8713233845326325</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.6888319388429962</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.6659966359698632</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="R2" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="S2" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U2" t="n">
+        <v>0.05164880067207411</v>
+      </c>
+      <c r="V2" t="n">
+        <v>1.168952129938766</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Pas de valeur</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -854,17 +949,17 @@
   <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -924,7 +1019,50 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>São Paulo - Santos</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0.7549537886281372</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1.251498194945848</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1.32458438524714</v>
+      </c>
+      <c r="I2" t="n">
+        <v>-0.05517669626435673</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualisation du 26/09/2026 10:03 UTC
</commit_message>
<xml_diff>
--- a/classeur/Analyse_football_paris_sportifs.xlsx
+++ b/classeur/Analyse_football_paris_sportifs.xlsx
@@ -452,7 +452,7 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Copie automatique du 2026-09-25T10:23+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
+          <t>Copie automatique du 2026-09-26T10:03+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fenetre : 2026-09-25 au 2026-10-02. Competitions : Brasileirao.</t>
+          <t>Fenetre : 2026-09-26 au 2026-10-03. Competitions : Brasileirao.</t>
         </is>
       </c>
     </row>
@@ -688,15 +688,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:X3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
@@ -935,6 +935,77 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Mineiro</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Bragantino</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1.873435177320872</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1.380053681163607</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.4891801195344466</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.228986687055412</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.2818331934101411</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Victoire Mineiro</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>0.8376459477287915</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.6311455230225416</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.6354764106404839</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Pas de cote</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -946,20 +1017,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="29" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1060,6 +1131,33 @@
       <c r="K2" t="inlineStr">
         <is>
           <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Mineiro - Bragantino</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualisation du 27/09/2026 10:41 UTC
</commit_message>
<xml_diff>
--- a/classeur/Analyse_football_paris_sportifs.xlsx
+++ b/classeur/Analyse_football_paris_sportifs.xlsx
@@ -452,7 +452,7 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Copie automatique du 2026-09-26T10:03+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
+          <t>Copie automatique du 2026-09-27T10:41+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fenetre : 2026-09-26 au 2026-10-03. Competitions : Brasileirao.</t>
+          <t>Fenetre : 2026-09-27 au 2026-10-04. Competitions : Brasileirao.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualisation du 28/09/2026 11:53 UTC
</commit_message>
<xml_diff>
--- a/classeur/Analyse_football_paris_sportifs.xlsx
+++ b/classeur/Analyse_football_paris_sportifs.xlsx
@@ -452,7 +452,7 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Copie automatique du 2026-09-27T10:41+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
+          <t>Copie automatique du 2026-09-28T11:53+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fenetre : 2026-09-27 au 2026-10-04. Competitions : Brasileirao.</t>
+          <t>Fenetre : 2026-09-28 au 2026-10-05. Competitions : Brasileirao.</t>
         </is>
       </c>
     </row>
@@ -872,13 +872,13 @@
         <v>1.387745500189346</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5108114321095949</v>
+        <v>0.5054503303984337</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2450462113718627</v>
+        <v>0.2454423912448603</v>
       </c>
       <c r="J2" t="n">
-        <v>0.2441423565185424</v>
+        <v>0.2491072783567059</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -905,13 +905,13 @@
         <v>0.6659966359698632</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.91</v>
+        <v>1.96</v>
       </c>
       <c r="R2" t="n">
         <v>3.2</v>
       </c>
       <c r="S2" t="n">
-        <v>3.63</v>
+        <v>3.5</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -919,10 +919,10 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0.05164880067207411</v>
+        <v>0.07917887398809698</v>
       </c>
       <c r="V2" t="n">
-        <v>1.168952129938766</v>
+        <v>1.196181685581194</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
@@ -1117,16 +1117,16 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.7549537886281372</v>
+        <v>0.7545576087551396</v>
       </c>
       <c r="G2" t="n">
-        <v>1.251498194945848</v>
+        <v>1.256410256410256</v>
       </c>
       <c r="H2" t="n">
-        <v>1.32458438524714</v>
+        <v>1.325279857226261</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.05517669626435673</v>
+        <v>-0.05196608130764524</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Actualisation du 29/09/2026 11:30 UTC
</commit_message>
<xml_diff>
--- a/classeur/Analyse_football_paris_sportifs.xlsx
+++ b/classeur/Analyse_football_paris_sportifs.xlsx
@@ -452,7 +452,7 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Copie automatique du 2026-09-28T11:53+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
+          <t>Copie automatique du 2026-09-29T11:30+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fenetre : 2026-09-28 au 2026-10-05. Competitions : Brasileirao.</t>
+          <t>Fenetre : 2026-09-29 au 2026-10-06. Competitions : Brasileirao.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualisation du 30/09/2026 11:18 UTC
</commit_message>
<xml_diff>
--- a/classeur/Analyse_football_paris_sportifs.xlsx
+++ b/classeur/Analyse_football_paris_sportifs.xlsx
@@ -452,7 +452,7 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Copie automatique du 2026-09-29T11:30+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
+          <t>Copie automatique du 2026-09-30T11:18+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fenetre : 2026-09-29 au 2026-10-06. Competitions : Brasileirao.</t>
+          <t>Fenetre : 2026-09-30 au 2026-10-07. Competitions : Brasileirao.</t>
         </is>
       </c>
     </row>
@@ -688,20 +688,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X3"/>
+  <dimension ref="A1:X8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
@@ -1006,6 +1006,461 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Bragantino</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Mirassol</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1.515210473535989</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2.180765627444329</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.3944833999030943</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.2320947428121561</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.3734218572847496</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Victoire Bragantino</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>1 - 2</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>0.8850690954809114</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.7138798779569785</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.6937450473114027</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="R4" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="S4" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U4" t="n">
+        <v>1.160007527713683</v>
+      </c>
+      <c r="V4" t="n">
+        <v>2.394549583880466</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Ecart suspect</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Corinthians</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1.897963915714285</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1.637780449186639</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.4426823621310089</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.2570919436845581</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.300225694184433</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Victoire Internacional</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>0.8696523292845325</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.6857114228613103</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.6866631300122457</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="R5" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="S5" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U5" t="n">
+        <v>0.1400727444693119</v>
+      </c>
+      <c r="V5" t="n">
+        <v>1.264693103914673</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Ecart suspect</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Clube do Remo</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Grêmio</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1.709145684387043</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1.886049231324674</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.3530780309948007</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.2222431048987616</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.4246788641064378</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Victoire Grêmio</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>0.8756066254830943</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.6963994203810919</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.6965342974634749</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Pas de cote</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Chapecoense</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1.892076895232119</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1.499705658642131</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.5090694790456718</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.2367287198083343</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.2542018011459941</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Victoire Vitória</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>0.8541312708503004</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.6586704189317067</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.6616033457763653</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="R7" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="S7" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U7" t="n">
+        <v>0.3602335659722968</v>
+      </c>
+      <c r="V7" t="n">
+        <v>1.507747905625524</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Ecart suspect</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>23:30</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Botafogo</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Vasco da Gama</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>2.084465151551401</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1.433418992861901</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.4317272932225192</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.2444857725984195</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.3237869341790614</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Victoire Botafogo</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Inter-champ.</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2 - 1</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>0.8677608400237566</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.682443995162441</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.6685677375928564</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="R8" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="S8" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U8" t="n">
+        <v>0.3884056659013422</v>
+      </c>
+      <c r="V8" t="n">
+        <v>1.543103336757135</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Ecart suspect</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1017,13 +1472,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
@@ -1158,6 +1613,192 @@
       <c r="K3" t="inlineStr">
         <is>
           <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Bragantino - Mirassol</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0.767905257187844</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.211683848797251</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1.30224398210544</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-0.06954160245899055</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Internacional - Corinthians</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>0.7429080563154419</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1.271086556169429</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1.346061590662567</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-0.05569955714748087</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Clube do Remo - Grêmio</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Vitória - Chapecoense</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>23:30</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Botafogo - Vasco da Gama</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>0.7555142274015807</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1.239859437751004</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1.323601811496353</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-0.06326855480099203</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualisation du 01/10/2026 11:45 UTC
</commit_message>
<xml_diff>
--- a/classeur/Analyse_football_paris_sportifs.xlsx
+++ b/classeur/Analyse_football_paris_sportifs.xlsx
@@ -452,7 +452,7 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Copie automatique du 2026-09-30T11:18+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
+          <t>Copie automatique du 2026-10-01T11:45+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fenetre : 2026-09-30 au 2026-10-07. Competitions : Brasileirao.</t>
+          <t>Fenetre : 2026-10-01 au 2026-10-08. Competitions : Brasileirao.</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X8"/>
+  <dimension ref="A1:X11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -705,7 +705,7 @@
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
     <col width="20" customWidth="1" min="16" max="16"/>
     <col width="9" customWidth="1" min="17" max="17"/>
     <col width="9" customWidth="1" min="18" max="18"/>
@@ -872,13 +872,13 @@
         <v>1.387745500189346</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5054503303984337</v>
+        <v>0.5008596253857878</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2454423912448603</v>
+        <v>0.2454500705774342</v>
       </c>
       <c r="J2" t="n">
-        <v>0.2491072783567059</v>
+        <v>0.2536903040367781</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -905,13 +905,13 @@
         <v>0.6659966359698632</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.96</v>
+        <v>2</v>
       </c>
       <c r="R2" t="n">
         <v>3.2</v>
       </c>
       <c r="S2" t="n">
-        <v>3.5</v>
+        <v>3.38</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -919,10 +919,10 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0.07917887398809698</v>
+        <v>0.1012029326409154</v>
       </c>
       <c r="V2" t="n">
-        <v>1.196181685581194</v>
+        <v>1.220527066984032</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
@@ -1398,13 +1398,13 @@
         <v>1.433418992861901</v>
       </c>
       <c r="H8" t="n">
-        <v>0.4317272932225192</v>
+        <v>0.4364315317281445</v>
       </c>
       <c r="I8" t="n">
-        <v>0.2444857725984195</v>
+        <v>0.2437313244114749</v>
       </c>
       <c r="J8" t="n">
-        <v>0.3237869341790614</v>
+        <v>0.3198371438603806</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -1431,13 +1431,13 @@
         <v>0.6685677375928564</v>
       </c>
       <c r="Q8" t="n">
-        <v>2.65</v>
+        <v>2.58</v>
       </c>
       <c r="R8" t="n">
-        <v>3.28</v>
+        <v>3.3</v>
       </c>
       <c r="S8" t="n">
-        <v>2.33</v>
+        <v>2.38</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
@@ -1445,10 +1445,10 @@
         </is>
       </c>
       <c r="U8" t="n">
-        <v>0.3884056659013422</v>
+        <v>0.3517307992548917</v>
       </c>
       <c r="V8" t="n">
-        <v>1.543103336757135</v>
+        <v>1.501496177425457</v>
       </c>
       <c r="W8" t="inlineStr">
         <is>
@@ -1458,6 +1458,269 @@
       <c r="X8" t="inlineStr">
         <is>
           <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Cruzeiro</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1.580980015688877</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1.159987529777633</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.4804543186759034</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.2623809911870489</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.2571646901370476</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Victoire Cruzeiro</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Inter-champ.</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>0.7610438446761185</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.5163567578630177</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.5476103789188483</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="R9" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="S9" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U9" t="n">
+        <v>0.05347467446740173</v>
+      </c>
+      <c r="V9" t="n">
+        <v>1.169258159613181</v>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Pas de valeur</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Flamengo</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>0.7450848416095041</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1.745175144772266</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.1937762336679176</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.246407017957737</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.5598167483743455</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Victoire Flamengo</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Inter-champ.</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>0 - 1</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>0.7128528166092001</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.4536847195661908</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0.4357353785333726</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="R10" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="S10" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U10" t="n">
+        <v>0.0811962476170609</v>
+      </c>
+      <c r="V10" t="n">
+        <v>1.200588745427882</v>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Pas de valeur</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Paranaense</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Mineiro</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1.924079535911576</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1.347175907780612</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.507674186872526</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.2257175072275834</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.2666083058998904</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Victoire Paranaense</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>0.8398353910692622</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.6347659434140894</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.6339424137952552</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Pas de cote</t>
         </is>
       </c>
     </row>
@@ -1472,7 +1735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1572,16 +1835,16 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.7545576087551396</v>
+        <v>0.7545499294225658</v>
       </c>
       <c r="G2" t="n">
-        <v>1.256410256410256</v>
+        <v>1.256505576208178</v>
       </c>
       <c r="H2" t="n">
-        <v>1.325279857226261</v>
+        <v>1.325293345087541</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.05196608130764524</v>
+        <v>-0.05190380615305856</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -1785,20 +2048,135 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.7555142274015807</v>
+        <v>0.7562686755885252</v>
       </c>
       <c r="G8" t="n">
-        <v>1.239859437751004</v>
+        <v>1.237983870967742</v>
       </c>
       <c r="H8" t="n">
-        <v>1.323601811496353</v>
+        <v>1.322281395856842</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.06326855480099203</v>
+        <v>-0.0637515775032701</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Cruzeiro - São Paulo</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>0.7376190088129509</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1.235168738898757</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1.355713434784305</v>
+      </c>
+      <c r="I9" t="n">
+        <v>-0.08891605909675637</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Santos - Flamengo</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>0.7535929820422631</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1.212544483985765</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1.326976264149867</v>
+      </c>
+      <c r="I10" t="n">
+        <v>-0.08623498645427019</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Paranaense - Mineiro</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualisation du 02/10/2026 11:15 UTC
</commit_message>
<xml_diff>
--- a/classeur/Analyse_football_paris_sportifs.xlsx
+++ b/classeur/Analyse_football_paris_sportifs.xlsx
@@ -452,7 +452,7 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Copie automatique du 2026-10-01T11:45+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
+          <t>Copie automatique du 2026-10-02T11:15+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fenetre : 2026-10-01 au 2026-10-08. Competitions : Brasileirao.</t>
+          <t>Fenetre : 2026-10-02 au 2026-10-09. Competitions : Brasileirao, Bundesliga, Championship, Eredivisie, Liga, Ligue 1, Primeira Liga.</t>
         </is>
       </c>
     </row>
@@ -688,30 +688,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X11"/>
+  <dimension ref="A1:X20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
     <col width="21" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
     <col width="9" customWidth="1" min="17" max="17"/>
     <col width="9" customWidth="1" min="18" max="18"/>
     <col width="9" customWidth="1" min="19" max="19"/>
     <col width="9" customWidth="1" min="20" max="20"/>
-    <col width="21" customWidth="1" min="21" max="21"/>
+    <col width="23" customWidth="1" min="21" max="21"/>
     <col width="20" customWidth="1" min="22" max="22"/>
     <col width="15" customWidth="1" min="23" max="23"/>
     <col width="18" customWidth="1" min="24" max="24"/>
@@ -872,13 +872,13 @@
         <v>1.387745500189346</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5008596253857878</v>
+        <v>0.5112234042296981</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2454500705774342</v>
+        <v>0.2444174715522009</v>
       </c>
       <c r="J2" t="n">
-        <v>0.2536903040367781</v>
+        <v>0.2443591242181009</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -905,13 +905,13 @@
         <v>0.6659966359698632</v>
       </c>
       <c r="Q2" t="n">
-        <v>2</v>
+        <v>1.91</v>
       </c>
       <c r="R2" t="n">
-        <v>3.2</v>
+        <v>3.22</v>
       </c>
       <c r="S2" t="n">
-        <v>3.38</v>
+        <v>3.63</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -919,10 +919,10 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0.1012029326409154</v>
+        <v>0.05164880067207411</v>
       </c>
       <c r="V2" t="n">
-        <v>1.220527066984032</v>
+        <v>1.166910886148641</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
@@ -1302,13 +1302,13 @@
         <v>1.499705658642131</v>
       </c>
       <c r="H7" t="n">
-        <v>0.5090694790456718</v>
+        <v>0.5137402269894117</v>
       </c>
       <c r="I7" t="n">
-        <v>0.2367287198083343</v>
+        <v>0.2355224429767717</v>
       </c>
       <c r="J7" t="n">
-        <v>0.2542018011459941</v>
+        <v>0.2507373300338167</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -1335,13 +1335,13 @@
         <v>0.6616033457763653</v>
       </c>
       <c r="Q7" t="n">
-        <v>1.64</v>
+        <v>1.61</v>
       </c>
       <c r="R7" t="n">
-        <v>3.65</v>
+        <v>3.68</v>
       </c>
       <c r="S7" t="n">
-        <v>4.45</v>
+        <v>4.6</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
@@ -1349,10 +1349,10 @@
         </is>
       </c>
       <c r="U7" t="n">
-        <v>0.3602335659722968</v>
+        <v>0.4060841356118123</v>
       </c>
       <c r="V7" t="n">
-        <v>1.507747905625524</v>
+        <v>1.561102728202556</v>
       </c>
       <c r="W7" t="inlineStr">
         <is>
@@ -1398,13 +1398,13 @@
         <v>1.433418992861901</v>
       </c>
       <c r="H8" t="n">
-        <v>0.4364315317281445</v>
+        <v>0.4317269590703463</v>
       </c>
       <c r="I8" t="n">
-        <v>0.2437313244114749</v>
+        <v>0.2436542505795293</v>
       </c>
       <c r="J8" t="n">
-        <v>0.3198371438603806</v>
+        <v>0.3246187903501244</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -1431,13 +1431,13 @@
         <v>0.6685677375928564</v>
       </c>
       <c r="Q8" t="n">
-        <v>2.58</v>
+        <v>2.65</v>
       </c>
       <c r="R8" t="n">
         <v>3.3</v>
       </c>
       <c r="S8" t="n">
-        <v>2.38</v>
+        <v>2.32</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
@@ -1445,10 +1445,10 @@
         </is>
       </c>
       <c r="U8" t="n">
-        <v>0.3517307992548917</v>
+        <v>0.3884056659013422</v>
       </c>
       <c r="V8" t="n">
-        <v>1.501496177425457</v>
+        <v>1.543106374105862</v>
       </c>
       <c r="W8" t="inlineStr">
         <is>
@@ -1721,6 +1721,845 @@
       <c r="W11" t="inlineStr">
         <is>
           <t>Pas de cote</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Fluminense</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Coritiba</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>2.282328654522728</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1.412574734844074</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.5978818716466003</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.2120191042052957</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.190099024148104</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Victoire Fluminense</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Elevee</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2 - 1</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>0.8849314308165422</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.7136953959838477</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.680888218550539</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="R12" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="S12" t="n">
+        <v>6</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U12" t="n">
+        <v>0.3786813259889474</v>
+      </c>
+      <c r="V12" t="n">
+        <v>1.527612950709976</v>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Ecart suspect</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Palmeiras</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Bahia</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>2.020364434899521</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.8002380715213437</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.6256659510642397</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.2160277085279048</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.1583063404078554</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Victoire Palmeiras</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Elevee</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2 - 0</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>0.7743307198682685</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.5354386975513514</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0.4796664818279436</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="R13" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="S13" t="n">
+        <v>5</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U13" t="n">
+        <v>-0.008551577712773706</v>
+      </c>
+      <c r="V13" t="n">
+        <v>1.103985687378819</v>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Pas de valeur</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Primeira Liga</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Moreirense</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Gil Vicente</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1.132066961647919</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1.708738690393662</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.259827275277081</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.2677674611251255</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.4724052635977934</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Victoire Gil Vicente</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>0.7780372156627533</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.5402153251103675</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0.5571766210366204</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="R14" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="S14" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U14" t="n">
+        <v>0.0278976304496843</v>
+      </c>
+      <c r="V14" t="n">
+        <v>1.154853259516969</v>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Pas de valeur</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>PSV</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Heerenveen</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>3.812898125222089</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1.633258249698224</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.7616468648318044</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.1252487350968674</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.1131044000713283</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Victoire PSV</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Elevee</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>3 - 1</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>0.972681750158093</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.9080556930107717</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0.7874392842670056</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="R15" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="S15" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U15" t="n">
+        <v>-0.02917852299273083</v>
+      </c>
+      <c r="V15" t="n">
+        <v>1.08423079980781</v>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Pas de valeur</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Borussia Dortmund</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Werder Breme</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>3.02447137871115</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.8062160515833473</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.7549641904356523</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.1447292148007416</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.100306594763606</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Victoire Borussia Dortmund</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Elevee</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>3 - 0</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>0.8962252431546965</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.7359413251415683</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0.5276165410477873</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="R16" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="S16" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U16" t="n">
+        <v>0.07372457445940883</v>
+      </c>
+      <c r="V16" t="n">
+        <v>1.167877849250974</v>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>Pas de valeur</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Ligue 1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Lens</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Lyon</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1.766608714336989</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1.58189971181059</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.4268704860825735</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.2420585735532551</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.3310709403641713</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Victoire Lens</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>0.849170985736324</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.6502210095405224</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0.6606042852093651</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="R17" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="S17" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U17" t="n">
+        <v>0.002606209369826473</v>
+      </c>
+      <c r="V17" t="n">
+        <v>1.092633477319896</v>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Pas de valeur</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>West Ham</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>QPR</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>3.171293367672211</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1.62697477653877</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.6803998984558641</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.1514448541932283</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.1681552473509074</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Victoire West Ham</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Elevee</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>3 - 1</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>0.9530279702766596</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0.8572303824194248</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0.770606811774713</v>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>Pas de cote</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Liga</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Malaga</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Espanyol</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1.505717205946246</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1.631360136729939</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.3575929248361211</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.2659585136395792</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.3764485615242997</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Victoire Espanyol</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>0.8225438804761739</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.606809015243296</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0.6280204070928681</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="R19" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="S19" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U19" t="n">
+        <v>0.077809915226976</v>
+      </c>
+      <c r="V19" t="n">
+        <v>1.17489442477738</v>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>Pas de valeur</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Primeira Liga</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Sporting CP</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>1.36306095859323</v>
+      </c>
+      <c r="G20" t="n">
+        <v>2.236828658194281</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.2537373855662913</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.2400243715370043</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.5062382428967045</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Victoire Sporting CP</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>1 - 2</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>0.8759634896036849</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0.6972265874252896</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0.6663182430647827</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="R20" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="S20" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U20" t="n">
+        <v>0.1524286107423656</v>
+      </c>
+      <c r="V20" t="n">
+        <v>1.290840405311452</v>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>Ecart suspect</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>Betclic</t>
         </is>
       </c>
     </row>
@@ -1735,18 +2574,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
     <col width="29" customWidth="1" min="11" max="11"/>
   </cols>
@@ -1835,16 +2674,16 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.7545499294225658</v>
+        <v>0.7555825284477991</v>
       </c>
       <c r="G2" t="n">
-        <v>1.256505576208178</v>
+        <v>1.251498194945848</v>
       </c>
       <c r="H2" t="n">
-        <v>1.325293345087541</v>
+        <v>1.323482164224086</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.05190380615305856</v>
+        <v>-0.05438982951495941</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -2048,16 +2887,16 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.7562686755885252</v>
+        <v>0.7563457494204707</v>
       </c>
       <c r="G8" t="n">
-        <v>1.237983870967742</v>
+        <v>1.237022132796781</v>
       </c>
       <c r="H8" t="n">
-        <v>1.322281395856842</v>
+        <v>1.322146651536315</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.0637515775032701</v>
+        <v>-0.0643835679201098</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -2177,6 +3016,317 @@
       <c r="K11" t="inlineStr">
         <is>
           <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Fluminense - Coritiba</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Palmeiras - Bahia</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Primeira Liga</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Moreirense - Gil Vicente</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>0.7322325388748745</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1.256848030018762</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1.365686372715106</v>
+      </c>
+      <c r="I14" t="n">
+        <v>-0.07969497599947772</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>PSV - Heerenveen</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Borussia Dortmund - Werder Breme</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Ligue 1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Lens - Lyon</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>0.7579414264467448</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1.228031809145129</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1.319363165948105</v>
+      </c>
+      <c r="I17" t="n">
+        <v>-0.06922381885456408</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>West Ham - QPR</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Liga</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Malaga - Espanyol</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>0.7340414863604208</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1.294305019305019</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1.362320820527835</v>
+      </c>
+      <c r="I19" t="n">
+        <v>-0.04992641982559065</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Primeira Liga</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Braga - Sporting CP</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>0.7599756284629957</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1.233795761078998</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1.315831669526612</v>
+      </c>
+      <c r="I20" t="n">
+        <v>-0.06234529107900832</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualisation du 05/10/2026 12:29 UTC
</commit_message>
<xml_diff>
--- a/classeur/Analyse_football_paris_sportifs.xlsx
+++ b/classeur/Analyse_football_paris_sportifs.xlsx
@@ -452,7 +452,7 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Copie automatique du 2026-10-04T11:14+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
+          <t>Copie automatique du 2026-10-05T12:29+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fenetre : 2026-10-04 au 2026-10-11. Competitions : Brasileirao, Bundesliga, Championship, Eredivisie, Liga, Ligue 1, Premier League, Primeira Liga, Serie A.</t>
+          <t>Fenetre : 2026-10-05 au 2026-10-12. Competitions : Brasileirao, Bundesliga, Championship, Eredivisie, Liga, Ligue 1, Premier League, Primeira Liga, Serie A.</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X91"/>
+  <dimension ref="A1:X99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -872,13 +872,13 @@
         <v>2.015729155698191</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4106378319513702</v>
+        <v>0.4069010970172698</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2369872395277625</v>
+        <v>0.2377231391680767</v>
       </c>
       <c r="J2" t="n">
-        <v>0.3523749285208673</v>
+        <v>0.3553757638146535</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -905,13 +905,13 @@
         <v>0.6846093035344661</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.72</v>
+        <v>1.74</v>
       </c>
       <c r="R2" t="n">
-        <v>3.53</v>
+        <v>3.5</v>
       </c>
       <c r="S2" t="n">
-        <v>4.1</v>
+        <v>3.98</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -919,10 +919,10 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0.9874227118498484</v>
+        <v>0.9292542422347312</v>
       </c>
       <c r="V2" t="n">
-        <v>2.203224834448569</v>
+        <v>2.144719550456027</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
@@ -968,13 +968,13 @@
         <v>1.51525557507413</v>
       </c>
       <c r="H3" t="n">
-        <v>0.4619253425478309</v>
+        <v>0.4574457965271893</v>
       </c>
       <c r="I3" t="n">
-        <v>0.2564371297078503</v>
+        <v>0.2549185436785928</v>
       </c>
       <c r="J3" t="n">
-        <v>0.2816375277443188</v>
+        <v>0.2876356597942179</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -1001,24 +1001,24 @@
         <v>0.6721505377373731</v>
       </c>
       <c r="Q3" t="n">
-        <v>2.03</v>
+        <v>2.07</v>
       </c>
       <c r="R3" t="n">
-        <v>3.1</v>
+        <v>3.13</v>
       </c>
       <c r="S3" t="n">
-        <v>3.4</v>
+        <v>3.25</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="U3" t="n">
-        <v>0.01367321267653576</v>
+        <v>-0.006853855393164188</v>
       </c>
       <c r="V3" t="n">
-        <v>1.124476949312382</v>
+        <v>1.102663263030486</v>
       </c>
       <c r="W3" t="inlineStr">
         <is>
@@ -1686,13 +1686,13 @@
         <v>0.7403710307211662</v>
       </c>
       <c r="H11" t="n">
-        <v>0.6396167886850987</v>
+        <v>0.6449614567710117</v>
       </c>
       <c r="I11" t="n">
-        <v>0.2109970594153197</v>
+        <v>0.2095448577541949</v>
       </c>
       <c r="J11" t="n">
-        <v>0.1493861518995817</v>
+        <v>0.1454936854747935</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1719,13 +1719,13 @@
         <v>0.4599427603142682</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.51</v>
+        <v>1.49</v>
       </c>
       <c r="R11" t="n">
-        <v>3.98</v>
+        <v>4.05</v>
       </c>
       <c r="S11" t="n">
-        <v>5</v>
+        <v>5.25</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
@@ -1733,10 +1733,10 @@
         </is>
       </c>
       <c r="U11" t="n">
-        <v>0.03357995190222018</v>
+        <v>0.01989015121477355</v>
       </c>
       <c r="V11" t="n">
-        <v>1.150899480004589</v>
+        <v>1.130579553774913</v>
       </c>
       <c r="W11" t="inlineStr">
         <is>
@@ -1782,13 +1782,13 @@
         <v>1.580905321131236</v>
       </c>
       <c r="H12" t="n">
-        <v>0.2745930234680899</v>
+        <v>0.2777635086694654</v>
       </c>
       <c r="I12" t="n">
-        <v>0.2729189615436902</v>
+        <v>0.2746335102641381</v>
       </c>
       <c r="J12" t="n">
-        <v>0.45248801498822</v>
+        <v>0.4476029810663965</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Moyenne</t>
+          <t>Faible</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1815,13 +1815,13 @@
         <v>0.5498063854656206</v>
       </c>
       <c r="Q12" t="n">
-        <v>3.3</v>
+        <v>3.23</v>
       </c>
       <c r="R12" t="n">
-        <v>3.05</v>
+        <v>3.02</v>
       </c>
       <c r="S12" t="n">
-        <v>2.03</v>
+        <v>2.08</v>
       </c>
       <c r="T12" t="inlineStr">
         <is>
@@ -1829,10 +1829,10 @@
         </is>
       </c>
       <c r="U12" t="n">
-        <v>-0.05296639890518362</v>
+        <v>-0.02964044813930133</v>
       </c>
       <c r="V12" t="n">
-        <v>1.064001714468372</v>
+        <v>1.088251039094053</v>
       </c>
       <c r="W12" t="inlineStr">
         <is>
@@ -2237,13 +2237,13 @@
         <v>1.509315576065982</v>
       </c>
       <c r="H17" t="n">
-        <v>0.371714464295635</v>
+        <v>0.3654299432894552</v>
       </c>
       <c r="I17" t="n">
-        <v>0.2732221105210015</v>
+        <v>0.2736446477362579</v>
       </c>
       <c r="J17" t="n">
-        <v>0.3550634251833633</v>
+        <v>0.3609254089742868</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -2270,13 +2270,13 @@
         <v>0.6165787364946821</v>
       </c>
       <c r="Q17" t="n">
-        <v>2.53</v>
+        <v>2.63</v>
       </c>
       <c r="R17" t="n">
         <v>2.98</v>
       </c>
       <c r="S17" t="n">
-        <v>2.63</v>
+        <v>2.55</v>
       </c>
       <c r="T17" t="inlineStr">
         <is>
@@ -2284,10 +2284,10 @@
         </is>
       </c>
       <c r="U17" t="n">
-        <v>-0.01916983873854672</v>
+        <v>0.01959815182514713</v>
       </c>
       <c r="V17" t="n">
-        <v>1.089756768458378</v>
+        <v>1.129669348931196</v>
       </c>
       <c r="W17" t="inlineStr">
         <is>
@@ -2333,13 +2333,13 @@
         <v>2.069488066301995</v>
       </c>
       <c r="H18" t="n">
-        <v>0.2698562427853091</v>
+        <v>0.2623284018963855</v>
       </c>
       <c r="I18" t="n">
-        <v>0.2460080734533724</v>
+        <v>0.2443568851071289</v>
       </c>
       <c r="J18" t="n">
-        <v>0.4841356837613185</v>
+        <v>0.4933147129964857</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -2366,13 +2366,13 @@
         <v>0.661675608838571</v>
       </c>
       <c r="Q18" t="n">
-        <v>3.17</v>
+        <v>3.35</v>
       </c>
       <c r="R18" t="n">
-        <v>3.23</v>
+        <v>3.27</v>
       </c>
       <c r="S18" t="n">
-        <v>2.02</v>
+        <v>1.94</v>
       </c>
       <c r="T18" t="inlineStr">
         <is>
@@ -2380,10 +2380,10 @@
         </is>
       </c>
       <c r="U18" t="n">
-        <v>0.06313427183540665</v>
+        <v>0.02102994423796489</v>
       </c>
       <c r="V18" t="n">
-        <v>1.190821419708147</v>
+        <v>1.143330726110962</v>
       </c>
       <c r="W18" t="inlineStr">
         <is>
@@ -2596,13 +2596,13 @@
         <v>1.44238685094107</v>
       </c>
       <c r="H21" t="n">
-        <v>0.3244528598730261</v>
+        <v>0.3284511572624188</v>
       </c>
       <c r="I21" t="n">
-        <v>0.2693875089935822</v>
+        <v>0.2703770343386609</v>
       </c>
       <c r="J21" t="n">
-        <v>0.4061596311333917</v>
+        <v>0.4011718083989203</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -2629,13 +2629,13 @@
         <v>0.5751971361758307</v>
       </c>
       <c r="Q21" t="n">
-        <v>3.03</v>
+        <v>2.95</v>
       </c>
       <c r="R21" t="n">
-        <v>3.1</v>
+        <v>3.08</v>
       </c>
       <c r="S21" t="n">
-        <v>2.05</v>
+        <v>2.1</v>
       </c>
       <c r="T21" t="inlineStr">
         <is>
@@ -2643,14 +2643,14 @@
         </is>
       </c>
       <c r="U21" t="n">
-        <v>0.08931327274633749</v>
+        <v>0.06055252627118679</v>
       </c>
       <c r="V21" t="n">
-        <v>1.242273037413601</v>
+        <v>1.208869579251808</v>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>PARI VALUE</t>
+          <t>Pas de valeur</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
@@ -2692,13 +2692,13 @@
         <v>0.7209491974602661</v>
       </c>
       <c r="H22" t="n">
-        <v>0.6930842931594754</v>
+        <v>0.6984371468110943</v>
       </c>
       <c r="I22" t="n">
-        <v>0.1891587457647037</v>
+        <v>0.1864689635676626</v>
       </c>
       <c r="J22" t="n">
-        <v>0.1177569610758209</v>
+        <v>0.1150938896212431</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -2725,13 +2725,13 @@
         <v>0.4599198685627431</v>
       </c>
       <c r="Q22" t="n">
-        <v>1.37</v>
+        <v>1.34</v>
       </c>
       <c r="R22" t="n">
-        <v>4.65</v>
+        <v>4.75</v>
       </c>
       <c r="S22" t="n">
-        <v>7</v>
+        <v>7.25</v>
       </c>
       <c r="T22" t="inlineStr">
         <is>
@@ -2739,10 +2739,10 @@
         </is>
       </c>
       <c r="U22" t="n">
-        <v>-0.02020363110920542</v>
+        <v>-0.04165902604841998</v>
       </c>
       <c r="V22" t="n">
-        <v>1.065859637684346</v>
+        <v>1.049120787747627</v>
       </c>
       <c r="W22" t="inlineStr">
         <is>
@@ -2884,13 +2884,13 @@
         <v>1.337395419164045</v>
       </c>
       <c r="H24" t="n">
-        <v>0.35820267215576</v>
+        <v>0.3592269051342017</v>
       </c>
       <c r="I24" t="n">
-        <v>0.2691293261578888</v>
+        <v>0.2687133541436557</v>
       </c>
       <c r="J24" t="n">
-        <v>0.3726680016863512</v>
+        <v>0.3720597407221425</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -2917,7 +2917,7 @@
         <v>0.584803544793031</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.05</v>
+        <v>3.02</v>
       </c>
       <c r="R24" t="n">
         <v>3.1</v>
@@ -2931,10 +2931,10 @@
         </is>
       </c>
       <c r="U24" t="n">
-        <v>0.2938879428834302</v>
+        <v>0.281161176232118</v>
       </c>
       <c r="V24" t="n">
-        <v>1.451933263785608</v>
+        <v>1.441824663371754</v>
       </c>
       <c r="W24" t="inlineStr">
         <is>
@@ -3172,13 +3172,13 @@
         <v>2.109890993669715</v>
       </c>
       <c r="H27" t="n">
-        <v>0.3614983388452696</v>
+        <v>0.3590394617213403</v>
       </c>
       <c r="I27" t="n">
-        <v>0.229274137844593</v>
+        <v>0.2295960344137179</v>
       </c>
       <c r="J27" t="n">
-        <v>0.4092275233101375</v>
+        <v>0.4113645038649419</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -3205,13 +3205,13 @@
         <v>0.7011060068226381</v>
       </c>
       <c r="Q27" t="n">
-        <v>2.12</v>
+        <v>2.15</v>
       </c>
       <c r="R27" t="n">
         <v>3.73</v>
       </c>
       <c r="S27" t="n">
-        <v>2.85</v>
+        <v>2.82</v>
       </c>
       <c r="T27" t="inlineStr">
         <is>
@@ -3219,10 +3219,10 @@
         </is>
       </c>
       <c r="U27" t="n">
-        <v>0.4157308001423268</v>
+        <v>0.4008283706671443</v>
       </c>
       <c r="V27" t="n">
-        <v>1.544097689745437</v>
+        <v>1.523852932485023</v>
       </c>
       <c r="W27" t="inlineStr">
         <is>
@@ -3268,13 +3268,13 @@
         <v>1.1803161511297</v>
       </c>
       <c r="H28" t="n">
-        <v>0.6972747424243124</v>
+        <v>0.6952380496130295</v>
       </c>
       <c r="I28" t="n">
-        <v>0.1650481538842581</v>
+        <v>0.1662937834007238</v>
       </c>
       <c r="J28" t="n">
-        <v>0.1376771036914296</v>
+        <v>0.1384681669862467</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -3304,10 +3304,10 @@
         <v>1.38</v>
       </c>
       <c r="R28" t="n">
-        <v>5.1</v>
+        <v>5</v>
       </c>
       <c r="S28" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="T28" t="inlineStr">
         <is>
@@ -3318,7 +3318,7 @@
         <v>0.002522355577379676</v>
       </c>
       <c r="V28" t="n">
-        <v>1.08738641309743</v>
+        <v>1.094057005434445</v>
       </c>
       <c r="W28" t="inlineStr">
         <is>
@@ -3364,13 +3364,13 @@
         <v>4.091636529830818</v>
       </c>
       <c r="H29" t="n">
-        <v>0.08145453922868484</v>
+        <v>0.07902164692102759</v>
       </c>
       <c r="I29" t="n">
-        <v>0.1045286950811523</v>
+        <v>0.1026956405920637</v>
       </c>
       <c r="J29" t="n">
-        <v>0.8140167656901628</v>
+        <v>0.8182827124869088</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -3397,13 +3397,13 @@
         <v>0.7015799731548024</v>
       </c>
       <c r="Q29" t="n">
-        <v>9.25</v>
+        <v>9.75</v>
       </c>
       <c r="R29" t="n">
-        <v>7.5</v>
+        <v>7.75</v>
       </c>
       <c r="S29" t="n">
-        <v>1.18</v>
+        <v>1.17</v>
       </c>
       <c r="T29" t="inlineStr">
         <is>
@@ -3411,10 +3411,10 @@
         </is>
       </c>
       <c r="U29" t="n">
-        <v>0.002720805530018078</v>
+        <v>-0.00577682841515148</v>
       </c>
       <c r="V29" t="n">
-        <v>1.091861751167456</v>
+        <v>1.080021862708658</v>
       </c>
       <c r="W29" t="inlineStr">
         <is>
@@ -4224,13 +4224,13 @@
         <v>1.34184830221176</v>
       </c>
       <c r="H39" t="n">
-        <v>0.4088969443820698</v>
+        <v>0.4079097160281986</v>
       </c>
       <c r="I39" t="n">
-        <v>0.2522729022758027</v>
+        <v>0.2520033377587345</v>
       </c>
       <c r="J39" t="n">
-        <v>0.3388301533421275</v>
+        <v>0.3400869462130669</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -4257,13 +4257,13 @@
         <v>0.6148596020833412</v>
       </c>
       <c r="Q39" t="n">
-        <v>2.67</v>
+        <v>2.68</v>
       </c>
       <c r="R39" t="n">
         <v>3.43</v>
       </c>
       <c r="S39" t="n">
-        <v>2.37</v>
+        <v>2.35</v>
       </c>
       <c r="T39" t="inlineStr">
         <is>
@@ -4271,10 +4271,10 @@
         </is>
       </c>
       <c r="U39" t="n">
-        <v>0.264407201960579</v>
+        <v>0.2691428094585586</v>
       </c>
       <c r="V39" t="n">
-        <v>1.375697735610834</v>
+        <v>1.383634000672043</v>
       </c>
       <c r="W39" t="inlineStr">
         <is>
@@ -4608,13 +4608,13 @@
         <v>1.613835703805611</v>
       </c>
       <c r="H43" t="n">
-        <v>0.1986935213439947</v>
+        <v>0.2036774011183924</v>
       </c>
       <c r="I43" t="n">
-        <v>0.2704911067097739</v>
+        <v>0.2682603793988715</v>
       </c>
       <c r="J43" t="n">
-        <v>0.5308153719462312</v>
+        <v>0.5280622194827358</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
@@ -4641,13 +4641,13 @@
         <v>0.4573326878990664</v>
       </c>
       <c r="Q43" t="n">
-        <v>4.35</v>
+        <v>4.15</v>
       </c>
       <c r="R43" t="n">
-        <v>3.1</v>
+        <v>3.15</v>
       </c>
       <c r="S43" t="n">
-        <v>1.76</v>
+        <v>1.78</v>
       </c>
       <c r="T43" t="inlineStr">
         <is>
@@ -4655,10 +4655,10 @@
         </is>
       </c>
       <c r="U43" t="n">
-        <v>-0.02387113224266757</v>
+        <v>-0.01277875874542511</v>
       </c>
       <c r="V43" t="n">
-        <v>1.093896395647595</v>
+        <v>1.105906879961252</v>
       </c>
       <c r="W43" t="inlineStr">
         <is>
@@ -4992,13 +4992,13 @@
         <v>0.6401931479937157</v>
       </c>
       <c r="H47" t="n">
-        <v>0.8194945059236322</v>
+        <v>0.8203480958759131</v>
       </c>
       <c r="I47" t="n">
-        <v>0.1217911147747655</v>
+        <v>0.1209001802620724</v>
       </c>
       <c r="J47" t="n">
-        <v>0.05871437930160246</v>
+        <v>0.05875172386201476</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
@@ -5028,7 +5028,7 @@
         <v>1.05</v>
       </c>
       <c r="R47" t="n">
-        <v>10.75</v>
+        <v>11</v>
       </c>
       <c r="S47" t="n">
         <v>24</v>
@@ -5042,7 +5042,7 @@
         <v>0.8983869847782044</v>
       </c>
       <c r="V47" t="n">
-        <v>2.063681200368666</v>
+        <v>2.0596676972296</v>
       </c>
       <c r="W47" t="inlineStr">
         <is>
@@ -5088,13 +5088,13 @@
         <v>1.122130451557203</v>
       </c>
       <c r="H48" t="n">
-        <v>0.6176036169403047</v>
+        <v>0.6183875745751082</v>
       </c>
       <c r="I48" t="n">
-        <v>0.2007218146814886</v>
+        <v>0.1996280071243581</v>
       </c>
       <c r="J48" t="n">
-        <v>0.1816745683782067</v>
+        <v>0.1819844183005337</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
@@ -5124,7 +5124,7 @@
         <v>1.66</v>
       </c>
       <c r="R48" t="n">
-        <v>4</v>
+        <v>4.05</v>
       </c>
       <c r="S48" t="n">
         <v>4.2</v>
@@ -5138,7 +5138,7 @@
         <v>0.1334375634174001</v>
       </c>
       <c r="V48" t="n">
-        <v>1.236019190284351</v>
+        <v>1.232520926199729</v>
       </c>
       <c r="W48" t="inlineStr">
         <is>
@@ -5422,13 +5422,13 @@
         <v>1.11264099148167</v>
       </c>
       <c r="H52" t="n">
-        <v>0.4851210862106586</v>
+        <v>0.4835773660401394</v>
       </c>
       <c r="I52" t="n">
-        <v>0.2554445715481236</v>
+        <v>0.2552942787201526</v>
       </c>
       <c r="J52" t="n">
-        <v>0.2594343422412178</v>
+        <v>0.2611283552397081</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -5455,13 +5455,13 @@
         <v>0.5397465778429353</v>
       </c>
       <c r="Q52" t="n">
-        <v>1.9</v>
+        <v>1.91</v>
       </c>
       <c r="R52" t="n">
         <v>3.55</v>
       </c>
       <c r="S52" t="n">
-        <v>3.55</v>
+        <v>3.5</v>
       </c>
       <c r="T52" t="inlineStr">
         <is>
@@ -5469,10 +5469,10 @@
         </is>
       </c>
       <c r="U52" t="n">
-        <v>-0.07422694722942902</v>
+        <v>-0.06935445747800495</v>
       </c>
       <c r="V52" t="n">
-        <v>1.008811258393432</v>
+        <v>1.015301375527119</v>
       </c>
       <c r="W52" t="inlineStr">
         <is>
@@ -5518,13 +5518,13 @@
         <v>1.529136542215973</v>
       </c>
       <c r="H53" t="n">
-        <v>0.3528668246941856</v>
+        <v>0.3511459195494743</v>
       </c>
       <c r="I53" t="n">
-        <v>0.2588831976025882</v>
+        <v>0.2608393387081809</v>
       </c>
       <c r="J53" t="n">
-        <v>0.3882499777032261</v>
+        <v>0.3880147417423447</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -5551,10 +5551,10 @@
         <v>0.6284429767793762</v>
       </c>
       <c r="Q53" t="n">
-        <v>2.97</v>
+        <v>3</v>
       </c>
       <c r="R53" t="n">
-        <v>3.32</v>
+        <v>3.27</v>
       </c>
       <c r="S53" t="n">
         <v>2.22</v>
@@ -5565,10 +5565,10 @@
         </is>
       </c>
       <c r="U53" t="n">
-        <v>0.177211601689985</v>
+        <v>0.1891026279696817</v>
       </c>
       <c r="V53" t="n">
-        <v>1.281224846651258</v>
+        <v>1.295639304448658</v>
       </c>
       <c r="W53" t="inlineStr">
         <is>
@@ -5614,13 +5614,13 @@
         <v>0.90759573691246</v>
       </c>
       <c r="H54" t="n">
-        <v>0.7973581376781287</v>
+        <v>0.7958944450894115</v>
       </c>
       <c r="I54" t="n">
-        <v>0.1256268366299308</v>
+        <v>0.1269630327868514</v>
       </c>
       <c r="J54" t="n">
-        <v>0.0770150256919406</v>
+        <v>0.07714252212373716</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
@@ -5647,10 +5647,10 @@
         <v>0.5502776864472912</v>
       </c>
       <c r="Q54" t="n">
-        <v>1.05</v>
+        <v>1.06</v>
       </c>
       <c r="R54" t="n">
-        <v>10.5</v>
+        <v>10.25</v>
       </c>
       <c r="S54" t="n">
         <v>22</v>
@@ -5664,7 +5664,7 @@
         <v>1.473809645296872</v>
       </c>
       <c r="V54" t="n">
-        <v>2.704055997564761</v>
+        <v>2.687575859678358</v>
       </c>
       <c r="W54" t="inlineStr">
         <is>
@@ -5710,13 +5710,13 @@
         <v>1.427558893552563</v>
       </c>
       <c r="H55" t="n">
-        <v>0.5781298421549753</v>
+        <v>0.583615334142649</v>
       </c>
       <c r="I55" t="n">
-        <v>0.2114948035080663</v>
+        <v>0.2100926057548347</v>
       </c>
       <c r="J55" t="n">
-        <v>0.2103753543369585</v>
+        <v>0.2062920601025164</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
@@ -5743,13 +5743,13 @@
         <v>0.6893569696047046</v>
       </c>
       <c r="Q55" t="n">
-        <v>1.59</v>
+        <v>1.56</v>
       </c>
       <c r="R55" t="n">
-        <v>4.05</v>
+        <v>4.1</v>
       </c>
       <c r="S55" t="n">
-        <v>4.65</v>
+        <v>4.85</v>
       </c>
       <c r="T55" t="inlineStr">
         <is>
@@ -5757,14 +5757,14 @@
         </is>
       </c>
       <c r="U55" t="n">
-        <v>0.03981494466557822</v>
+        <v>0.08453816809205472</v>
       </c>
       <c r="V55" t="n">
-        <v>1.134332211225691</v>
+        <v>1.183354395963062</v>
       </c>
       <c r="W55" t="inlineStr">
         <is>
-          <t>Pas de valeur</t>
+          <t>PARI VALUE</t>
         </is>
       </c>
       <c r="X55" t="inlineStr">
@@ -5806,13 +5806,13 @@
         <v>1.279464126758056</v>
       </c>
       <c r="H56" t="n">
-        <v>0.5601492517408571</v>
+        <v>0.5630883488443332</v>
       </c>
       <c r="I56" t="n">
-        <v>0.2184846665795057</v>
+        <v>0.2166638741433221</v>
       </c>
       <c r="J56" t="n">
-        <v>0.2213660816796373</v>
+        <v>0.2202477770123447</v>
       </c>
       <c r="K56" t="inlineStr">
         <is>
@@ -5839,13 +5839,13 @@
         <v>0.5894224972165162</v>
       </c>
       <c r="Q56" t="n">
-        <v>1.4</v>
+        <v>1.39</v>
       </c>
       <c r="R56" t="n">
-        <v>4.75</v>
+        <v>4.85</v>
       </c>
       <c r="S56" t="n">
-        <v>6</v>
+        <v>6.1</v>
       </c>
       <c r="T56" t="inlineStr">
         <is>
@@ -5853,10 +5853,10 @@
         </is>
       </c>
       <c r="U56" t="n">
-        <v>0.7402046908330298</v>
+        <v>0.7692081023469135</v>
       </c>
       <c r="V56" t="n">
-        <v>1.899396348014498</v>
+        <v>1.92763087530271</v>
       </c>
       <c r="W56" t="inlineStr">
         <is>
@@ -5902,13 +5902,13 @@
         <v>1.768893310395192</v>
       </c>
       <c r="H57" t="n">
-        <v>0.6696481847748125</v>
+        <v>0.6557815228140289</v>
       </c>
       <c r="I57" t="n">
-        <v>0.1653561658659211</v>
+        <v>0.1618550034864507</v>
       </c>
       <c r="J57" t="n">
-        <v>0.1649956493592665</v>
+        <v>0.1823634736995204</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
@@ -5935,13 +5935,13 @@
         <v>0.7874684227946003</v>
       </c>
       <c r="Q57" t="n">
-        <v>1.23</v>
+        <v>1.27</v>
       </c>
       <c r="R57" t="n">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
       <c r="S57" t="n">
-        <v>7.5</v>
+        <v>5.75</v>
       </c>
       <c r="T57" t="inlineStr">
         <is>
@@ -5949,10 +5949,10 @@
         </is>
       </c>
       <c r="U57" t="n">
-        <v>0.5911729648820514</v>
+        <v>0.2198992730762395</v>
       </c>
       <c r="V57" t="n">
-        <v>1.800454612295626</v>
+        <v>1.390546159945527</v>
       </c>
       <c r="W57" t="inlineStr">
         <is>
@@ -6236,13 +6236,13 @@
         <v>0.9450506815788465</v>
       </c>
       <c r="H61" t="n">
-        <v>0.6229563560482517</v>
+        <v>0.6265300686262469</v>
       </c>
       <c r="I61" t="n">
-        <v>0.2209877144838659</v>
+        <v>0.217452778583227</v>
       </c>
       <c r="J61" t="n">
-        <v>0.1560559294678824</v>
+        <v>0.1560171527905261</v>
       </c>
       <c r="K61" t="inlineStr">
         <is>
@@ -6269,10 +6269,10 @@
         <v>0.5502897941356736</v>
       </c>
       <c r="Q61" t="n">
-        <v>1.57</v>
+        <v>1.55</v>
       </c>
       <c r="R61" t="n">
-        <v>3.55</v>
+        <v>3.65</v>
       </c>
       <c r="S61" t="n">
         <v>5.25</v>
@@ -6283,10 +6283,10 @@
         </is>
       </c>
       <c r="U61" t="n">
-        <v>0.05445832582548826</v>
+        <v>0.04102573568758383</v>
       </c>
       <c r="V61" t="n">
-        <v>1.169509226131395</v>
+        <v>1.155132653542025</v>
       </c>
       <c r="W61" t="inlineStr">
         <is>
@@ -6428,13 +6428,13 @@
         <v>1.267735705596107</v>
       </c>
       <c r="H63" t="n">
-        <v>0.3835062791805128</v>
+        <v>0.3849937928254214</v>
       </c>
       <c r="I63" t="n">
-        <v>0.2658257065103567</v>
+        <v>0.265788211680313</v>
       </c>
       <c r="J63" t="n">
-        <v>0.3506680143091305</v>
+        <v>0.3492179954942656</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -6461,13 +6461,13 @@
         <v>0.5397814678090256</v>
       </c>
       <c r="Q63" t="n">
-        <v>2.45</v>
+        <v>2.43</v>
       </c>
       <c r="R63" t="n">
         <v>3.45</v>
       </c>
       <c r="S63" t="n">
-        <v>2.55</v>
+        <v>2.57</v>
       </c>
       <c r="T63" t="inlineStr">
         <is>
@@ -6475,10 +6475,10 @@
         </is>
       </c>
       <c r="U63" t="n">
-        <v>-0.03810298560629488</v>
+        <v>-0.0459552061319578</v>
       </c>
       <c r="V63" t="n">
-        <v>1.048636270541426</v>
+        <v>1.04036940434502</v>
       </c>
       <c r="W63" t="inlineStr">
         <is>
@@ -6620,13 +6620,13 @@
         <v>1.768677962550518</v>
       </c>
       <c r="H65" t="n">
-        <v>0.336532257371548</v>
+        <v>0.3351926848105896</v>
       </c>
       <c r="I65" t="n">
-        <v>0.2606343436621112</v>
+        <v>0.2605573656327125</v>
       </c>
       <c r="J65" t="n">
-        <v>0.402833398966341</v>
+        <v>0.4042499495566981</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
@@ -6653,13 +6653,13 @@
         <v>0.6515954800796417</v>
       </c>
       <c r="Q65" t="n">
-        <v>2.7</v>
+        <v>2.72</v>
       </c>
       <c r="R65" t="n">
         <v>3.18</v>
       </c>
       <c r="S65" t="n">
-        <v>2.47</v>
+        <v>2.45</v>
       </c>
       <c r="T65" t="inlineStr">
         <is>
@@ -6667,10 +6667,10 @@
         </is>
       </c>
       <c r="U65" t="n">
-        <v>0.07230823816758458</v>
+        <v>0.06362558036865673</v>
       </c>
       <c r="V65" t="n">
-        <v>1.168487937748091</v>
+        <v>1.159645159204515</v>
       </c>
       <c r="W65" t="inlineStr">
         <is>
@@ -6954,13 +6954,13 @@
         <v>1.523965627828707</v>
       </c>
       <c r="H69" t="n">
-        <v>0.2892484885230557</v>
+        <v>0.2924266152569004</v>
       </c>
       <c r="I69" t="n">
-        <v>0.2667127154849229</v>
+        <v>0.2667927711945851</v>
       </c>
       <c r="J69" t="n">
-        <v>0.4440387959920215</v>
+        <v>0.4407806135485146</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -6987,13 +6987,13 @@
         <v>0.5650680958204189</v>
       </c>
       <c r="Q69" t="n">
-        <v>3.48</v>
+        <v>3.4</v>
       </c>
       <c r="R69" t="n">
         <v>3.3</v>
       </c>
       <c r="S69" t="n">
-        <v>2</v>
+        <v>2.03</v>
       </c>
       <c r="T69" t="inlineStr">
         <is>
@@ -7001,14 +7001,14 @@
         </is>
       </c>
       <c r="U69" t="n">
-        <v>0.09606358649325197</v>
+        <v>0.07086672243593584</v>
       </c>
       <c r="V69" t="n">
-        <v>1.195133074718609</v>
+        <v>1.166986421045387</v>
       </c>
       <c r="W69" t="inlineStr">
         <is>
-          <t>PARI VALUE</t>
+          <t>Pas de valeur</t>
         </is>
       </c>
       <c r="X69" t="inlineStr">
@@ -7146,13 +7146,13 @@
         <v>1.368315802227365</v>
       </c>
       <c r="H71" t="n">
-        <v>0.2489484827101855</v>
+        <v>0.2517654131192861</v>
       </c>
       <c r="I71" t="n">
-        <v>0.2752790429030879</v>
+        <v>0.2780204783147732</v>
       </c>
       <c r="J71" t="n">
-        <v>0.4757724743867267</v>
+        <v>0.4702141085659407</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -7179,13 +7179,13 @@
         <v>0.4706324666789738</v>
       </c>
       <c r="Q71" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="R71" t="n">
-        <v>3.37</v>
+        <v>3.3</v>
       </c>
       <c r="S71" t="n">
-        <v>1.84</v>
+        <v>1.88</v>
       </c>
       <c r="T71" t="inlineStr">
         <is>
@@ -7193,10 +7193,10 @@
         </is>
       </c>
       <c r="U71" t="n">
-        <v>0.07433689277523881</v>
+        <v>0.04747847045585774</v>
       </c>
       <c r="V71" t="n">
-        <v>1.171257299467677</v>
+        <v>1.143171340692414</v>
       </c>
       <c r="W71" t="inlineStr">
         <is>
@@ -7242,13 +7242,13 @@
         <v>1.013619913753882</v>
       </c>
       <c r="H72" t="n">
-        <v>0.5699496931914108</v>
+        <v>0.5661858587164007</v>
       </c>
       <c r="I72" t="n">
-        <v>0.2380931129894224</v>
+        <v>0.2396549356510249</v>
       </c>
       <c r="J72" t="n">
-        <v>0.191957193819167</v>
+        <v>0.1941592056325745</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -7275,13 +7275,13 @@
         <v>0.5215284007993123</v>
       </c>
       <c r="Q72" t="n">
-        <v>1.5</v>
+        <v>1.52</v>
       </c>
       <c r="R72" t="n">
-        <v>3.98</v>
+        <v>3.93</v>
       </c>
       <c r="S72" t="n">
-        <v>5.75</v>
+        <v>5.6</v>
       </c>
       <c r="T72" t="inlineStr">
         <is>
@@ -7289,10 +7289,10 @@
         </is>
       </c>
       <c r="U72" t="n">
-        <v>0.291619255067699</v>
+        <v>0.2579248397181069</v>
       </c>
       <c r="V72" t="n">
-        <v>1.410236390064449</v>
+        <v>1.37229422347426</v>
       </c>
       <c r="W72" t="inlineStr">
         <is>
@@ -7338,13 +7338,13 @@
         <v>1.610986105612227</v>
       </c>
       <c r="H73" t="n">
-        <v>0.5103432029242074</v>
+        <v>0.5079921563290901</v>
       </c>
       <c r="I73" t="n">
-        <v>0.2187172644803023</v>
+        <v>0.2187722437034678</v>
       </c>
       <c r="J73" t="n">
-        <v>0.2709395325954903</v>
+        <v>0.2732355999674421</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
@@ -7371,13 +7371,13 @@
         <v>0.7263015743474893</v>
       </c>
       <c r="Q73" t="n">
-        <v>1.92</v>
+        <v>1.94</v>
       </c>
       <c r="R73" t="n">
         <v>3.83</v>
       </c>
       <c r="S73" t="n">
-        <v>3.23</v>
+        <v>3.18</v>
       </c>
       <c r="T73" t="inlineStr">
         <is>
@@ -7385,10 +7385,10 @@
         </is>
       </c>
       <c r="U73" t="n">
-        <v>0.04357054193264132</v>
+        <v>0.0544410684111063</v>
       </c>
       <c r="V73" t="n">
-        <v>1.139085905363926</v>
+        <v>1.150422549481312</v>
       </c>
       <c r="W73" t="inlineStr">
         <is>
@@ -7434,13 +7434,13 @@
         <v>1.567579328799631</v>
       </c>
       <c r="H74" t="n">
-        <v>0.502300772004559</v>
+        <v>0.5057380716584359</v>
       </c>
       <c r="I74" t="n">
-        <v>0.2369356591704675</v>
+        <v>0.2344711008656905</v>
       </c>
       <c r="J74" t="n">
-        <v>0.2607635688249734</v>
+        <v>0.2597908274758738</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -7467,13 +7467,13 @@
         <v>0.6733258878586383</v>
       </c>
       <c r="Q74" t="n">
-        <v>1.72</v>
+        <v>1.7</v>
       </c>
       <c r="R74" t="n">
-        <v>3.82</v>
+        <v>3.9</v>
       </c>
       <c r="S74" t="n">
-        <v>4.75</v>
+        <v>4.8</v>
       </c>
       <c r="T74" t="inlineStr">
         <is>
@@ -7481,10 +7481,10 @@
         </is>
       </c>
       <c r="U74" t="n">
-        <v>0.5282187697047758</v>
+        <v>0.5443052830700892</v>
       </c>
       <c r="V74" t="n">
-        <v>1.610286821574572</v>
+        <v>1.626120853308154</v>
       </c>
       <c r="W74" t="inlineStr">
         <is>
@@ -7493,7 +7493,7 @@
       </c>
       <c r="X74" t="inlineStr">
         <is>
-          <t>mediane de 17 bookmakers</t>
+          <t>mediane de 19 bookmakers</t>
         </is>
       </c>
     </row>
@@ -7818,13 +7818,13 @@
         <v>1.054941555353019</v>
       </c>
       <c r="H78" t="n">
-        <v>0.5482059616353565</v>
+        <v>0.5468489569829098</v>
       </c>
       <c r="I78" t="n">
-        <v>0.2372297232241121</v>
+        <v>0.2374202986791014</v>
       </c>
       <c r="J78" t="n">
-        <v>0.2145643151405315</v>
+        <v>0.215730744337989</v>
       </c>
       <c r="K78" t="inlineStr">
         <is>
@@ -7851,13 +7851,13 @@
         <v>0.5304410055933737</v>
       </c>
       <c r="Q78" t="n">
-        <v>1.57</v>
+        <v>1.58</v>
       </c>
       <c r="R78" t="n">
         <v>4.05</v>
       </c>
       <c r="S78" t="n">
-        <v>4.8</v>
+        <v>4.75</v>
       </c>
       <c r="T78" t="inlineStr">
         <is>
@@ -7865,10 +7865,10 @@
         </is>
       </c>
       <c r="U78" t="n">
-        <v>0.1442254710675022</v>
+        <v>0.1323064557438824</v>
       </c>
       <c r="V78" t="n">
-        <v>1.249711146670456</v>
+        <v>1.234611802930914</v>
       </c>
       <c r="W78" t="inlineStr">
         <is>
@@ -7914,13 +7914,13 @@
         <v>2.037331410174504</v>
       </c>
       <c r="H79" t="n">
-        <v>0.3068132963751727</v>
+        <v>0.3087534199557552</v>
       </c>
       <c r="I79" t="n">
-        <v>0.2372148485499755</v>
+        <v>0.2370705183568286</v>
       </c>
       <c r="J79" t="n">
-        <v>0.4559718550748517</v>
+        <v>0.4541760616874162</v>
       </c>
       <c r="K79" t="inlineStr">
         <is>
@@ -7947,13 +7947,13 @@
         <v>0.6489241778337835</v>
       </c>
       <c r="Q79" t="n">
-        <v>2.55</v>
+        <v>2.52</v>
       </c>
       <c r="R79" t="n">
         <v>3.58</v>
       </c>
       <c r="S79" t="n">
-        <v>2.4</v>
+        <v>2.42</v>
       </c>
       <c r="T79" t="inlineStr">
         <is>
@@ -7961,10 +7961,10 @@
         </is>
       </c>
       <c r="U79" t="n">
-        <v>0.2696766068885446</v>
+        <v>0.2802572452792824</v>
       </c>
       <c r="V79" t="n">
-        <v>1.381602584475745</v>
+        <v>1.394684264598038</v>
       </c>
       <c r="W79" t="inlineStr">
         <is>
@@ -8010,13 +8010,13 @@
         <v>1.764238868118608</v>
       </c>
       <c r="H80" t="n">
-        <v>0.2443965918382721</v>
+        <v>0.244578174930169</v>
       </c>
       <c r="I80" t="n">
-        <v>0.2445349391674378</v>
+        <v>0.2454308201025694</v>
       </c>
       <c r="J80" t="n">
-        <v>0.5110684689942899</v>
+        <v>0.5099910049672614</v>
       </c>
       <c r="K80" t="inlineStr">
         <is>
@@ -8046,10 +8046,10 @@
         <v>4.1</v>
       </c>
       <c r="R80" t="n">
-        <v>3.65</v>
+        <v>3.63</v>
       </c>
       <c r="S80" t="n">
-        <v>1.74</v>
+        <v>1.75</v>
       </c>
       <c r="T80" t="inlineStr">
         <is>
@@ -8060,7 +8060,7 @@
         <v>0.08879370509492102</v>
       </c>
       <c r="V80" t="n">
-        <v>1.189602594173781</v>
+        <v>1.187670441197503</v>
       </c>
       <c r="W80" t="inlineStr">
         <is>
@@ -8106,13 +8106,13 @@
         <v>0.9939750569230624</v>
       </c>
       <c r="H81" t="n">
-        <v>0.5942030248806922</v>
+        <v>0.6031904228086916</v>
       </c>
       <c r="I81" t="n">
-        <v>0.2226269442916311</v>
+        <v>0.2196110570242801</v>
       </c>
       <c r="J81" t="n">
-        <v>0.1831700308276766</v>
+        <v>0.1771985201670284</v>
       </c>
       <c r="K81" t="inlineStr">
         <is>
@@ -8139,13 +8139,13 @@
         <v>0.5536122953975022</v>
       </c>
       <c r="Q81" t="n">
-        <v>1.62</v>
+        <v>1.57</v>
       </c>
       <c r="R81" t="n">
-        <v>3.85</v>
+        <v>3.95</v>
       </c>
       <c r="S81" t="n">
-        <v>4.65</v>
+        <v>4.95</v>
       </c>
       <c r="T81" t="inlineStr">
         <is>
@@ -8153,10 +8153,10 @@
         </is>
       </c>
       <c r="U81" t="n">
-        <v>0.00953226900084525</v>
+        <v>-0.02162613436337835</v>
       </c>
       <c r="V81" t="n">
-        <v>1.102487954814548</v>
+        <v>1.068508939508788</v>
       </c>
       <c r="W81" t="inlineStr">
         <is>
@@ -8273,13 +8273,13 @@
         <v>1.912431955956947</v>
       </c>
       <c r="H83" t="n">
-        <v>0.2810044133674068</v>
+        <v>0.2820890670176779</v>
       </c>
       <c r="I83" t="n">
-        <v>0.2331771337870576</v>
+        <v>0.2332908504560206</v>
       </c>
       <c r="J83" t="n">
-        <v>0.4858184528455355</v>
+        <v>0.4846200825263014</v>
       </c>
       <c r="K83" t="inlineStr">
         <is>
@@ -8306,13 +8306,13 @@
         <v>0.6780798948880914</v>
       </c>
       <c r="Q83" t="n">
-        <v>3.78</v>
+        <v>3.75</v>
       </c>
       <c r="R83" t="n">
         <v>3.78</v>
       </c>
       <c r="S83" t="n">
-        <v>1.78</v>
+        <v>1.79</v>
       </c>
       <c r="T83" t="inlineStr">
         <is>
@@ -8320,10 +8320,10 @@
         </is>
       </c>
       <c r="U83" t="n">
-        <v>0.2077176157387945</v>
+        <v>0.1981325552964233</v>
       </c>
       <c r="V83" t="n">
-        <v>1.317497072041311</v>
+        <v>1.305816095470651</v>
       </c>
       <c r="W83" t="inlineStr">
         <is>
@@ -8536,13 +8536,13 @@
         <v>1.749070691683812</v>
       </c>
       <c r="H86" t="n">
-        <v>0.4826036190352839</v>
+        <v>0.4817105301202224</v>
       </c>
       <c r="I86" t="n">
-        <v>0.2302003615355227</v>
+        <v>0.2314488839177302</v>
       </c>
       <c r="J86" t="n">
-        <v>0.2871960194291934</v>
+        <v>0.2868405859620474</v>
       </c>
       <c r="K86" t="inlineStr">
         <is>
@@ -8569,13 +8569,13 @@
         <v>0.7520466936701869</v>
       </c>
       <c r="Q86" t="n">
-        <v>2.07</v>
+        <v>2.08</v>
       </c>
       <c r="R86" t="n">
-        <v>3.48</v>
+        <v>3.45</v>
       </c>
       <c r="S86" t="n">
-        <v>3.12</v>
+        <v>3.13</v>
       </c>
       <c r="T86" t="inlineStr">
         <is>
@@ -8583,10 +8583,10 @@
         </is>
       </c>
       <c r="U86" t="n">
-        <v>0.08135587313055037</v>
+        <v>0.0865798145466401</v>
       </c>
       <c r="V86" t="n">
-        <v>1.17971700878602</v>
+        <v>1.18449491298618</v>
       </c>
       <c r="W86" t="inlineStr">
         <is>
@@ -8895,13 +8895,13 @@
         <v>0.8894617645963668</v>
       </c>
       <c r="H90" t="n">
-        <v>0.7138940175921742</v>
+        <v>0.7072353331868311</v>
       </c>
       <c r="I90" t="n">
-        <v>0.1774548263562853</v>
+        <v>0.1794722708293573</v>
       </c>
       <c r="J90" t="n">
-        <v>0.1086511560515402</v>
+        <v>0.1132923959838114</v>
       </c>
       <c r="K90" t="inlineStr">
         <is>
@@ -8928,13 +8928,13 @@
         <v>0.5621628806380513</v>
       </c>
       <c r="Q90" t="n">
-        <v>1.44</v>
+        <v>1.47</v>
       </c>
       <c r="R90" t="n">
-        <v>3.9</v>
+        <v>3.83</v>
       </c>
       <c r="S90" t="n">
-        <v>6.4</v>
+        <v>6</v>
       </c>
       <c r="T90" t="inlineStr">
         <is>
@@ -8942,10 +8942,10 @@
         </is>
       </c>
       <c r="U90" t="n">
-        <v>0.1527578345979101</v>
+        <v>0.1767736228187</v>
       </c>
       <c r="V90" t="n">
-        <v>1.276223617630432</v>
+        <v>1.303906809809957</v>
       </c>
       <c r="W90" t="inlineStr">
         <is>
@@ -9049,6 +9049,749 @@
         </is>
       </c>
       <c r="X91" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Serie A</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Atalanta</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Venise</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>1.805794070483333</v>
+      </c>
+      <c r="G92" t="n">
+        <v>1.172842116194884</v>
+      </c>
+      <c r="H92" t="n">
+        <v>0.5626817573286196</v>
+      </c>
+      <c r="I92" t="n">
+        <v>0.2272171630524921</v>
+      </c>
+      <c r="J92" t="n">
+        <v>0.2101010796188883</v>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Victoire Atalanta</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Elevee</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N92" t="n">
+        <v>0.7997917734005214</v>
+      </c>
+      <c r="O92" t="n">
+        <v>0.5720051309090468</v>
+      </c>
+      <c r="P92" t="n">
+        <v>0.57918621375896</v>
+      </c>
+      <c r="Q92" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="R92" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="S92" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U92" t="n">
+        <v>0.2856461110848323</v>
+      </c>
+      <c r="V92" t="n">
+        <v>1.39681100038916</v>
+      </c>
+      <c r="W92" t="inlineStr">
+        <is>
+          <t>Ecart suspect</t>
+        </is>
+      </c>
+      <c r="X92" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Serie A</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Torino</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Udinese</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>1.6954549395</v>
+      </c>
+      <c r="G93" t="n">
+        <v>1.712704896346409</v>
+      </c>
+      <c r="H93" t="n">
+        <v>0.3965227373526081</v>
+      </c>
+      <c r="I93" t="n">
+        <v>0.256196699806629</v>
+      </c>
+      <c r="J93" t="n">
+        <v>0.3472805628407629</v>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Victoire Torino</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N93" t="n">
+        <v>0.8560027458128453</v>
+      </c>
+      <c r="O93" t="n">
+        <v>0.6618302163929339</v>
+      </c>
+      <c r="P93" t="n">
+        <v>0.6711310015512051</v>
+      </c>
+      <c r="Q93" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="R93" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="S93" t="n">
+        <v>3</v>
+      </c>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U93" t="n">
+        <v>0.1657941949865296</v>
+      </c>
+      <c r="V93" t="n">
+        <v>1.270081637058453</v>
+      </c>
+      <c r="W93" t="inlineStr">
+        <is>
+          <t>Ecart suspect</t>
+        </is>
+      </c>
+      <c r="X93" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Coritiba</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Botafogo</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>1.366820794073465</v>
+      </c>
+      <c r="G94" t="n">
+        <v>1.417042931316009</v>
+      </c>
+      <c r="H94" t="n">
+        <v>0.3635758096842384</v>
+      </c>
+      <c r="I94" t="n">
+        <v>0.2686421196064118</v>
+      </c>
+      <c r="J94" t="n">
+        <v>0.3677820707093499</v>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Victoire Botafogo</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>Inter-champ.</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N94" t="n">
+        <v>0.7685537687782122</v>
+      </c>
+      <c r="O94" t="n">
+        <v>0.5266907306709407</v>
+      </c>
+      <c r="P94" t="n">
+        <v>0.566847138141709</v>
+      </c>
+      <c r="Q94" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="R94" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="S94" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="T94" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U94" t="n">
+        <v>-0.02527918131779949</v>
+      </c>
+      <c r="V94" t="n">
+        <v>1.081859841716728</v>
+      </c>
+      <c r="W94" t="inlineStr">
+        <is>
+          <t>Pas de valeur</t>
+        </is>
+      </c>
+      <c r="X94" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Liga</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Levante</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Seville</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>1.837086306390977</v>
+      </c>
+      <c r="G95" t="n">
+        <v>1.65270919420681</v>
+      </c>
+      <c r="H95" t="n">
+        <v>0.3942827792551387</v>
+      </c>
+      <c r="I95" t="n">
+        <v>0.2561958427464249</v>
+      </c>
+      <c r="J95" t="n">
+        <v>0.3495213779984364</v>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Victoire Levante</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N95" t="n">
+        <v>0.8648811094967791</v>
+      </c>
+      <c r="O95" t="n">
+        <v>0.677259588992032</v>
+      </c>
+      <c r="P95" t="n">
+        <v>0.6815477448220307</v>
+      </c>
+      <c r="Q95" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="R95" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="S95" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U95" t="n">
+        <v>0.07059894430079061</v>
+      </c>
+      <c r="V95" t="n">
+        <v>1.168028572266853</v>
+      </c>
+      <c r="W95" t="inlineStr">
+        <is>
+          <t>Pas de valeur</t>
+        </is>
+      </c>
+      <c r="X95" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Coventry</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Newcastle</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>1.867581045880609</v>
+      </c>
+      <c r="G96" t="n">
+        <v>1.578568129405063</v>
+      </c>
+      <c r="H96" t="n">
+        <v>0.3690228014926289</v>
+      </c>
+      <c r="I96" t="n">
+        <v>0.2432301786716001</v>
+      </c>
+      <c r="J96" t="n">
+        <v>0.387747019835771</v>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Victoire Newcastle</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N96" t="n">
+        <v>0.8601878575537536</v>
+      </c>
+      <c r="O96" t="n">
+        <v>0.6690758322967889</v>
+      </c>
+      <c r="P96" t="n">
+        <v>0.6729792714700736</v>
+      </c>
+      <c r="Q96" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="R96" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="S96" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U96" t="n">
+        <v>0.4061915044018494</v>
+      </c>
+      <c r="V96" t="n">
+        <v>1.530711610540274</v>
+      </c>
+      <c r="W96" t="inlineStr">
+        <is>
+          <t>Ecart suspect</t>
+        </is>
+      </c>
+      <c r="X96" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Primeira Liga</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Alverca</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>1.947816828888613</v>
+      </c>
+      <c r="G97" t="n">
+        <v>0.7813812821631765</v>
+      </c>
+      <c r="H97" t="n">
+        <v>0.5829372629528005</v>
+      </c>
+      <c r="I97" t="n">
+        <v>0.2442026403789883</v>
+      </c>
+      <c r="J97" t="n">
+        <v>0.1728600966682112</v>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Victoire Famalicão</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>Elevee</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>1 - 0</t>
+        </is>
+      </c>
+      <c r="N97" t="n">
+        <v>0.7585745173657138</v>
+      </c>
+      <c r="O97" t="n">
+        <v>0.5134975501590651</v>
+      </c>
+      <c r="P97" t="n">
+        <v>0.4668996901747453</v>
+      </c>
+      <c r="Q97" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="R97" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="S97" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U97" t="n">
+        <v>0.1116273437483575</v>
+      </c>
+      <c r="V97" t="n">
+        <v>1.243880665791579</v>
+      </c>
+      <c r="W97" t="inlineStr">
+        <is>
+          <t>PARI VALUE</t>
+        </is>
+      </c>
+      <c r="X97" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Chapecoense</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Paranaense</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>1.453328975421544</v>
+      </c>
+      <c r="G98" t="n">
+        <v>2.459021403132006</v>
+      </c>
+      <c r="H98" t="n">
+        <v>0.2153138223739966</v>
+      </c>
+      <c r="I98" t="n">
+        <v>0.1900589715374354</v>
+      </c>
+      <c r="J98" t="n">
+        <v>0.594627206088568</v>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Victoire Paranaense</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>Elevee</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>1 - 2</t>
+        </is>
+      </c>
+      <c r="N98" t="n">
+        <v>0.9032089900184148</v>
+      </c>
+      <c r="O98" t="n">
+        <v>0.748756900399124</v>
+      </c>
+      <c r="P98" t="n">
+        <v>0.7021096829403661</v>
+      </c>
+      <c r="W98" t="inlineStr">
+        <is>
+          <t>Pas de cote</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Bragantino</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Cruzeiro</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>1.276642557459911</v>
+      </c>
+      <c r="G99" t="n">
+        <v>1.874149870390754</v>
+      </c>
+      <c r="H99" t="n">
+        <v>0.3522180104223431</v>
+      </c>
+      <c r="I99" t="n">
+        <v>0.2501033480571685</v>
+      </c>
+      <c r="J99" t="n">
+        <v>0.3976786415204884</v>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Victoire Cruzeiro</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N99" t="n">
+        <v>0.8243187419374816</v>
+      </c>
+      <c r="O99" t="n">
+        <v>0.6097301827771995</v>
+      </c>
+      <c r="P99" t="n">
+        <v>0.6124088565222914</v>
+      </c>
+      <c r="Q99" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="R99" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="S99" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U99" t="n">
+        <v>0.6281852577804612</v>
+      </c>
+      <c r="V99" t="n">
+        <v>1.806984770386164</v>
+      </c>
+      <c r="W99" t="inlineStr">
+        <is>
+          <t>Ecart suspect</t>
+        </is>
+      </c>
+      <c r="X99" t="inlineStr">
         <is>
           <t>Betclic</t>
         </is>
@@ -9065,7 +9808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K91"/>
+  <dimension ref="A1:K99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9165,16 +9908,16 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.7630127604722374</v>
+        <v>0.7622768608319233</v>
       </c>
       <c r="G2" t="n">
-        <v>1.211683848797251</v>
+        <v>1.210699300699301</v>
       </c>
       <c r="H2" t="n">
-        <v>1.310594071036359</v>
+        <v>1.311859314355461</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.07546976170958453</v>
+        <v>-0.07711193765153235</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -9209,16 +9952,16 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.7435628702921497</v>
+        <v>0.7450814563214072</v>
       </c>
       <c r="G3" t="n">
-        <v>1.271086556169429</v>
+        <v>1.264567669172932</v>
       </c>
       <c r="H3" t="n">
-        <v>1.344876189967763</v>
+        <v>1.342135133703593</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.05486723190489562</v>
+        <v>-0.05779407943566417</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -9520,16 +10263,16 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.7270810384563099</v>
+        <v>0.7253664897358619</v>
       </c>
       <c r="G12" t="n">
-        <v>1.256848030018762</v>
+        <v>1.265235404896422</v>
       </c>
       <c r="H12" t="n">
-        <v>1.375362507215335</v>
+        <v>1.378613451476294</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.0861696291521914</v>
+        <v>-0.08224063566075057</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -9689,16 +10432,16 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.7267778894789982</v>
+        <v>0.726355352263742</v>
       </c>
       <c r="G17" t="n">
-        <v>1.289515503875969</v>
+        <v>1.294691119691119</v>
       </c>
       <c r="H17" t="n">
-        <v>1.375936189689074</v>
+        <v>1.3767366026607</v>
       </c>
       <c r="I17" t="n">
-        <v>-0.06280864364257632</v>
+        <v>-0.05959417568401826</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -9733,16 +10476,16 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.7539919265466276</v>
+        <v>0.7556431148928712</v>
       </c>
       <c r="G18" t="n">
-        <v>1.233795761078998</v>
+        <v>1.228544423440454</v>
       </c>
       <c r="H18" t="n">
-        <v>1.326274148027179</v>
+        <v>1.323376049210442</v>
       </c>
       <c r="I18" t="n">
-        <v>-0.06972795713898361</v>
+        <v>-0.07165886508718911</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -9848,16 +10591,16 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.7306124910064178</v>
+        <v>0.7296229656613391</v>
       </c>
       <c r="G21" t="n">
-        <v>1.222736220472441</v>
+        <v>1.226732673267327</v>
       </c>
       <c r="H21" t="n">
-        <v>1.368714622744132</v>
+        <v>1.370570893548544</v>
       </c>
       <c r="I21" t="n">
-        <v>-0.1066536441168574</v>
+        <v>-0.1049476688570306</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -9963,16 +10706,16 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.7308706738421111</v>
+        <v>0.7312866458563442</v>
       </c>
       <c r="G24" t="n">
-        <v>1.250676982591876</v>
+        <v>1.245603112840467</v>
       </c>
       <c r="H24" t="n">
-        <v>1.368231119115922</v>
+        <v>1.367452839001305</v>
       </c>
       <c r="I24" t="n">
-        <v>-0.08591687097425715</v>
+        <v>-0.08910707754267355</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -10078,16 +10821,16 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>0.7707258621554071</v>
+        <v>0.7704039655862822</v>
       </c>
       <c r="G27" t="n">
-        <v>1.21569416498994</v>
+        <v>1.219919517102616</v>
       </c>
       <c r="H27" t="n">
-        <v>1.297478194391202</v>
+        <v>1.298020317482392</v>
       </c>
       <c r="I27" t="n">
-        <v>-0.06303306657083096</v>
+        <v>-0.06016916632804248</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -10453,16 +11196,16 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>0.7477270977241973</v>
+        <v>0.7479966622412655</v>
       </c>
       <c r="G39" t="n">
-        <v>1.255535714285714</v>
+        <v>1.252087475149106</v>
       </c>
       <c r="H39" t="n">
-        <v>1.337386331247894</v>
+        <v>1.336904361315788</v>
       </c>
       <c r="I39" t="n">
-        <v>-0.0612019242680657</v>
+        <v>-0.06344274775437564</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -10612,16 +11355,16 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>0.7295088932902258</v>
+        <v>0.7317396206011282</v>
       </c>
       <c r="G43" t="n">
-        <v>1.253027823240589</v>
+        <v>1.245699831365936</v>
       </c>
       <c r="H43" t="n">
-        <v>1.370785207963411</v>
+        <v>1.366606333518601</v>
       </c>
       <c r="I43" t="n">
-        <v>-0.0859050594058971</v>
+        <v>-0.08847207801340085</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
@@ -10889,16 +11632,16 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>0.7445554284518764</v>
+        <v>0.7447057212798476</v>
       </c>
       <c r="G52" t="n">
-        <v>1.237614678899083</v>
+        <v>1.235674676524954</v>
       </c>
       <c r="H52" t="n">
-        <v>1.343083351200943</v>
+        <v>1.342812296757174</v>
       </c>
       <c r="I52" t="n">
-        <v>-0.07852727249396207</v>
+        <v>-0.07978599875124193</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -10933,16 +11676,16 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>0.7411168023974117</v>
+        <v>0.7391606612918189</v>
       </c>
       <c r="G53" t="n">
-        <v>1.270404624277457</v>
+        <v>1.275862068965517</v>
       </c>
       <c r="H53" t="n">
-        <v>1.34931497540622</v>
+        <v>1.352885850624567</v>
       </c>
       <c r="I53" t="n">
-        <v>-0.05848178710460583</v>
+        <v>-0.05693294938629989</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -11160,26 +11903,9 @@
           <t>São Paulo - Vitória</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>12 (pas de nul)</t>
-        </is>
-      </c>
-      <c r="F61" t="n">
-        <v>0.7790122855161341</v>
-      </c>
-      <c r="G61" t="n">
-        <v>1.208577712609971</v>
-      </c>
-      <c r="H61" t="n">
-        <v>1.283676802782963</v>
-      </c>
-      <c r="I61" t="n">
-        <v>-0.05850311387584517</v>
-      </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>Cote insuffisante</t>
+          <t>Aucune selection a ce seuil</t>
         </is>
       </c>
     </row>
@@ -11237,16 +11963,16 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>0.7341742934896434</v>
+        <v>0.734211788319687</v>
       </c>
       <c r="G63" t="n">
-        <v>1.2495</v>
+        <v>1.24902</v>
       </c>
       <c r="H63" t="n">
-        <v>1.362074385970184</v>
+        <v>1.362004827365404</v>
       </c>
       <c r="I63" t="n">
-        <v>-0.08264922028469057</v>
+        <v>-0.08295479215294455</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -11308,16 +12034,16 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>0.739365656337889</v>
+        <v>0.7394426343672877</v>
       </c>
       <c r="G65" t="n">
-        <v>1.289941972920696</v>
+        <v>1.288974854932302</v>
       </c>
       <c r="H65" t="n">
-        <v>1.352510752194042</v>
+        <v>1.352369952072971</v>
       </c>
       <c r="I65" t="n">
-        <v>-0.04626120655369781</v>
+        <v>-0.04687703763566609</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
@@ -11450,16 +12176,16 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>0.7332872845150772</v>
+        <v>0.733207228805415</v>
       </c>
       <c r="G69" t="n">
-        <v>1.27007299270073</v>
+        <v>1.271086556169429</v>
       </c>
       <c r="H69" t="n">
-        <v>1.363721996981442</v>
+        <v>1.36387089585745</v>
       </c>
       <c r="I69" t="n">
-        <v>-0.06867162404654426</v>
+        <v>-0.06803014857919454</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -11538,16 +12264,16 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>0.7247209570969122</v>
+        <v>0.7219795216852268</v>
       </c>
       <c r="G71" t="n">
-        <v>1.26027397260274</v>
+        <v>1.268512110726644</v>
       </c>
       <c r="H71" t="n">
-        <v>1.379841427527915</v>
+        <v>1.385080836733187</v>
       </c>
       <c r="I71" t="n">
-        <v>-0.08665304037101462</v>
+        <v>-0.08416023304566023</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -11585,13 +12311,13 @@
         <v>0.7538174238186578</v>
       </c>
       <c r="G72" t="n">
-        <v>1.215000403165333</v>
+        <v>1.216021591439419</v>
       </c>
       <c r="H72" t="n">
         <v>1.326581169926055</v>
       </c>
       <c r="I72" t="n">
-        <v>-0.08411152614727846</v>
+        <v>-0.08334173663327271</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -11626,16 +12352,16 @@
         </is>
       </c>
       <c r="F73" t="n">
-        <v>0.7812827355196977</v>
+        <v>0.7812277562965322</v>
       </c>
       <c r="G73" t="n">
-        <v>1.204194174757282</v>
+        <v>1.204921875</v>
       </c>
       <c r="H73" t="n">
-        <v>1.279946368371771</v>
+        <v>1.280036445121425</v>
       </c>
       <c r="I73" t="n">
-        <v>-0.05918388104874617</v>
+        <v>-0.05868158708113946</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
@@ -11670,16 +12396,16 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>0.7630643408295325</v>
+        <v>0.7655288991343097</v>
       </c>
       <c r="G74" t="n">
-        <v>1.262751159196291</v>
+        <v>1.255384615384615</v>
       </c>
       <c r="H74" t="n">
-        <v>1.31050547967278</v>
+        <v>1.306286413394504</v>
       </c>
       <c r="I74" t="n">
-        <v>-0.03643961907615456</v>
+        <v>-0.03896679739446673</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -11815,13 +12541,13 @@
         <v>0.7567423739018653</v>
       </c>
       <c r="G78" t="n">
-        <v>1.209912363649845</v>
+        <v>1.211952240414579</v>
       </c>
       <c r="H78" t="n">
         <v>1.321453686865539</v>
       </c>
       <c r="I78" t="n">
-        <v>-0.08440804571839977</v>
+        <v>-0.08286438453298717</v>
       </c>
       <c r="K78" t="inlineStr">
         <is>
@@ -11856,16 +12582,16 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>0.7627851514500245</v>
+        <v>0.7629294816431714</v>
       </c>
       <c r="G79" t="n">
-        <v>1.236363636363636</v>
+        <v>1.234493927125506</v>
       </c>
       <c r="H79" t="n">
-        <v>1.310985141883058</v>
+        <v>1.310737131099239</v>
       </c>
       <c r="I79" t="n">
-        <v>-0.05692017638906066</v>
+        <v>-0.05816818808649471</v>
       </c>
       <c r="K79" t="inlineStr">
         <is>
@@ -11900,16 +12626,16 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>0.755465060832562</v>
+        <v>0.7545691798974303</v>
       </c>
       <c r="G80" t="n">
-        <v>1.221575342465753</v>
+        <v>1.226495726495727</v>
       </c>
       <c r="H80" t="n">
-        <v>1.323687953084088</v>
+        <v>1.325259534368912</v>
       </c>
       <c r="I80" t="n">
-        <v>-0.07714250959255176</v>
+        <v>-0.07452412551041654</v>
       </c>
       <c r="K80" t="inlineStr">
         <is>
@@ -11938,26 +12664,9 @@
           <t>Real Betis - Osasuna</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>12 (pas de nul)</t>
-        </is>
-      </c>
-      <c r="F81" t="n">
-        <v>0.7773730557083689</v>
-      </c>
-      <c r="G81" t="n">
-        <v>1.201435406698565</v>
-      </c>
-      <c r="H81" t="n">
-        <v>1.286383664389764</v>
-      </c>
-      <c r="I81" t="n">
-        <v>-0.0660364866585097</v>
-      </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>Cote insuffisante</t>
+          <t>Aucune selection a ce seuil</t>
         </is>
       </c>
     </row>
@@ -12015,16 +12724,16 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>0.7668228662129424</v>
+        <v>0.7667091495439793</v>
       </c>
       <c r="G83" t="n">
-        <v>1.210143884892086</v>
+        <v>1.211642599277978</v>
       </c>
       <c r="H83" t="n">
-        <v>1.304082134298673</v>
+        <v>1.304275552984827</v>
       </c>
       <c r="I83" t="n">
-        <v>-0.07203399765698537</v>
+        <v>-0.07102253315632479</v>
       </c>
       <c r="K83" t="inlineStr">
         <is>
@@ -12130,16 +12839,16 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>0.7697996384644773</v>
+        <v>0.7685511160822698</v>
       </c>
       <c r="G86" t="n">
-        <v>1.244393063583815</v>
+        <v>1.249596928982726</v>
       </c>
       <c r="H86" t="n">
-        <v>1.299039321445648</v>
+        <v>1.301149629575133</v>
       </c>
       <c r="I86" t="n">
-        <v>-0.04206666954547589</v>
+        <v>-0.03962088557734944</v>
       </c>
       <c r="K86" t="inlineStr">
         <is>
@@ -12313,6 +13022,324 @@
       <c r="K91" t="inlineStr">
         <is>
           <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Serie A</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Atalanta - Venise</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Serie A</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Torino - Udinese</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>0.743803300193371</v>
+      </c>
+      <c r="G93" t="n">
+        <v>1.279158699808795</v>
+      </c>
+      <c r="H93" t="n">
+        <v>1.344441466903984</v>
+      </c>
+      <c r="I93" t="n">
+        <v>-0.04855753761115633</v>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Coritiba - Botafogo</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>0.7313578803935883</v>
+      </c>
+      <c r="G94" t="n">
+        <v>1.2495</v>
+      </c>
+      <c r="H94" t="n">
+        <v>1.36731964857183</v>
+      </c>
+      <c r="I94" t="n">
+        <v>-0.08616832844821143</v>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Liga</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Levante - Seville</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>0.743804157253575</v>
+      </c>
+      <c r="G95" t="n">
+        <v>1.284513618677043</v>
+      </c>
+      <c r="H95" t="n">
+        <v>1.34443991774986</v>
+      </c>
+      <c r="I95" t="n">
+        <v>-0.04457343037918216</v>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Coventry - Newcastle</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>0.7567698213284</v>
+      </c>
+      <c r="G96" t="n">
+        <v>1.241826923076923</v>
+      </c>
+      <c r="H96" t="n">
+        <v>1.321405758814014</v>
+      </c>
+      <c r="I96" t="n">
+        <v>-0.06022286130228016</v>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Primeira Liga</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Famalicão - Alverca</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>0.7557973596210117</v>
+      </c>
+      <c r="G97" t="n">
+        <v>1.232619439868204</v>
+      </c>
+      <c r="H97" t="n">
+        <v>1.323105971819539</v>
+      </c>
+      <c r="I97" t="n">
+        <v>-0.06838948193008088</v>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Chapecoense - Paranaense</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Brasileirao</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Bragantino - Cruzeiro</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>0.7498966519428315</v>
+      </c>
+      <c r="G99" t="n">
+        <v>1.235307692307692</v>
+      </c>
+      <c r="H99" t="n">
+        <v>1.333517088533735</v>
+      </c>
+      <c r="I99" t="n">
+        <v>-0.07364689741923591</v>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualisation du 06/10/2026 12:10 UTC
</commit_message>
<xml_diff>
--- a/classeur/Analyse_football_paris_sportifs.xlsx
+++ b/classeur/Analyse_football_paris_sportifs.xlsx
@@ -452,7 +452,7 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Copie automatique du 2026-10-05T12:29+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
+          <t>Copie automatique du 2026-10-06T12:10+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fenetre : 2026-10-05 au 2026-10-12. Competitions : Brasileirao, Bundesliga, Championship, Eredivisie, Liga, Ligue 1, Premier League, Primeira Liga, Serie A.</t>
+          <t>Fenetre : 2026-10-06 au 2026-10-13. Competitions : Brasileirao, Bundesliga, Championship, Eredivisie, Liga, Ligue 1, Ligue des Champions, Premier League, Primeira Liga, Serie A.</t>
         </is>
       </c>
     </row>
@@ -688,12 +688,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X99"/>
+  <dimension ref="A1:X112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
@@ -711,7 +711,7 @@
     <col width="9" customWidth="1" min="18" max="18"/>
     <col width="9" customWidth="1" min="19" max="19"/>
     <col width="9" customWidth="1" min="20" max="20"/>
-    <col width="23" customWidth="1" min="21" max="21"/>
+    <col width="24" customWidth="1" min="21" max="21"/>
     <col width="20" customWidth="1" min="22" max="22"/>
     <col width="15" customWidth="1" min="23" max="23"/>
     <col width="26" customWidth="1" min="24" max="24"/>
@@ -872,13 +872,13 @@
         <v>2.015729155698191</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4069010970172698</v>
+        <v>0.4061855206938333</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2377231391680767</v>
+        <v>0.2381038869979266</v>
       </c>
       <c r="J2" t="n">
-        <v>0.3553757638146535</v>
+        <v>0.3557105923082401</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -905,7 +905,7 @@
         <v>0.6846093035344661</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.74</v>
+        <v>1.75</v>
       </c>
       <c r="R2" t="n">
         <v>3.5</v>
@@ -922,7 +922,7 @@
         <v>0.9292542422347312</v>
       </c>
       <c r="V2" t="n">
-        <v>2.144719550456027</v>
+        <v>2.138383740136701</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
@@ -968,13 +968,13 @@
         <v>1.51525557507413</v>
       </c>
       <c r="H3" t="n">
-        <v>0.4574457965271893</v>
+        <v>0.4524175148012684</v>
       </c>
       <c r="I3" t="n">
-        <v>0.2549185436785928</v>
+        <v>0.2563811788782319</v>
       </c>
       <c r="J3" t="n">
-        <v>0.2876356597942179</v>
+        <v>0.2912013063204998</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -1001,13 +1001,13 @@
         <v>0.6721505377373731</v>
       </c>
       <c r="Q3" t="n">
-        <v>2.07</v>
+        <v>2.12</v>
       </c>
       <c r="R3" t="n">
-        <v>3.13</v>
+        <v>3.1</v>
       </c>
       <c r="S3" t="n">
-        <v>3.25</v>
+        <v>3.17</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -1015,10 +1015,10 @@
         </is>
       </c>
       <c r="U3" t="n">
-        <v>-0.006853855393164188</v>
+        <v>0.0171351819161798</v>
       </c>
       <c r="V3" t="n">
-        <v>1.102663263030486</v>
+        <v>1.128751702797689</v>
       </c>
       <c r="W3" t="inlineStr">
         <is>
@@ -1135,13 +1135,13 @@
         <v>1.387510371952636</v>
       </c>
       <c r="H5" t="n">
-        <v>0.5324587990395419</v>
+        <v>0.5343971985492191</v>
       </c>
       <c r="I5" t="n">
-        <v>0.2341255396634928</v>
+        <v>0.2352147355784542</v>
       </c>
       <c r="J5" t="n">
-        <v>0.2334156612969652</v>
+        <v>0.2303880658723265</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -1168,13 +1168,13 @@
         <v>0.6458611013694736</v>
       </c>
       <c r="Q5" t="n">
-        <v>1.61</v>
+        <v>1.6</v>
       </c>
       <c r="R5" t="n">
-        <v>3.68</v>
+        <v>3.65</v>
       </c>
       <c r="S5" t="n">
-        <v>4.6</v>
+        <v>4.75</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
@@ -1182,10 +1182,10 @@
         </is>
       </c>
       <c r="U5" t="n">
-        <v>0.2467247832327795</v>
+        <v>0.2873788522512397</v>
       </c>
       <c r="V5" t="n">
-        <v>1.384174254676145</v>
+        <v>1.428345444310113</v>
       </c>
       <c r="W5" t="inlineStr">
         <is>
@@ -1231,13 +1231,13 @@
         <v>1.326182713580325</v>
       </c>
       <c r="H6" t="n">
-        <v>0.450397115620121</v>
+        <v>0.4506801536040676</v>
       </c>
       <c r="I6" t="n">
-        <v>0.2409357624397665</v>
+        <v>0.2411630505177842</v>
       </c>
       <c r="J6" t="n">
-        <v>0.3086671219401125</v>
+        <v>0.3081567958781482</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -1270,7 +1270,7 @@
         <v>3.3</v>
       </c>
       <c r="S6" t="n">
-        <v>2.32</v>
+        <v>2.33</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
@@ -1281,7 +1281,7 @@
         <v>0.4873574956151483</v>
       </c>
       <c r="V6" t="n">
-        <v>1.653083740887698</v>
+        <v>1.650332228575254</v>
       </c>
       <c r="W6" t="inlineStr">
         <is>
@@ -1423,13 +1423,13 @@
         <v>1.609501646597387</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2049720318723091</v>
+        <v>0.2014382694120476</v>
       </c>
       <c r="I8" t="n">
-        <v>0.2550625811274115</v>
+        <v>0.2565033082290326</v>
       </c>
       <c r="J8" t="n">
-        <v>0.5399653870002794</v>
+        <v>0.5420584223589199</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -1456,13 +1456,13 @@
         <v>0.4326093754136387</v>
       </c>
       <c r="Q8" t="n">
-        <v>3.85</v>
+        <v>3.98</v>
       </c>
       <c r="R8" t="n">
-        <v>3.5</v>
+        <v>3.47</v>
       </c>
       <c r="S8" t="n">
-        <v>1.77</v>
+        <v>1.76</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="U8" t="n">
-        <v>0.01092242835286705</v>
+        <v>0.005211002203980852</v>
       </c>
       <c r="V8" t="n">
-        <v>1.122554848535644</v>
+        <v>1.113394361113964</v>
       </c>
       <c r="W8" t="inlineStr">
         <is>
@@ -1878,13 +1878,13 @@
         <v>1.511071688284041</v>
       </c>
       <c r="H13" t="n">
-        <v>0.7779975644090266</v>
+        <v>0.7747980206630399</v>
       </c>
       <c r="I13" t="n">
-        <v>0.1195639317957917</v>
+        <v>0.1210693131415462</v>
       </c>
       <c r="J13" t="n">
-        <v>0.1024385037951815</v>
+        <v>0.1041326661954137</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1911,13 +1911,13 @@
         <v>0.7645988950706237</v>
       </c>
       <c r="Q13" t="n">
-        <v>1.18</v>
+        <v>1.19</v>
       </c>
       <c r="R13" t="n">
-        <v>6.75</v>
+        <v>6.6</v>
       </c>
       <c r="S13" t="n">
-        <v>8.25</v>
+        <v>8</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
@@ -1925,10 +1925,10 @@
         </is>
       </c>
       <c r="U13" t="n">
-        <v>-0.05932687216434485</v>
+        <v>-0.05135506599624606</v>
       </c>
       <c r="V13" t="n">
-        <v>1.050560583903656</v>
+        <v>1.059495314470006</v>
       </c>
       <c r="W13" t="inlineStr">
         <is>
@@ -1974,13 +1974,13 @@
         <v>0.7459017889013188</v>
       </c>
       <c r="H14" t="n">
-        <v>0.7630672994705359</v>
+        <v>0.7641387855868687</v>
       </c>
       <c r="I14" t="n">
-        <v>0.1392350122267059</v>
+        <v>0.1394989152886915</v>
       </c>
       <c r="J14" t="n">
-        <v>0.0976976883027583</v>
+        <v>0.09636229912443983</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -2013,7 +2013,7 @@
         <v>5.4</v>
       </c>
       <c r="S14" t="n">
-        <v>6.6</v>
+        <v>6.75</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
@@ -2024,7 +2024,7 @@
         <v>0.1111311096148815</v>
       </c>
       <c r="V14" t="n">
-        <v>1.209555143248016</v>
+        <v>1.205813961060761</v>
       </c>
       <c r="W14" t="inlineStr">
         <is>
@@ -2070,13 +2070,13 @@
         <v>1.46355536159902</v>
       </c>
       <c r="H15" t="n">
-        <v>0.4290518906811358</v>
+        <v>0.4292920771048514</v>
       </c>
       <c r="I15" t="n">
-        <v>0.2425768246731481</v>
+        <v>0.2434411670817831</v>
       </c>
       <c r="J15" t="n">
-        <v>0.328371284645716</v>
+        <v>0.3272667558133655</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -2106,10 +2106,10 @@
         <v>2.3</v>
       </c>
       <c r="R15" t="n">
-        <v>3.6</v>
+        <v>3.58</v>
       </c>
       <c r="S15" t="n">
-        <v>2.63</v>
+        <v>2.65</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
@@ -2120,7 +2120,7 @@
         <v>0.05854855972094564</v>
       </c>
       <c r="V15" t="n">
-        <v>1.156769717477606</v>
+        <v>1.155374746142962</v>
       </c>
       <c r="W15" t="inlineStr">
         <is>
@@ -2237,13 +2237,13 @@
         <v>1.509315576065982</v>
       </c>
       <c r="H17" t="n">
-        <v>0.3654299432894552</v>
+        <v>0.3741914589951574</v>
       </c>
       <c r="I17" t="n">
-        <v>0.2736446477362579</v>
+        <v>0.2696105173830409</v>
       </c>
       <c r="J17" t="n">
-        <v>0.3609254089742868</v>
+        <v>0.3561980236218015</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -2270,13 +2270,13 @@
         <v>0.6165787364946821</v>
       </c>
       <c r="Q17" t="n">
-        <v>2.63</v>
+        <v>2.55</v>
       </c>
       <c r="R17" t="n">
-        <v>2.98</v>
+        <v>3.12</v>
       </c>
       <c r="S17" t="n">
-        <v>2.55</v>
+        <v>2.67</v>
       </c>
       <c r="T17" t="inlineStr">
         <is>
@@ -2284,10 +2284,10 @@
         </is>
       </c>
       <c r="U17" t="n">
-        <v>0.01959815182514713</v>
+        <v>-0.01141624062580793</v>
       </c>
       <c r="V17" t="n">
-        <v>1.129669348931196</v>
+        <v>1.074789764320383</v>
       </c>
       <c r="W17" t="inlineStr">
         <is>
@@ -2333,13 +2333,13 @@
         <v>2.069488066301995</v>
       </c>
       <c r="H18" t="n">
-        <v>0.2623284018963855</v>
+        <v>0.2583186847671807</v>
       </c>
       <c r="I18" t="n">
-        <v>0.2443568851071289</v>
+        <v>0.2437867045823969</v>
       </c>
       <c r="J18" t="n">
-        <v>0.4933147129964857</v>
+        <v>0.4978946106504223</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -2366,13 +2366,13 @@
         <v>0.661675608838571</v>
       </c>
       <c r="Q18" t="n">
-        <v>3.35</v>
+        <v>3.45</v>
       </c>
       <c r="R18" t="n">
-        <v>3.27</v>
+        <v>3.28</v>
       </c>
       <c r="S18" t="n">
-        <v>1.94</v>
+        <v>1.9</v>
       </c>
       <c r="T18" t="inlineStr">
         <is>
@@ -2380,10 +2380,10 @@
         </is>
       </c>
       <c r="U18" t="n">
-        <v>0.02102994423796489</v>
+        <v>-2.221956075609821e-05</v>
       </c>
       <c r="V18" t="n">
-        <v>1.143330726110962</v>
+        <v>1.121024001503558</v>
       </c>
       <c r="W18" t="inlineStr">
         <is>
@@ -2500,13 +2500,13 @@
         <v>1.541288913531921</v>
       </c>
       <c r="H20" t="n">
-        <v>0.4472903455878872</v>
+        <v>0.4514170763615597</v>
       </c>
       <c r="I20" t="n">
-        <v>0.2408735550801318</v>
+        <v>0.2395548890600154</v>
       </c>
       <c r="J20" t="n">
-        <v>0.3118360993319813</v>
+        <v>0.3090280345784251</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -2515,7 +2515,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Faible</t>
+          <t>Moyenne</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2533,13 +2533,13 @@
         <v>0.6948602572676411</v>
       </c>
       <c r="Q20" t="n">
-        <v>2.3</v>
+        <v>2.25</v>
       </c>
       <c r="R20" t="n">
-        <v>3.25</v>
+        <v>3.28</v>
       </c>
       <c r="S20" t="n">
-        <v>2.53</v>
+        <v>2.57</v>
       </c>
       <c r="T20" t="inlineStr">
         <is>
@@ -2547,10 +2547,10 @@
         </is>
       </c>
       <c r="U20" t="n">
-        <v>0.1785938473205286</v>
+        <v>0.1529722419439956</v>
       </c>
       <c r="V20" t="n">
-        <v>1.340923738727096</v>
+        <v>1.312575366448333</v>
       </c>
       <c r="W20" t="inlineStr">
         <is>
@@ -2692,13 +2692,13 @@
         <v>0.7209491974602661</v>
       </c>
       <c r="H22" t="n">
-        <v>0.6984371468110943</v>
+        <v>0.7005646498481556</v>
       </c>
       <c r="I22" t="n">
-        <v>0.1864689635676626</v>
+        <v>0.186061279021318</v>
       </c>
       <c r="J22" t="n">
-        <v>0.1150938896212431</v>
+        <v>0.1133740711305264</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -2728,10 +2728,10 @@
         <v>1.34</v>
       </c>
       <c r="R22" t="n">
-        <v>4.75</v>
+        <v>4.8</v>
       </c>
       <c r="S22" t="n">
-        <v>7.25</v>
+        <v>7.5</v>
       </c>
       <c r="T22" t="inlineStr">
         <is>
@@ -2742,7 +2742,7 @@
         <v>-0.04165902604841998</v>
       </c>
       <c r="V22" t="n">
-        <v>1.049120787747627</v>
+        <v>1.042612997407272</v>
       </c>
       <c r="W22" t="inlineStr">
         <is>
@@ -2788,13 +2788,13 @@
         <v>1.258903593920413</v>
       </c>
       <c r="H23" t="n">
-        <v>0.385466912621456</v>
+        <v>0.3902030896943928</v>
       </c>
       <c r="I23" t="n">
-        <v>0.2613692162112949</v>
+        <v>0.2632199425257202</v>
       </c>
       <c r="J23" t="n">
-        <v>0.353163871167249</v>
+        <v>0.3465769677798869</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -2821,13 +2821,13 @@
         <v>0.576945687615827</v>
       </c>
       <c r="Q23" t="n">
-        <v>2.92</v>
+        <v>2.83</v>
       </c>
       <c r="R23" t="n">
-        <v>3.35</v>
+        <v>3.3</v>
       </c>
       <c r="S23" t="n">
-        <v>2.23</v>
+        <v>2.3</v>
       </c>
       <c r="T23" t="inlineStr">
         <is>
@@ -2835,10 +2835,10 @@
         </is>
       </c>
       <c r="U23" t="n">
-        <v>0.3331934164579706</v>
+        <v>0.2921018385534442</v>
       </c>
       <c r="V23" t="n">
-        <v>1.452385853216664</v>
+        <v>1.409902507577649</v>
       </c>
       <c r="W23" t="inlineStr">
         <is>
@@ -2884,13 +2884,13 @@
         <v>1.337395419164045</v>
       </c>
       <c r="H24" t="n">
-        <v>0.3592269051342017</v>
+        <v>0.3634928172953928</v>
       </c>
       <c r="I24" t="n">
-        <v>0.2687133541436557</v>
+        <v>0.2674023828448891</v>
       </c>
       <c r="J24" t="n">
-        <v>0.3720597407221425</v>
+        <v>0.369104799859718</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -2917,13 +2917,13 @@
         <v>0.584803544793031</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.02</v>
+        <v>3.03</v>
       </c>
       <c r="R24" t="n">
-        <v>3.1</v>
+        <v>3.23</v>
       </c>
       <c r="S24" t="n">
-        <v>2.12</v>
+        <v>2.22</v>
       </c>
       <c r="T24" t="inlineStr">
         <is>
@@ -2931,10 +2931,10 @@
         </is>
       </c>
       <c r="U24" t="n">
-        <v>0.281161176232118</v>
+        <v>0.2854034317825553</v>
       </c>
       <c r="V24" t="n">
-        <v>1.441824663371754</v>
+        <v>1.401193828718883</v>
       </c>
       <c r="W24" t="inlineStr">
         <is>
@@ -3172,13 +3172,13 @@
         <v>2.109890993669715</v>
       </c>
       <c r="H27" t="n">
-        <v>0.3590394617213403</v>
+        <v>0.3553937966639609</v>
       </c>
       <c r="I27" t="n">
-        <v>0.2295960344137179</v>
+        <v>0.2308534403214916</v>
       </c>
       <c r="J27" t="n">
-        <v>0.4113645038649419</v>
+        <v>0.4137527630145476</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -3205,13 +3205,13 @@
         <v>0.7011060068226381</v>
       </c>
       <c r="Q27" t="n">
-        <v>2.15</v>
+        <v>2.18</v>
       </c>
       <c r="R27" t="n">
-        <v>3.73</v>
+        <v>3.68</v>
       </c>
       <c r="S27" t="n">
-        <v>2.82</v>
+        <v>2.77</v>
       </c>
       <c r="T27" t="inlineStr">
         <is>
@@ -3219,10 +3219,10 @@
         </is>
       </c>
       <c r="U27" t="n">
-        <v>0.4008283706671443</v>
+        <v>0.3759909882085071</v>
       </c>
       <c r="V27" t="n">
-        <v>1.523852932485023</v>
+        <v>1.501846770495773</v>
       </c>
       <c r="W27" t="inlineStr">
         <is>
@@ -3268,13 +3268,13 @@
         <v>1.1803161511297</v>
       </c>
       <c r="H28" t="n">
-        <v>0.6952380496130295</v>
+        <v>0.6980801134267747</v>
       </c>
       <c r="I28" t="n">
-        <v>0.1662937834007238</v>
+        <v>0.164609514320417</v>
       </c>
       <c r="J28" t="n">
-        <v>0.1384681669862467</v>
+        <v>0.1373103722528084</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -3301,13 +3301,13 @@
         <v>0.6562540716683233</v>
       </c>
       <c r="Q28" t="n">
-        <v>1.38</v>
+        <v>1.37</v>
       </c>
       <c r="R28" t="n">
-        <v>5</v>
+        <v>5.1</v>
       </c>
       <c r="S28" t="n">
-        <v>6</v>
+        <v>6.1</v>
       </c>
       <c r="T28" t="inlineStr">
         <is>
@@ -3315,10 +3315,10 @@
         </is>
       </c>
       <c r="U28" t="n">
-        <v>0.002522355577379676</v>
+        <v>-0.004742299173180919</v>
       </c>
       <c r="V28" t="n">
-        <v>1.094057005434445</v>
+        <v>1.084771043981189</v>
       </c>
       <c r="W28" t="inlineStr">
         <is>
@@ -3364,13 +3364,13 @@
         <v>4.091636529830818</v>
       </c>
       <c r="H29" t="n">
-        <v>0.07902164692102759</v>
+        <v>0.07763878760763415</v>
       </c>
       <c r="I29" t="n">
-        <v>0.1026956405920637</v>
+        <v>0.1024341486337306</v>
       </c>
       <c r="J29" t="n">
-        <v>0.8182827124869088</v>
+        <v>0.8199270637586351</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -3397,13 +3397,13 @@
         <v>0.7015799731548024</v>
       </c>
       <c r="Q29" t="n">
-        <v>9.75</v>
+        <v>10</v>
       </c>
       <c r="R29" t="n">
         <v>7.75</v>
       </c>
       <c r="S29" t="n">
-        <v>1.17</v>
+        <v>1.16</v>
       </c>
       <c r="T29" t="inlineStr">
         <is>
@@ -3411,10 +3411,10 @@
         </is>
       </c>
       <c r="U29" t="n">
-        <v>-0.00577682841515148</v>
+        <v>-0.01427446236032115</v>
       </c>
       <c r="V29" t="n">
-        <v>1.080021862708658</v>
+        <v>1.075526340234439</v>
       </c>
       <c r="W29" t="inlineStr">
         <is>
@@ -3460,13 +3460,13 @@
         <v>1.278946641111108</v>
       </c>
       <c r="H30" t="n">
-        <v>0.4622680116626857</v>
+        <v>0.4628024512933257</v>
       </c>
       <c r="I30" t="n">
-        <v>0.2577422363790816</v>
+        <v>0.2588869954239827</v>
       </c>
       <c r="J30" t="n">
-        <v>0.2799897519582328</v>
+        <v>0.2783105532826916</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -3496,10 +3496,10 @@
         <v>1.88</v>
       </c>
       <c r="R30" t="n">
-        <v>3.25</v>
+        <v>3.23</v>
       </c>
       <c r="S30" t="n">
-        <v>3.3</v>
+        <v>3.35</v>
       </c>
       <c r="T30" t="inlineStr">
         <is>
@@ -3507,10 +3507,10 @@
         </is>
       </c>
       <c r="U30" t="n">
-        <v>-0.02723583013959852</v>
+        <v>-0.01249697908110758</v>
       </c>
       <c r="V30" t="n">
-        <v>1.111516823360303</v>
+        <v>1.125773074936952</v>
       </c>
       <c r="W30" t="inlineStr">
         <is>
@@ -3556,13 +3556,13 @@
         <v>1.408237920953257</v>
       </c>
       <c r="H31" t="n">
-        <v>0.4190885255472075</v>
+        <v>0.4244991234925725</v>
       </c>
       <c r="I31" t="n">
-        <v>0.2410330341509648</v>
+        <v>0.240872733411308</v>
       </c>
       <c r="J31" t="n">
-        <v>0.3398784403018277</v>
+        <v>0.3346281430961196</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
@@ -3589,13 +3589,13 @@
         <v>0.6635932622617695</v>
       </c>
       <c r="Q31" t="n">
-        <v>2.85</v>
+        <v>2.75</v>
       </c>
       <c r="R31" t="n">
         <v>3.28</v>
       </c>
       <c r="S31" t="n">
-        <v>2.07</v>
+        <v>2.12</v>
       </c>
       <c r="T31" t="inlineStr">
         <is>
@@ -3603,10 +3603,10 @@
         </is>
       </c>
       <c r="U31" t="n">
-        <v>0.5107235413968847</v>
+        <v>0.4577156978390993</v>
       </c>
       <c r="V31" t="n">
-        <v>1.720483017066209</v>
+        <v>1.662105697475452</v>
       </c>
       <c r="W31" t="inlineStr">
         <is>
@@ -4032,13 +4032,13 @@
         <v>1.867601730563736</v>
       </c>
       <c r="H37" t="n">
-        <v>0.2874513439721651</v>
+        <v>0.2882211162554782</v>
       </c>
       <c r="I37" t="n">
-        <v>0.250083224717451</v>
+        <v>0.2497766782329458</v>
       </c>
       <c r="J37" t="n">
-        <v>0.462465431310384</v>
+        <v>0.4620022055115761</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -4065,7 +4065,7 @@
         <v>0.6047993974448378</v>
       </c>
       <c r="Q37" t="n">
-        <v>2.85</v>
+        <v>2.83</v>
       </c>
       <c r="R37" t="n">
         <v>3.4</v>
@@ -4082,7 +4082,7 @@
         <v>0.1631910623050006</v>
       </c>
       <c r="V37" t="n">
-        <v>1.267226038637749</v>
+        <v>1.270110400580108</v>
       </c>
       <c r="W37" t="inlineStr">
         <is>
@@ -4128,13 +4128,13 @@
         <v>1.739432984348578</v>
       </c>
       <c r="H38" t="n">
-        <v>0.5243426633910397</v>
+        <v>0.5272823352564746</v>
       </c>
       <c r="I38" t="n">
-        <v>0.2153686289752191</v>
+        <v>0.2151947581392757</v>
       </c>
       <c r="J38" t="n">
-        <v>0.2602887076337412</v>
+        <v>0.2575229066042498</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
@@ -4161,13 +4161,13 @@
         <v>0.73919370799807</v>
       </c>
       <c r="Q38" t="n">
-        <v>1.66</v>
+        <v>1.64</v>
       </c>
       <c r="R38" t="n">
         <v>4.05</v>
       </c>
       <c r="S38" t="n">
-        <v>4.15</v>
+        <v>4.25</v>
       </c>
       <c r="T38" t="inlineStr">
         <is>
@@ -4175,10 +4175,10 @@
         </is>
       </c>
       <c r="U38" t="n">
-        <v>0.243206641709302</v>
+        <v>0.2731634282565141</v>
       </c>
       <c r="V38" t="n">
-        <v>1.355452132043609</v>
+        <v>1.390248369353416</v>
       </c>
       <c r="W38" t="inlineStr">
         <is>
@@ -4224,13 +4224,13 @@
         <v>1.34184830221176</v>
       </c>
       <c r="H39" t="n">
-        <v>0.4079097160281986</v>
+        <v>0.4077760090530064</v>
       </c>
       <c r="I39" t="n">
-        <v>0.2520033377587345</v>
+        <v>0.2522895275822308</v>
       </c>
       <c r="J39" t="n">
-        <v>0.3400869462130669</v>
+        <v>0.3399344633647627</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -4260,7 +4260,7 @@
         <v>2.68</v>
       </c>
       <c r="R39" t="n">
-        <v>3.43</v>
+        <v>3.42</v>
       </c>
       <c r="S39" t="n">
         <v>2.35</v>
@@ -4274,7 +4274,7 @@
         <v>0.2691428094585586</v>
       </c>
       <c r="V39" t="n">
-        <v>1.383634000672043</v>
+        <v>1.384715908510908</v>
       </c>
       <c r="W39" t="inlineStr">
         <is>
@@ -4320,13 +4320,13 @@
         <v>1.642979463599926</v>
       </c>
       <c r="H40" t="n">
-        <v>0.3628922949976124</v>
+        <v>0.3585809255499413</v>
       </c>
       <c r="I40" t="n">
-        <v>0.250717641870989</v>
+        <v>0.25129967915506</v>
       </c>
       <c r="J40" t="n">
-        <v>0.3863900631313985</v>
+        <v>0.3901193952949987</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -4353,24 +4353,24 @@
         <v>0.6432708745489725</v>
       </c>
       <c r="Q40" t="n">
-        <v>2.57</v>
+        <v>2.63</v>
       </c>
       <c r="R40" t="n">
-        <v>3.47</v>
+        <v>3.45</v>
       </c>
       <c r="S40" t="n">
-        <v>2.42</v>
+        <v>2.37</v>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="U40" t="n">
-        <v>-0.04687201371217586</v>
+        <v>-0.02959500600719667</v>
       </c>
       <c r="V40" t="n">
-        <v>1.039398113631802</v>
+        <v>1.059705676703192</v>
       </c>
       <c r="W40" t="inlineStr">
         <is>
@@ -4704,13 +4704,13 @@
         <v>0.6984852279550878</v>
       </c>
       <c r="H44" t="n">
-        <v>0.6596725921302802</v>
+        <v>0.6603809715201751</v>
       </c>
       <c r="I44" t="n">
-        <v>0.2065418754549589</v>
+        <v>0.205682011857071</v>
       </c>
       <c r="J44" t="n">
-        <v>0.1337855324147609</v>
+        <v>0.1339370166227539</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -4740,7 +4740,7 @@
         <v>1.39</v>
       </c>
       <c r="R44" t="n">
-        <v>4.6</v>
+        <v>4.65</v>
       </c>
       <c r="S44" t="n">
         <v>6.5</v>
@@ -4751,10 +4751,10 @@
         </is>
       </c>
       <c r="U44" t="n">
-        <v>-0.01668915292682249</v>
+        <v>-0.006000991545592194</v>
       </c>
       <c r="V44" t="n">
-        <v>1.07245969507423</v>
+        <v>1.081793352329117</v>
       </c>
       <c r="W44" t="inlineStr">
         <is>
@@ -4800,13 +4800,13 @@
         <v>0.6525267046466084</v>
       </c>
       <c r="H45" t="n">
-        <v>0.839072475166928</v>
+        <v>0.8395114742348266</v>
       </c>
       <c r="I45" t="n">
-        <v>0.1073830642824964</v>
+        <v>0.1074465067284379</v>
       </c>
       <c r="J45" t="n">
-        <v>0.05354446055057568</v>
+        <v>0.05304201903673553</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
@@ -4839,7 +4839,7 @@
         <v>7.75</v>
       </c>
       <c r="S45" t="n">
-        <v>14.5</v>
+        <v>14.75</v>
       </c>
       <c r="T45" t="inlineStr">
         <is>
@@ -4850,7 +4850,7 @@
         <v>-0.03718984470798536</v>
       </c>
       <c r="V45" t="n">
-        <v>1.050286193157612</v>
+        <v>1.049160757558206</v>
       </c>
       <c r="W45" t="inlineStr">
         <is>
@@ -4896,13 +4896,13 @@
         <v>1.669079606418681</v>
       </c>
       <c r="H46" t="n">
-        <v>0.6568656888240033</v>
+        <v>0.6562688951096317</v>
       </c>
       <c r="I46" t="n">
-        <v>0.1690037539083944</v>
+        <v>0.1688178055510744</v>
       </c>
       <c r="J46" t="n">
-        <v>0.1741305572676023</v>
+        <v>0.1749132993392939</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
@@ -4935,7 +4935,7 @@
         <v>4.75</v>
       </c>
       <c r="S46" t="n">
-        <v>4.9</v>
+        <v>4.85</v>
       </c>
       <c r="T46" t="inlineStr">
         <is>
@@ -4946,7 +4946,7 @@
         <v>0.02712990490408584</v>
       </c>
       <c r="V46" t="n">
-        <v>1.11986291515902</v>
+        <v>1.122023929055304</v>
       </c>
       <c r="W46" t="inlineStr">
         <is>
@@ -4992,13 +4992,13 @@
         <v>0.6401931479937157</v>
       </c>
       <c r="H47" t="n">
-        <v>0.8203480958759131</v>
+        <v>0.8186038226791237</v>
       </c>
       <c r="I47" t="n">
-        <v>0.1209001802620724</v>
+        <v>0.1227207654112213</v>
       </c>
       <c r="J47" t="n">
-        <v>0.05875172386201476</v>
+        <v>0.05867541190965522</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
@@ -5028,7 +5028,7 @@
         <v>1.05</v>
       </c>
       <c r="R47" t="n">
-        <v>11</v>
+        <v>10.5</v>
       </c>
       <c r="S47" t="n">
         <v>24</v>
@@ -5042,7 +5042,7 @@
         <v>0.8983869847782044</v>
       </c>
       <c r="V47" t="n">
-        <v>2.0596676972296</v>
+        <v>2.06788582270483</v>
       </c>
       <c r="W47" t="inlineStr">
         <is>
@@ -5088,13 +5088,13 @@
         <v>1.122130451557203</v>
       </c>
       <c r="H48" t="n">
-        <v>0.6183875745751082</v>
+        <v>0.617658793695226</v>
       </c>
       <c r="I48" t="n">
-        <v>0.1996280071243581</v>
+        <v>0.1993292969365545</v>
       </c>
       <c r="J48" t="n">
-        <v>0.1819844183005337</v>
+        <v>0.1830119093682194</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
@@ -5127,7 +5127,7 @@
         <v>4.05</v>
       </c>
       <c r="S48" t="n">
-        <v>4.2</v>
+        <v>4.15</v>
       </c>
       <c r="T48" t="inlineStr">
         <is>
@@ -5138,7 +5138,7 @@
         <v>0.1334375634174001</v>
       </c>
       <c r="V48" t="n">
-        <v>1.232520926199729</v>
+        <v>1.235772324832596</v>
       </c>
       <c r="W48" t="inlineStr">
         <is>
@@ -5422,13 +5422,13 @@
         <v>1.11264099148167</v>
       </c>
       <c r="H52" t="n">
-        <v>0.4835773660401394</v>
+        <v>0.4841126219674445</v>
       </c>
       <c r="I52" t="n">
-        <v>0.2552942787201526</v>
+        <v>0.2555822614866745</v>
       </c>
       <c r="J52" t="n">
-        <v>0.2611283552397081</v>
+        <v>0.260305116545881</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -5461,7 +5461,7 @@
         <v>3.55</v>
       </c>
       <c r="S52" t="n">
-        <v>3.5</v>
+        <v>3.53</v>
       </c>
       <c r="T52" t="inlineStr">
         <is>
@@ -5472,7 +5472,7 @@
         <v>-0.06935445747800495</v>
       </c>
       <c r="V52" t="n">
-        <v>1.015301375527119</v>
+        <v>1.013041612979514</v>
       </c>
       <c r="W52" t="inlineStr">
         <is>
@@ -5518,13 +5518,13 @@
         <v>1.529136542215973</v>
       </c>
       <c r="H53" t="n">
-        <v>0.3511459195494743</v>
+        <v>0.3476949077166279</v>
       </c>
       <c r="I53" t="n">
-        <v>0.2608393387081809</v>
+        <v>0.2604458696801017</v>
       </c>
       <c r="J53" t="n">
-        <v>0.3880147417423447</v>
+        <v>0.3918592226032703</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -5551,13 +5551,13 @@
         <v>0.6284429767793762</v>
       </c>
       <c r="Q53" t="n">
-        <v>3</v>
+        <v>3.07</v>
       </c>
       <c r="R53" t="n">
-        <v>3.27</v>
+        <v>3.28</v>
       </c>
       <c r="S53" t="n">
-        <v>2.22</v>
+        <v>2.18</v>
       </c>
       <c r="T53" t="inlineStr">
         <is>
@@ -5565,10 +5565,10 @@
         </is>
       </c>
       <c r="U53" t="n">
-        <v>0.1891026279696817</v>
+        <v>0.2168483559556409</v>
       </c>
       <c r="V53" t="n">
-        <v>1.295639304448658</v>
+        <v>1.325545214327768</v>
       </c>
       <c r="W53" t="inlineStr">
         <is>
@@ -5614,13 +5614,13 @@
         <v>0.90759573691246</v>
       </c>
       <c r="H54" t="n">
-        <v>0.7958944450894115</v>
+        <v>0.7981472108928505</v>
       </c>
       <c r="I54" t="n">
-        <v>0.1269630327868514</v>
+        <v>0.125705743951403</v>
       </c>
       <c r="J54" t="n">
-        <v>0.07714252212373716</v>
+        <v>0.07614704515574656</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
@@ -5647,13 +5647,13 @@
         <v>0.5502776864472912</v>
       </c>
       <c r="Q54" t="n">
-        <v>1.06</v>
+        <v>1.05</v>
       </c>
       <c r="R54" t="n">
-        <v>10.25</v>
+        <v>10.5</v>
       </c>
       <c r="S54" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="T54" t="inlineStr">
         <is>
@@ -5661,10 +5661,10 @@
         </is>
       </c>
       <c r="U54" t="n">
-        <v>1.473809645296872</v>
+        <v>1.586255538264911</v>
       </c>
       <c r="V54" t="n">
-        <v>2.687575859678358</v>
+        <v>2.821856456864613</v>
       </c>
       <c r="W54" t="inlineStr">
         <is>
@@ -5710,13 +5710,13 @@
         <v>1.427558893552563</v>
       </c>
       <c r="H55" t="n">
-        <v>0.583615334142649</v>
+        <v>0.5844085925793456</v>
       </c>
       <c r="I55" t="n">
-        <v>0.2100926057548347</v>
+        <v>0.2090441961508707</v>
       </c>
       <c r="J55" t="n">
-        <v>0.2062920601025164</v>
+        <v>0.2065472112697838</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
@@ -5746,7 +5746,7 @@
         <v>1.56</v>
       </c>
       <c r="R55" t="n">
-        <v>4.1</v>
+        <v>4.15</v>
       </c>
       <c r="S55" t="n">
         <v>4.85</v>
@@ -5760,7 +5760,7 @@
         <v>0.08453816809205472</v>
       </c>
       <c r="V55" t="n">
-        <v>1.183354395963062</v>
+        <v>1.180167389885801</v>
       </c>
       <c r="W55" t="inlineStr">
         <is>
@@ -5998,13 +5998,13 @@
         <v>1.411562315208403</v>
       </c>
       <c r="H58" t="n">
-        <v>0.6804274615085708</v>
+        <v>0.6848498312407429</v>
       </c>
       <c r="I58" t="n">
-        <v>0.1650059065400211</v>
+        <v>0.1632685428552959</v>
       </c>
       <c r="J58" t="n">
-        <v>0.154566631951408</v>
+        <v>0.151881625903961</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
@@ -6031,13 +6031,13 @@
         <v>0.7112637155253232</v>
       </c>
       <c r="Q58" t="n">
-        <v>1.31</v>
+        <v>1.3</v>
       </c>
       <c r="R58" t="n">
-        <v>5.6</v>
+        <v>5.75</v>
       </c>
       <c r="S58" t="n">
-        <v>6.6</v>
+        <v>6.9</v>
       </c>
       <c r="T58" t="inlineStr">
         <is>
@@ -6045,14 +6045,14 @@
         </is>
       </c>
       <c r="U58" t="n">
-        <v>0.1257391012765481</v>
+        <v>0.1769090604254822</v>
       </c>
       <c r="V58" t="n">
-        <v>1.230934195412061</v>
+        <v>1.280561028957938</v>
       </c>
       <c r="W58" t="inlineStr">
         <is>
-          <t>Pas de valeur</t>
+          <t>Ecart suspect</t>
         </is>
       </c>
       <c r="X58" t="inlineStr">
@@ -6140,7 +6140,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -6332,13 +6332,13 @@
         <v>1.445413289458153</v>
       </c>
       <c r="H62" t="n">
-        <v>0.6680584089665118</v>
+        <v>0.6680232672007123</v>
       </c>
       <c r="I62" t="n">
-        <v>0.1764329287950061</v>
+        <v>0.1741140331278498</v>
       </c>
       <c r="J62" t="n">
-        <v>0.155508662238482</v>
+        <v>0.157862699671438</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
@@ -6368,10 +6368,10 @@
         <v>1.42</v>
       </c>
       <c r="R62" t="n">
-        <v>4.35</v>
+        <v>4.45</v>
       </c>
       <c r="S62" t="n">
-        <v>5.4</v>
+        <v>5.25</v>
       </c>
       <c r="T62" t="inlineStr">
         <is>
@@ -6382,7 +6382,7 @@
         <v>0.003866837672205747</v>
       </c>
       <c r="V62" t="n">
-        <v>1.123623729141313</v>
+        <v>1.123749261628614</v>
       </c>
       <c r="W62" t="inlineStr">
         <is>
@@ -6428,13 +6428,13 @@
         <v>1.267735705596107</v>
       </c>
       <c r="H63" t="n">
-        <v>0.3849937928254214</v>
+        <v>0.3871767943875938</v>
       </c>
       <c r="I63" t="n">
-        <v>0.265788211680313</v>
+        <v>0.2637691963598924</v>
       </c>
       <c r="J63" t="n">
-        <v>0.3492179954942656</v>
+        <v>0.3490540092525139</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -6461,10 +6461,10 @@
         <v>0.5397814678090256</v>
       </c>
       <c r="Q63" t="n">
-        <v>2.43</v>
+        <v>2.4</v>
       </c>
       <c r="R63" t="n">
-        <v>3.45</v>
+        <v>3.5</v>
       </c>
       <c r="S63" t="n">
         <v>2.57</v>
@@ -6475,10 +6475,10 @@
         </is>
       </c>
       <c r="U63" t="n">
-        <v>-0.0459552061319578</v>
+        <v>-0.05773353692045224</v>
       </c>
       <c r="V63" t="n">
-        <v>1.04036940434502</v>
+        <v>1.028470662847109</v>
       </c>
       <c r="W63" t="inlineStr">
         <is>
@@ -7050,13 +7050,13 @@
         <v>1.336616924815223</v>
       </c>
       <c r="H70" t="n">
-        <v>0.3670225112702341</v>
+        <v>0.3684347049803396</v>
       </c>
       <c r="I70" t="n">
-        <v>0.2757469106787422</v>
+        <v>0.2756944229118428</v>
       </c>
       <c r="J70" t="n">
-        <v>0.3572305780510238</v>
+        <v>0.3558708721078176</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -7083,13 +7083,13 @@
         <v>0.545531836322639</v>
       </c>
       <c r="Q70" t="n">
-        <v>2.5</v>
+        <v>2.48</v>
       </c>
       <c r="R70" t="n">
         <v>3.2</v>
       </c>
       <c r="S70" t="n">
-        <v>2.65</v>
+        <v>2.67</v>
       </c>
       <c r="T70" t="inlineStr">
         <is>
@@ -7097,10 +7097,10 @@
         </is>
       </c>
       <c r="U70" t="n">
-        <v>-0.02422825011446883</v>
+        <v>-0.01686393502099315</v>
       </c>
       <c r="V70" t="n">
-        <v>1.063453126467226</v>
+        <v>1.07187160763255</v>
       </c>
       <c r="W70" t="inlineStr">
         <is>
@@ -7146,13 +7146,13 @@
         <v>1.368315802227365</v>
       </c>
       <c r="H71" t="n">
-        <v>0.2517654131192861</v>
+        <v>0.2497539289071898</v>
       </c>
       <c r="I71" t="n">
-        <v>0.2780204783147732</v>
+        <v>0.2792914535068446</v>
       </c>
       <c r="J71" t="n">
-        <v>0.4702141085659407</v>
+        <v>0.4709546175859657</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -7179,10 +7179,10 @@
         <v>0.4706324666789738</v>
       </c>
       <c r="Q71" t="n">
-        <v>3.9</v>
+        <v>3.98</v>
       </c>
       <c r="R71" t="n">
-        <v>3.3</v>
+        <v>3.28</v>
       </c>
       <c r="S71" t="n">
         <v>1.88</v>
@@ -7193,10 +7193,10 @@
         </is>
       </c>
       <c r="U71" t="n">
-        <v>0.04747847045585774</v>
+        <v>0.06896520831136255</v>
       </c>
       <c r="V71" t="n">
-        <v>1.143171340692414</v>
+        <v>1.163086765177241</v>
       </c>
       <c r="W71" t="inlineStr">
         <is>
@@ -7434,13 +7434,13 @@
         <v>1.567579328799631</v>
       </c>
       <c r="H74" t="n">
-        <v>0.5057380716584359</v>
+        <v>0.5093202293765956</v>
       </c>
       <c r="I74" t="n">
-        <v>0.2344711008656905</v>
+        <v>0.2322423959841554</v>
       </c>
       <c r="J74" t="n">
-        <v>0.2597908274758738</v>
+        <v>0.258437374639249</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -7467,13 +7467,13 @@
         <v>0.6733258878586383</v>
       </c>
       <c r="Q74" t="n">
-        <v>1.7</v>
+        <v>1.69</v>
       </c>
       <c r="R74" t="n">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="S74" t="n">
-        <v>4.8</v>
+        <v>4.9</v>
       </c>
       <c r="T74" t="inlineStr">
         <is>
@@ -7481,10 +7481,10 @@
         </is>
       </c>
       <c r="U74" t="n">
-        <v>0.5443052830700892</v>
+        <v>0.5764783098007162</v>
       </c>
       <c r="V74" t="n">
-        <v>1.626120853308154</v>
+        <v>1.648677247005392</v>
       </c>
       <c r="W74" t="inlineStr">
         <is>
@@ -7493,7 +7493,7 @@
       </c>
       <c r="X74" t="inlineStr">
         <is>
-          <t>mediane de 19 bookmakers</t>
+          <t>mediane de 18 bookmakers</t>
         </is>
       </c>
     </row>
@@ -7722,13 +7722,13 @@
         <v>1.242407984639045</v>
       </c>
       <c r="H77" t="n">
-        <v>0.647996418225617</v>
+        <v>0.6463655970333539</v>
       </c>
       <c r="I77" t="n">
-        <v>0.1881290770938235</v>
+        <v>0.1883398785661869</v>
       </c>
       <c r="J77" t="n">
-        <v>0.1638745046805594</v>
+        <v>0.1652945244004591</v>
       </c>
       <c r="K77" t="inlineStr">
         <is>
@@ -7755,13 +7755,13 @@
         <v>0.6512717116489252</v>
       </c>
       <c r="Q77" t="n">
-        <v>1.39</v>
+        <v>1.4</v>
       </c>
       <c r="R77" t="n">
         <v>4.8</v>
       </c>
       <c r="S77" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="T77" t="inlineStr">
         <is>
@@ -7769,10 +7769,10 @@
         </is>
       </c>
       <c r="U77" t="n">
-        <v>0.08325986435226729</v>
+        <v>0.06550150592026305</v>
       </c>
       <c r="V77" t="n">
-        <v>1.182586366145663</v>
+        <v>1.160635568948858</v>
       </c>
       <c r="W77" t="inlineStr">
         <is>
@@ -7818,13 +7818,13 @@
         <v>1.054941555353019</v>
       </c>
       <c r="H78" t="n">
-        <v>0.5468489569829098</v>
+        <v>0.546080348201736</v>
       </c>
       <c r="I78" t="n">
-        <v>0.2374202986791014</v>
+        <v>0.2378351727371213</v>
       </c>
       <c r="J78" t="n">
-        <v>0.215730744337989</v>
+        <v>0.2160844790611429</v>
       </c>
       <c r="K78" t="inlineStr">
         <is>
@@ -7851,7 +7851,7 @@
         <v>0.5304410055933737</v>
       </c>
       <c r="Q78" t="n">
-        <v>1.58</v>
+        <v>1.59</v>
       </c>
       <c r="R78" t="n">
         <v>4.05</v>
@@ -7868,7 +7868,7 @@
         <v>0.1323064557438824</v>
       </c>
       <c r="V78" t="n">
-        <v>1.234611802930914</v>
+        <v>1.230104572392964</v>
       </c>
       <c r="W78" t="inlineStr">
         <is>
@@ -7914,13 +7914,13 @@
         <v>2.037331410174504</v>
       </c>
       <c r="H79" t="n">
-        <v>0.3087534199557552</v>
+        <v>0.3152438824044571</v>
       </c>
       <c r="I79" t="n">
-        <v>0.2370705183568286</v>
+        <v>0.236897270335737</v>
       </c>
       <c r="J79" t="n">
-        <v>0.4541760616874162</v>
+        <v>0.4478588472598058</v>
       </c>
       <c r="K79" t="inlineStr">
         <is>
@@ -7929,7 +7929,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>Moyenne</t>
+          <t>Faible</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
@@ -7947,13 +7947,13 @@
         <v>0.6489241778337835</v>
       </c>
       <c r="Q79" t="n">
-        <v>2.52</v>
+        <v>2.43</v>
       </c>
       <c r="R79" t="n">
         <v>3.58</v>
       </c>
       <c r="S79" t="n">
-        <v>2.42</v>
+        <v>2.5</v>
       </c>
       <c r="T79" t="inlineStr">
         <is>
@@ -7961,10 +7961,10 @@
         </is>
       </c>
       <c r="U79" t="n">
-        <v>0.2802572452792824</v>
+        <v>0.3225797988422339</v>
       </c>
       <c r="V79" t="n">
-        <v>1.394684264598038</v>
+        <v>1.442739139694815</v>
       </c>
       <c r="W79" t="inlineStr">
         <is>
@@ -8010,13 +8010,13 @@
         <v>1.764238868118608</v>
       </c>
       <c r="H80" t="n">
-        <v>0.244578174930169</v>
+        <v>0.2446252268898116</v>
       </c>
       <c r="I80" t="n">
-        <v>0.2454308201025694</v>
+        <v>0.2437675663507765</v>
       </c>
       <c r="J80" t="n">
-        <v>0.5099910049672614</v>
+        <v>0.5116072067594117</v>
       </c>
       <c r="K80" t="inlineStr">
         <is>
@@ -8046,10 +8046,10 @@
         <v>4.1</v>
       </c>
       <c r="R80" t="n">
-        <v>3.63</v>
+        <v>3.68</v>
       </c>
       <c r="S80" t="n">
-        <v>1.75</v>
+        <v>1.74</v>
       </c>
       <c r="T80" t="inlineStr">
         <is>
@@ -8060,7 +8060,7 @@
         <v>0.08879370509492102</v>
       </c>
       <c r="V80" t="n">
-        <v>1.187670441197503</v>
+        <v>1.187170803587655</v>
       </c>
       <c r="W80" t="inlineStr">
         <is>
@@ -8106,13 +8106,13 @@
         <v>0.9939750569230624</v>
       </c>
       <c r="H81" t="n">
-        <v>0.6031904228086916</v>
+        <v>0.6053560665447039</v>
       </c>
       <c r="I81" t="n">
-        <v>0.2196110570242801</v>
+        <v>0.2182778382128666</v>
       </c>
       <c r="J81" t="n">
-        <v>0.1771985201670284</v>
+        <v>0.1763660952424296</v>
       </c>
       <c r="K81" t="inlineStr">
         <is>
@@ -8139,13 +8139,13 @@
         <v>0.5536122953975022</v>
       </c>
       <c r="Q81" t="n">
-        <v>1.57</v>
+        <v>1.56</v>
       </c>
       <c r="R81" t="n">
-        <v>3.95</v>
+        <v>4</v>
       </c>
       <c r="S81" t="n">
-        <v>4.95</v>
+        <v>5</v>
       </c>
       <c r="T81" t="inlineStr">
         <is>
@@ -8153,10 +8153,10 @@
         </is>
       </c>
       <c r="U81" t="n">
-        <v>-0.02162613436337835</v>
+        <v>-0.02785781503622309</v>
       </c>
       <c r="V81" t="n">
-        <v>1.068508939508788</v>
+        <v>1.060632050518172</v>
       </c>
       <c r="W81" t="inlineStr">
         <is>
@@ -8273,13 +8273,13 @@
         <v>1.912431955956947</v>
       </c>
       <c r="H83" t="n">
-        <v>0.2820890670176779</v>
+        <v>0.2818933743778043</v>
       </c>
       <c r="I83" t="n">
-        <v>0.2332908504560206</v>
+        <v>0.2324589583894952</v>
       </c>
       <c r="J83" t="n">
-        <v>0.4846200825263014</v>
+        <v>0.4856476672327006</v>
       </c>
       <c r="K83" t="inlineStr">
         <is>
@@ -8309,10 +8309,10 @@
         <v>3.75</v>
       </c>
       <c r="R83" t="n">
-        <v>3.78</v>
+        <v>3.8</v>
       </c>
       <c r="S83" t="n">
-        <v>1.79</v>
+        <v>1.78</v>
       </c>
       <c r="T83" t="inlineStr">
         <is>
@@ -8323,7 +8323,7 @@
         <v>0.1981325552964233</v>
       </c>
       <c r="V83" t="n">
-        <v>1.305816095470651</v>
+        <v>1.307908232746015</v>
       </c>
       <c r="W83" t="inlineStr">
         <is>
@@ -8369,13 +8369,13 @@
         <v>1.559880014539196</v>
       </c>
       <c r="H84" t="n">
-        <v>0.1905633869305592</v>
+        <v>0.1891619977052077</v>
       </c>
       <c r="I84" t="n">
-        <v>0.2479258938884661</v>
+        <v>0.2456703159351602</v>
       </c>
       <c r="J84" t="n">
-        <v>0.5615107191809747</v>
+        <v>0.565167686359632</v>
       </c>
       <c r="K84" t="inlineStr">
         <is>
@@ -8402,13 +8402,13 @@
         <v>0.4843050401336683</v>
       </c>
       <c r="Q84" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="R84" t="n">
-        <v>3.88</v>
+        <v>3.95</v>
       </c>
       <c r="S84" t="n">
-        <v>1.51</v>
+        <v>1.49</v>
       </c>
       <c r="T84" t="inlineStr">
         <is>
@@ -8416,10 +8416,10 @@
         </is>
       </c>
       <c r="U84" t="n">
-        <v>0.3307747959815022</v>
+        <v>0.3533303009981377</v>
       </c>
       <c r="V84" t="n">
-        <v>1.449846056915229</v>
+        <v>1.476445686039242</v>
       </c>
       <c r="W84" t="inlineStr">
         <is>
@@ -8536,13 +8536,13 @@
         <v>1.749070691683812</v>
       </c>
       <c r="H86" t="n">
-        <v>0.4817105301202224</v>
+        <v>0.4772579361640552</v>
       </c>
       <c r="I86" t="n">
-        <v>0.2314488839177302</v>
+        <v>0.2312694749860071</v>
       </c>
       <c r="J86" t="n">
-        <v>0.2868405859620474</v>
+        <v>0.2914725888499377</v>
       </c>
       <c r="K86" t="inlineStr">
         <is>
@@ -8569,13 +8569,13 @@
         <v>0.7520466936701869</v>
       </c>
       <c r="Q86" t="n">
-        <v>2.08</v>
+        <v>2.12</v>
       </c>
       <c r="R86" t="n">
         <v>3.45</v>
       </c>
       <c r="S86" t="n">
-        <v>3.13</v>
+        <v>3.03</v>
       </c>
       <c r="T86" t="inlineStr">
         <is>
@@ -8583,10 +8583,10 @@
         </is>
       </c>
       <c r="U86" t="n">
-        <v>0.0865798145466401</v>
+        <v>0.1074755802109986</v>
       </c>
       <c r="V86" t="n">
-        <v>1.18449491298618</v>
+        <v>1.208905047981686</v>
       </c>
       <c r="W86" t="inlineStr">
         <is>
@@ -9087,13 +9087,13 @@
         <v>1.172842116194884</v>
       </c>
       <c r="H92" t="n">
-        <v>0.5626817573286196</v>
+        <v>0.561128576051344</v>
       </c>
       <c r="I92" t="n">
-        <v>0.2272171630524921</v>
+        <v>0.2266550593521447</v>
       </c>
       <c r="J92" t="n">
-        <v>0.2101010796188883</v>
+        <v>0.2122163645965112</v>
       </c>
       <c r="K92" t="inlineStr">
         <is>
@@ -9126,7 +9126,7 @@
         <v>4.2</v>
       </c>
       <c r="S92" t="n">
-        <v>5.25</v>
+        <v>5.1</v>
       </c>
       <c r="T92" t="inlineStr">
         <is>
@@ -9134,10 +9134,10 @@
         </is>
       </c>
       <c r="U92" t="n">
-        <v>0.2856461110848323</v>
+        <v>0.2489133650538371</v>
       </c>
       <c r="V92" t="n">
-        <v>1.39681100038916</v>
+        <v>1.363898828193469</v>
       </c>
       <c r="W92" t="inlineStr">
         <is>
@@ -9183,13 +9183,13 @@
         <v>1.712704896346409</v>
       </c>
       <c r="H93" t="n">
-        <v>0.3965227373526081</v>
+        <v>0.3945396440631941</v>
       </c>
       <c r="I93" t="n">
-        <v>0.256196699806629</v>
+        <v>0.2582950814008343</v>
       </c>
       <c r="J93" t="n">
-        <v>0.3472805628407629</v>
+        <v>0.3471652745359715</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -9216,10 +9216,10 @@
         <v>0.6711310015512051</v>
       </c>
       <c r="Q93" t="n">
-        <v>2.23</v>
+        <v>2.25</v>
       </c>
       <c r="R93" t="n">
-        <v>3.25</v>
+        <v>3.2</v>
       </c>
       <c r="S93" t="n">
         <v>3</v>
@@ -9233,7 +9233,7 @@
         <v>0.1657941949865296</v>
       </c>
       <c r="V93" t="n">
-        <v>1.270081637058453</v>
+        <v>1.271039504256147</v>
       </c>
       <c r="W93" t="inlineStr">
         <is>
@@ -9792,6 +9792,1054 @@
         </is>
       </c>
       <c r="X99" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Lens</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Sporting CP</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>1.579540668035497</v>
+      </c>
+      <c r="G100" t="n">
+        <v>2.456568352541854</v>
+      </c>
+      <c r="H100" t="n">
+        <v>0.3153854595295835</v>
+      </c>
+      <c r="I100" t="n">
+        <v>0.2221495333613384</v>
+      </c>
+      <c r="J100" t="n">
+        <v>0.4624650071090782</v>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Victoire Sporting CP</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>Inter-champ.</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>1 - 2</t>
+        </is>
+      </c>
+      <c r="N100" t="n">
+        <v>0.9123979761709814</v>
+      </c>
+      <c r="O100" t="n">
+        <v>0.7671274380231462</v>
+      </c>
+      <c r="P100" t="n">
+        <v>0.7272349907651137</v>
+      </c>
+      <c r="Q100" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="R100" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="S100" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U100" t="n">
+        <v>0.4774284182919459</v>
+      </c>
+      <c r="V100" t="n">
+        <v>1.59310433127599</v>
+      </c>
+      <c r="W100" t="inlineStr">
+        <is>
+          <t>Ecart suspect</t>
+        </is>
+      </c>
+      <c r="X100" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Wolverhampton</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Bolton</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>3.04475704394842</v>
+      </c>
+      <c r="G101" t="n">
+        <v>1.538119463095111</v>
+      </c>
+      <c r="H101" t="n">
+        <v>0.6777315728211989</v>
+      </c>
+      <c r="I101" t="n">
+        <v>0.1556907814717814</v>
+      </c>
+      <c r="J101" t="n">
+        <v>0.1665776457070197</v>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Victoire Wolverhampton</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>Elevee</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>3 - 1</t>
+        </is>
+      </c>
+      <c r="N101" t="n">
+        <v>0.9438517858215855</v>
+      </c>
+      <c r="O101" t="n">
+        <v>0.8354769110653351</v>
+      </c>
+      <c r="P101" t="n">
+        <v>0.7487784996096181</v>
+      </c>
+      <c r="W101" t="inlineStr">
+        <is>
+          <t>Pas de cote</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Wrexham</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>West Brom</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>1.863113193610717</v>
+      </c>
+      <c r="G102" t="n">
+        <v>1.379578254700691</v>
+      </c>
+      <c r="H102" t="n">
+        <v>0.4869472677869082</v>
+      </c>
+      <c r="I102" t="n">
+        <v>0.2296886444287424</v>
+      </c>
+      <c r="J102" t="n">
+        <v>0.2833640877843496</v>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Victoire Wrexham</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N102" t="n">
+        <v>0.8362933980569751</v>
+      </c>
+      <c r="O102" t="n">
+        <v>0.6289329201061127</v>
+      </c>
+      <c r="P102" t="n">
+        <v>0.6341925192576207</v>
+      </c>
+      <c r="W102" t="inlineStr">
+        <is>
+          <t>Pas de cote</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Millwall</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Swansea</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>1.870735020311852</v>
+      </c>
+      <c r="G103" t="n">
+        <v>1.48417037089417</v>
+      </c>
+      <c r="H103" t="n">
+        <v>0.4664907897836355</v>
+      </c>
+      <c r="I103" t="n">
+        <v>0.2278023084471008</v>
+      </c>
+      <c r="J103" t="n">
+        <v>0.3057069017692637</v>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Victoire Millwall</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N103" t="n">
+        <v>0.8498965584516748</v>
+      </c>
+      <c r="O103" t="n">
+        <v>0.6514789990366209</v>
+      </c>
+      <c r="P103" t="n">
+        <v>0.6561499962820434</v>
+      </c>
+      <c r="W103" t="inlineStr">
+        <is>
+          <t>Pas de cote</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Cardiff</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>1.885849458365065</v>
+      </c>
+      <c r="G104" t="n">
+        <v>1.314993295318606</v>
+      </c>
+      <c r="H104" t="n">
+        <v>0.5061599239765125</v>
+      </c>
+      <c r="I104" t="n">
+        <v>0.2285986132089722</v>
+      </c>
+      <c r="J104" t="n">
+        <v>0.2652414628145155</v>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Victoire Cardiff</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N104" t="n">
+        <v>0.8309278015239225</v>
+      </c>
+      <c r="O104" t="n">
+        <v>0.620270225199741</v>
+      </c>
+      <c r="P104" t="n">
+        <v>0.6225710444535784</v>
+      </c>
+      <c r="W104" t="inlineStr">
+        <is>
+          <t>Pas de cote</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Burnley</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Charlton</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>1.629425418120181</v>
+      </c>
+      <c r="G105" t="n">
+        <v>1.430353886066146</v>
+      </c>
+      <c r="H105" t="n">
+        <v>0.4216292406861701</v>
+      </c>
+      <c r="I105" t="n">
+        <v>0.2433947650600129</v>
+      </c>
+      <c r="J105" t="n">
+        <v>0.3349759942538171</v>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Victoire Burnley</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N105" t="n">
+        <v>0.8117900585506721</v>
+      </c>
+      <c r="O105" t="n">
+        <v>0.590068054484655</v>
+      </c>
+      <c r="P105" t="n">
+        <v>0.6138174288447785</v>
+      </c>
+      <c r="W105" t="inlineStr">
+        <is>
+          <t>Pas de cote</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Bristol City</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Blackburn</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>1.863579585582767</v>
+      </c>
+      <c r="G106" t="n">
+        <v>1.24404783964945</v>
+      </c>
+      <c r="H106" t="n">
+        <v>0.5169046793321698</v>
+      </c>
+      <c r="I106" t="n">
+        <v>0.230514390352963</v>
+      </c>
+      <c r="J106" t="n">
+        <v>0.2525809303148668</v>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>Victoire Bristol City</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N106" t="n">
+        <v>0.8184328641100521</v>
+      </c>
+      <c r="O106" t="n">
+        <v>0.6004838986613213</v>
+      </c>
+      <c r="P106" t="n">
+        <v>0.6034477764651902</v>
+      </c>
+      <c r="W106" t="inlineStr">
+        <is>
+          <t>Pas de cote</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Birmingham</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Preston NE</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>2.138529926579257</v>
+      </c>
+      <c r="G107" t="n">
+        <v>1.265410866706178</v>
+      </c>
+      <c r="H107" t="n">
+        <v>0.5717859553611343</v>
+      </c>
+      <c r="I107" t="n">
+        <v>0.2094143393240224</v>
+      </c>
+      <c r="J107" t="n">
+        <v>0.2187997053148433</v>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Victoire Birmingham</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>Elevee</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>2 - 1</t>
+        </is>
+      </c>
+      <c r="N107" t="n">
+        <v>0.8554010560411971</v>
+      </c>
+      <c r="O107" t="n">
+        <v>0.6610144368649541</v>
+      </c>
+      <c r="P107" t="n">
+        <v>0.6350885657743116</v>
+      </c>
+      <c r="W107" t="inlineStr">
+        <is>
+          <t>Pas de cote</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Stoke</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Middlesbrough</t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>1.563989621444187</v>
+      </c>
+      <c r="G108" t="n">
+        <v>1.829096938422859</v>
+      </c>
+      <c r="H108" t="n">
+        <v>0.3307015210891077</v>
+      </c>
+      <c r="I108" t="n">
+        <v>0.2285804287124483</v>
+      </c>
+      <c r="J108" t="n">
+        <v>0.4407180501984441</v>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Victoire Middlesbrough</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N108" t="n">
+        <v>0.8542932415439546</v>
+      </c>
+      <c r="O108" t="n">
+        <v>0.6589231091599292</v>
+      </c>
+      <c r="P108" t="n">
+        <v>0.6656689788642458</v>
+      </c>
+      <c r="W108" t="inlineStr">
+        <is>
+          <t>Pas de cote</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Atletico Madrid</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Manchester United</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>2.34661487987909</v>
+      </c>
+      <c r="G109" t="n">
+        <v>1.491975066709752</v>
+      </c>
+      <c r="H109" t="n">
+        <v>0.5030238591313618</v>
+      </c>
+      <c r="I109" t="n">
+        <v>0.2215093513669412</v>
+      </c>
+      <c r="J109" t="n">
+        <v>0.275466789501697</v>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>Victoire Atletico Madrid</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>Inter-champ.</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>2 - 1</t>
+        </is>
+      </c>
+      <c r="N109" t="n">
+        <v>0.8973580014539196</v>
+      </c>
+      <c r="O109" t="n">
+        <v>0.7372700207971709</v>
+      </c>
+      <c r="P109" t="n">
+        <v>0.7024078926980601</v>
+      </c>
+      <c r="Q109" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="R109" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="S109" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U109" t="n">
+        <v>0.1865374176540455</v>
+      </c>
+      <c r="V109" t="n">
+        <v>1.281132679450696</v>
+      </c>
+      <c r="W109" t="inlineStr">
+        <is>
+          <t>Ecart suspect</t>
+        </is>
+      </c>
+      <c r="X109" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Lille</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>1.752351817381355</v>
+      </c>
+      <c r="G110" t="n">
+        <v>0.8388993159386002</v>
+      </c>
+      <c r="H110" t="n">
+        <v>0.6720887358983385</v>
+      </c>
+      <c r="I110" t="n">
+        <v>0.1974018801223755</v>
+      </c>
+      <c r="J110" t="n">
+        <v>0.1305093839792862</v>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Victoire Arsenal</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>Inter-champ.</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>1 - 0</t>
+        </is>
+      </c>
+      <c r="N110" t="n">
+        <v>0.7331233133372206</v>
+      </c>
+      <c r="O110" t="n">
+        <v>0.4793705921077304</v>
+      </c>
+      <c r="P110" t="n">
+        <v>0.4715772048956923</v>
+      </c>
+      <c r="Q110" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="R110" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="S110" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U110" t="n">
+        <v>0.8761714696343508</v>
+      </c>
+      <c r="V110" t="n">
+        <v>2.017865401154752</v>
+      </c>
+      <c r="W110" t="inlineStr">
+        <is>
+          <t>Ecart suspect</t>
+        </is>
+      </c>
+      <c r="X110" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>RB Leipzig</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>PSV</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>2.302740787764551</v>
+      </c>
+      <c r="G111" t="n">
+        <v>2.846947581180713</v>
+      </c>
+      <c r="H111" t="n">
+        <v>0.3966771018146482</v>
+      </c>
+      <c r="I111" t="n">
+        <v>0.2059720404337906</v>
+      </c>
+      <c r="J111" t="n">
+        <v>0.3973508577515614</v>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Victoire PSV</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>Inter-champ.</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>2 - 2</t>
+        </is>
+      </c>
+      <c r="N111" t="n">
+        <v>0.9650773589320762</v>
+      </c>
+      <c r="O111" t="n">
+        <v>0.8873777523276902</v>
+      </c>
+      <c r="P111" t="n">
+        <v>0.8485437689991057</v>
+      </c>
+      <c r="Q111" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="R111" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="S111" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U111" t="n">
+        <v>0.6016115811288711</v>
+      </c>
+      <c r="V111" t="n">
+        <v>1.730461999342083</v>
+      </c>
+      <c r="W111" t="inlineStr">
+        <is>
+          <t>Ecart suspect</t>
+        </is>
+      </c>
+      <c r="X111" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Villarreal</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Naples</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>1.948346642971428</v>
+      </c>
+      <c r="G112" t="n">
+        <v>1.641562094661614</v>
+      </c>
+      <c r="H112" t="n">
+        <v>0.4429635312805151</v>
+      </c>
+      <c r="I112" t="n">
+        <v>0.2425587281573245</v>
+      </c>
+      <c r="J112" t="n">
+        <v>0.3144777405621603</v>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Victoire Villarreal</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>Inter-champ.</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N112" t="n">
+        <v>0.8750791755920148</v>
+      </c>
+      <c r="O112" t="n">
+        <v>0.6954600247402651</v>
+      </c>
+      <c r="P112" t="n">
+        <v>0.6931786695436087</v>
+      </c>
+      <c r="Q112" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="R112" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="S112" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U112" t="n">
+        <v>0.005764684538395404</v>
+      </c>
+      <c r="V112" t="n">
+        <v>1.087161977610017</v>
+      </c>
+      <c r="W112" t="inlineStr">
+        <is>
+          <t>Pas de valeur</t>
+        </is>
+      </c>
+      <c r="X112" t="inlineStr">
         <is>
           <t>Betclic</t>
         </is>
@@ -9808,12 +10856,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K99"/>
+  <dimension ref="A1:K112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
@@ -9908,16 +10956,16 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.7622768608319233</v>
+        <v>0.7618961130020734</v>
       </c>
       <c r="G2" t="n">
-        <v>1.210699300699301</v>
+        <v>1.215532286212915</v>
       </c>
       <c r="H2" t="n">
-        <v>1.311859314355461</v>
+        <v>1.312514899255404</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.07711193765153235</v>
+        <v>-0.07389067590585663</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -9952,16 +11000,16 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.7450814563214072</v>
+        <v>0.7436188211217682</v>
       </c>
       <c r="G3" t="n">
-        <v>1.264567669172932</v>
+        <v>1.270396975425331</v>
       </c>
       <c r="H3" t="n">
-        <v>1.342135133703593</v>
+        <v>1.344774999765974</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.05779407943566417</v>
+        <v>-0.0553088987775554</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -10050,16 +11098,16 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.7590642375602334</v>
+        <v>0.7588369494822158</v>
       </c>
       <c r="G6" t="n">
-        <v>1.237022132796781</v>
+        <v>1.239859437751004</v>
       </c>
       <c r="H6" t="n">
-        <v>1.317411558228822</v>
+        <v>1.317806151482659</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.06102073792347773</v>
+        <v>-0.05914884647029295</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -10138,16 +11186,16 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.7449374188725885</v>
+        <v>0.7434966917709676</v>
       </c>
       <c r="G8" t="n">
-        <v>1.212544483985765</v>
+        <v>1.220348432055749</v>
       </c>
       <c r="H8" t="n">
-        <v>1.342394642376042</v>
+        <v>1.344995897181541</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.09673024183144951</v>
+        <v>-0.09267497795866309</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -10361,16 +11409,16 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.7574231753268518</v>
+        <v>0.7565588329182169</v>
       </c>
       <c r="G15" t="n">
-        <v>1.226977687626775</v>
+        <v>1.231313131313131</v>
       </c>
       <c r="H15" t="n">
-        <v>1.320265912867624</v>
+        <v>1.321774271199473</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.07065866378253016</v>
+        <v>-0.06843917441686231</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -10432,16 +11480,16 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.726355352263742</v>
+        <v>0.7303894826169589</v>
       </c>
       <c r="G17" t="n">
-        <v>1.294691119691119</v>
+        <v>1.304310344827586</v>
       </c>
       <c r="H17" t="n">
-        <v>1.3767366026607</v>
+        <v>1.369132529697767</v>
       </c>
       <c r="I17" t="n">
-        <v>-0.05959417568401826</v>
+        <v>-0.04734544206943214</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -10476,16 +11524,16 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.7556431148928712</v>
+        <v>0.7562132954176031</v>
       </c>
       <c r="G18" t="n">
-        <v>1.228544423440454</v>
+        <v>1.225233644859813</v>
       </c>
       <c r="H18" t="n">
-        <v>1.323376049210442</v>
+        <v>1.322378231194376</v>
       </c>
       <c r="I18" t="n">
-        <v>-0.07165886508718911</v>
+        <v>-0.07346202776403954</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -10541,26 +11589,9 @@
           <t>Swansea - Norwich</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>12 (pas de nul)</t>
-        </is>
-      </c>
-      <c r="F20" t="n">
-        <v>0.7591264449198685</v>
-      </c>
-      <c r="G20" t="n">
-        <v>1.204761904761905</v>
-      </c>
-      <c r="H20" t="n">
-        <v>1.317303601649074</v>
-      </c>
-      <c r="I20" t="n">
-        <v>-0.08543337826320607</v>
-      </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Cote insuffisante</t>
+          <t>Aucune selection a ce seuil</t>
         </is>
       </c>
     </row>
@@ -10662,16 +11693,16 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.7386307837887051</v>
+        <v>0.7367800574742798</v>
       </c>
       <c r="G23" t="n">
-        <v>1.264388349514563</v>
+        <v>1.268810916179337</v>
       </c>
       <c r="H23" t="n">
-        <v>1.353856381222886</v>
+        <v>1.357257148663947</v>
       </c>
       <c r="I23" t="n">
-        <v>-0.06608384238475107</v>
+        <v>-0.06516542025339433</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -10706,16 +11737,16 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.7312866458563442</v>
+        <v>0.7325976171551107</v>
       </c>
       <c r="G24" t="n">
-        <v>1.245603112840467</v>
+        <v>1.281257142857143</v>
       </c>
       <c r="H24" t="n">
-        <v>1.367452839001305</v>
+        <v>1.365005804800854</v>
       </c>
       <c r="I24" t="n">
-        <v>-0.08910707754267355</v>
+        <v>-0.06135407017989181</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -10821,16 +11852,16 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>0.7704039655862822</v>
+        <v>0.7691465596785085</v>
       </c>
       <c r="G27" t="n">
-        <v>1.219919517102616</v>
+        <v>1.219919191919192</v>
       </c>
       <c r="H27" t="n">
-        <v>1.298020317482392</v>
+        <v>1.3001423297245</v>
       </c>
       <c r="I27" t="n">
-        <v>-0.06016916632804248</v>
+        <v>-0.06170335044956721</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -10913,9 +11944,26 @@
           <t>Sheffield Utd - Lincoln City</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>0.7411130045760173</v>
+      </c>
+      <c r="G30" t="n">
+        <v>1.204206500956023</v>
+      </c>
+      <c r="H30" t="n">
+        <v>1.349321889948604</v>
+      </c>
+      <c r="I30" t="n">
+        <v>-0.1075469019465092</v>
+      </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Aucune selection a ce seuil</t>
+          <t>Cote insuffisante</t>
         </is>
       </c>
     </row>
@@ -11125,16 +12173,16 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>0.7125486560278349</v>
+        <v>0.7117788837445219</v>
       </c>
       <c r="G37" t="n">
         <v>1.353982300884956</v>
       </c>
       <c r="H37" t="n">
-        <v>1.403412934036797</v>
+        <v>1.404930692435277</v>
       </c>
       <c r="I37" t="n">
-        <v>-0.03522173121894934</v>
+        <v>-0.03626398926626684</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -11196,16 +12244,16 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>0.7479966622412655</v>
+        <v>0.7477104724177691</v>
       </c>
       <c r="G39" t="n">
         <v>1.252087475149106</v>
       </c>
       <c r="H39" t="n">
-        <v>1.336904361315788</v>
+        <v>1.337416067968711</v>
       </c>
       <c r="I39" t="n">
-        <v>-0.06344274775437564</v>
+        <v>-0.06380108244789051</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -11240,16 +12288,16 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>0.7492823581290109</v>
+        <v>0.74870032084494</v>
       </c>
       <c r="G40" t="n">
-        <v>1.246372745490982</v>
+        <v>1.24662</v>
       </c>
       <c r="H40" t="n">
-        <v>1.334610363037295</v>
+        <v>1.335647884952764</v>
       </c>
       <c r="I40" t="n">
-        <v>-0.06611489015078753</v>
+        <v>-0.0666552060282809</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -11402,13 +12450,13 @@
         <v>0.7364086038126073</v>
       </c>
       <c r="G44" t="n">
-        <v>1.245062051645665</v>
+        <v>1.247736239173774</v>
       </c>
       <c r="H44" t="n">
         <v>1.35794176605583</v>
       </c>
       <c r="I44" t="n">
-        <v>-0.08312559288755528</v>
+        <v>-0.08115629818364745</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -11632,16 +12680,16 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>0.7447057212798476</v>
+        <v>0.7444177385133255</v>
       </c>
       <c r="G52" t="n">
-        <v>1.235674676524954</v>
+        <v>1.239393382352941</v>
       </c>
       <c r="H52" t="n">
-        <v>1.342812296757174</v>
+        <v>1.343331772288362</v>
       </c>
       <c r="I52" t="n">
-        <v>-0.07978599875124193</v>
+        <v>-0.07737358118044213</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -11676,16 +12724,16 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>0.7391606612918189</v>
+        <v>0.7395541303198983</v>
       </c>
       <c r="G53" t="n">
-        <v>1.275862068965517</v>
+        <v>1.274780952380952</v>
       </c>
       <c r="H53" t="n">
-        <v>1.352885850624567</v>
+        <v>1.352166067367434</v>
       </c>
       <c r="I53" t="n">
-        <v>-0.05693294938629989</v>
+        <v>-0.05723048141353315</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -11863,7 +12911,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -11959,20 +13007,20 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>12 (pas de nul)</t>
+          <t>Plus de 1,5 but</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>0.734211788319687</v>
+        <v>0.7436987278148628</v>
       </c>
       <c r="G63" t="n">
-        <v>1.24902</v>
+        <v>1.231926471990655</v>
       </c>
       <c r="H63" t="n">
-        <v>1.362004827365404</v>
+        <v>1.34463051044635</v>
       </c>
       <c r="I63" t="n">
-        <v>-0.08295479215294455</v>
+        <v>-0.08381785001909758</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -12220,16 +13268,16 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>0.7242530893212579</v>
+        <v>0.7243055770881572</v>
       </c>
       <c r="G70" t="n">
-        <v>1.286407766990291</v>
+        <v>1.285747572815534</v>
       </c>
       <c r="H70" t="n">
-        <v>1.380732805623462</v>
+        <v>1.380632748984463</v>
       </c>
       <c r="I70" t="n">
-        <v>-0.06831520063042085</v>
+        <v>-0.06872586228214728</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -12264,16 +13312,16 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>0.7219795216852268</v>
+        <v>0.7207085464931555</v>
       </c>
       <c r="G71" t="n">
-        <v>1.268512110726644</v>
+        <v>1.276860068259386</v>
       </c>
       <c r="H71" t="n">
-        <v>1.385080836733187</v>
+        <v>1.387523437686189</v>
       </c>
       <c r="I71" t="n">
-        <v>-0.08416023304566023</v>
+        <v>-0.07975603612962667</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -12396,16 +13444,16 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>0.7655288991343097</v>
+        <v>0.7677576040158446</v>
       </c>
       <c r="G74" t="n">
-        <v>1.255384615384615</v>
+        <v>1.25660091047041</v>
       </c>
       <c r="H74" t="n">
-        <v>1.306286413394504</v>
+        <v>1.302494426325946</v>
       </c>
       <c r="I74" t="n">
-        <v>-0.03896679739446673</v>
+        <v>-0.03523509577310946</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -12541,13 +13589,13 @@
         <v>0.7567423739018653</v>
       </c>
       <c r="G78" t="n">
-        <v>1.211952240414579</v>
+        <v>1.216392958928378</v>
       </c>
       <c r="H78" t="n">
         <v>1.321453686865539</v>
       </c>
       <c r="I78" t="n">
-        <v>-0.08286438453298717</v>
+        <v>-0.07950390466302515</v>
       </c>
       <c r="K78" t="inlineStr">
         <is>
@@ -12582,16 +13630,16 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>0.7629294816431714</v>
+        <v>0.763102729664263</v>
       </c>
       <c r="G79" t="n">
-        <v>1.234493927125506</v>
+        <v>1.232251521298174</v>
       </c>
       <c r="H79" t="n">
-        <v>1.310737131099239</v>
+        <v>1.310439553059865</v>
       </c>
       <c r="I79" t="n">
-        <v>-0.05816818808649471</v>
+        <v>-0.05966550046442243</v>
       </c>
       <c r="K79" t="inlineStr">
         <is>
@@ -12626,16 +13674,16 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>0.7545691798974303</v>
+        <v>0.7562324336492234</v>
       </c>
       <c r="G80" t="n">
-        <v>1.226495726495727</v>
+        <v>1.221575342465753</v>
       </c>
       <c r="H80" t="n">
-        <v>1.325259534368912</v>
+        <v>1.322344765318341</v>
       </c>
       <c r="I80" t="n">
-        <v>-0.07452412551041654</v>
+        <v>-0.07620510588123974</v>
       </c>
       <c r="K80" t="inlineStr">
         <is>
@@ -12724,16 +13772,16 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>0.7667091495439793</v>
+        <v>0.7675410416105048</v>
       </c>
       <c r="G83" t="n">
-        <v>1.211642599277978</v>
+        <v>1.207052441229656</v>
       </c>
       <c r="H83" t="n">
-        <v>1.304275552984827</v>
+        <v>1.302861926316975</v>
       </c>
       <c r="I83" t="n">
-        <v>-0.07102253315632479</v>
+        <v>-0.07353771198008685</v>
       </c>
       <c r="K83" t="inlineStr">
         <is>
@@ -12771,13 +13819,13 @@
         <v>0.7154791223096694</v>
       </c>
       <c r="G84" t="n">
-        <v>1.282879040322057</v>
+        <v>1.281118683806446</v>
       </c>
       <c r="H84" t="n">
         <v>1.397664821821574</v>
       </c>
       <c r="I84" t="n">
-        <v>-0.08212683020090394</v>
+        <v>-0.08338632853564532</v>
       </c>
       <c r="K84" t="inlineStr">
         <is>
@@ -12839,16 +13887,16 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>0.7685511160822698</v>
+        <v>0.7687305250139929</v>
       </c>
       <c r="G86" t="n">
-        <v>1.249596928982726</v>
+        <v>1.247300970873787</v>
       </c>
       <c r="H86" t="n">
-        <v>1.301149629575133</v>
+        <v>1.300845962870796</v>
       </c>
       <c r="I86" t="n">
-        <v>-0.03962088557734944</v>
+        <v>-0.04116166980973102</v>
       </c>
       <c r="K86" t="inlineStr">
         <is>
@@ -13079,16 +14127,16 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>0.743803300193371</v>
+        <v>0.7417049185991655</v>
       </c>
       <c r="G93" t="n">
-        <v>1.279158699808795</v>
+        <v>1.285714285714286</v>
       </c>
       <c r="H93" t="n">
-        <v>1.344441466903984</v>
+        <v>1.348245070140115</v>
       </c>
       <c r="I93" t="n">
-        <v>-0.04855753761115633</v>
+        <v>-0.04637939037250138</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -13338,6 +14386,442 @@
         <v>-0.07364689741923591</v>
       </c>
       <c r="K99" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Lens - Sporting CP</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>0.7778504666386616</v>
+      </c>
+      <c r="G100" t="n">
+        <v>1.239839034205231</v>
+      </c>
+      <c r="H100" t="n">
+        <v>1.285594137805582</v>
+      </c>
+      <c r="I100" t="n">
+        <v>-0.0355906286866331</v>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Wolverhampton - Bolton</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Wrexham - West Brom</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Millwall - Swansea</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Cardiff - Watford</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Burnley - Charlton</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Bristol City - Blackburn</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Birmingham - Preston NE</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Stoke - Middlesbrough</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Atletico Madrid - Manchester United</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>1N (ne perd pas domicile)</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>0.724533210498303</v>
+      </c>
+      <c r="G109" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="H109" t="n">
+        <v>1.380198982614258</v>
+      </c>
+      <c r="I109" t="n">
+        <v>-0.02188016582729091</v>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Arsenal - Lille</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Plus de 1,5 but</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>0.7331233133372206</v>
+      </c>
+      <c r="G110" t="n">
+        <v>1.268245422025781</v>
+      </c>
+      <c r="H110" t="n">
+        <v>1.36402700856414</v>
+      </c>
+      <c r="I110" t="n">
+        <v>-0.07021971407969774</v>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>RB Leipzig - PSV</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>0.7940279595662096</v>
+      </c>
+      <c r="G111" t="n">
+        <v>1.208771929824561</v>
+      </c>
+      <c r="H111" t="n">
+        <v>1.259401495819261</v>
+      </c>
+      <c r="I111" t="n">
+        <v>-0.04020129098049419</v>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Villarreal - Naples</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>0.7574412718426754</v>
+      </c>
+      <c r="G112" t="n">
+        <v>1.257519230769231</v>
+      </c>
+      <c r="H112" t="n">
+        <v>1.320234369546878</v>
+      </c>
+      <c r="I112" t="n">
+        <v>-0.04750303447953108</v>
+      </c>
+      <c r="K112" t="inlineStr">
         <is>
           <t>Cote insuffisante</t>
         </is>

</xml_diff>

<commit_message>
Actualisation du 07/10/2026 11:56 UTC
</commit_message>
<xml_diff>
--- a/classeur/Analyse_football_paris_sportifs.xlsx
+++ b/classeur/Analyse_football_paris_sportifs.xlsx
@@ -452,7 +452,7 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Copie automatique du 2026-10-06T12:10+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
+          <t>Copie automatique du 2026-10-07T11:56+00:00. Ce fichier ne calcule rien : il reprend en valeurs</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fenetre : 2026-10-06 au 2026-10-13. Competitions : Brasileirao, Bundesliga, Championship, Eredivisie, Liga, Ligue 1, Ligue des Champions, Premier League, Primeira Liga, Serie A.</t>
+          <t>Fenetre : 2026-10-07 au 2026-10-14. Competitions : Brasileirao, Bundesliga, Championship, Eredivisie, Liga, Ligue 1, Ligue des Champions, Premier League, Primeira Liga, Serie A.</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X112"/>
+  <dimension ref="A1:X120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -872,13 +872,13 @@
         <v>2.015729155698191</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4061855206938333</v>
+        <v>0.41965925985278</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2381038869979266</v>
+        <v>0.2332586373536886</v>
       </c>
       <c r="J2" t="n">
-        <v>0.3557105923082401</v>
+        <v>0.3470821027935315</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -905,13 +905,13 @@
         <v>0.6846093035344661</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.75</v>
+        <v>1.66</v>
       </c>
       <c r="R2" t="n">
-        <v>3.5</v>
+        <v>3.63</v>
       </c>
       <c r="S2" t="n">
-        <v>3.98</v>
+        <v>4.3</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -919,10 +919,10 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0.9292542422347312</v>
+        <v>1.084370161208378</v>
       </c>
       <c r="V2" t="n">
-        <v>2.138383740136701</v>
+        <v>2.314588578199649</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
@@ -968,13 +968,13 @@
         <v>1.51525557507413</v>
       </c>
       <c r="H3" t="n">
-        <v>0.4524175148012684</v>
+        <v>0.4476316100673187</v>
       </c>
       <c r="I3" t="n">
-        <v>0.2563811788782319</v>
+        <v>0.2578799339514747</v>
       </c>
       <c r="J3" t="n">
-        <v>0.2912013063204998</v>
+        <v>0.2944884559812066</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -983,7 +983,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Moyenne</t>
+          <t>Faible</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -1001,24 +1001,24 @@
         <v>0.6721505377373731</v>
       </c>
       <c r="Q3" t="n">
-        <v>2.12</v>
+        <v>2.17</v>
       </c>
       <c r="R3" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="S3" t="n">
         <v>3.1</v>
       </c>
-      <c r="S3" t="n">
-        <v>3.17</v>
-      </c>
       <c r="T3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="U3" t="n">
-        <v>0.0171351819161798</v>
+        <v>0.04112421922552345</v>
       </c>
       <c r="V3" t="n">
-        <v>1.128751702797689</v>
+        <v>1.154755678688872</v>
       </c>
       <c r="W3" t="inlineStr">
         <is>
@@ -1135,13 +1135,13 @@
         <v>1.387510371952636</v>
       </c>
       <c r="H5" t="n">
-        <v>0.5343971985492191</v>
+        <v>0.5565175233447721</v>
       </c>
       <c r="I5" t="n">
-        <v>0.2352147355784542</v>
+        <v>0.2247109640089243</v>
       </c>
       <c r="J5" t="n">
-        <v>0.2303880658723265</v>
+        <v>0.2187715126463034</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Moyenne</t>
+          <t>Elevee</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -1168,13 +1168,13 @@
         <v>0.6458611013694736</v>
       </c>
       <c r="Q5" t="n">
-        <v>1.6</v>
+        <v>1.48</v>
       </c>
       <c r="R5" t="n">
-        <v>3.65</v>
+        <v>3.98</v>
       </c>
       <c r="S5" t="n">
-        <v>4.75</v>
+        <v>5.4</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
@@ -1182,10 +1182,10 @@
         </is>
       </c>
       <c r="U5" t="n">
-        <v>0.2873788522512397</v>
+        <v>0.4635464846645674</v>
       </c>
       <c r="V5" t="n">
-        <v>1.428345444310113</v>
+        <v>1.627635134101384</v>
       </c>
       <c r="W5" t="inlineStr">
         <is>
@@ -1231,13 +1231,13 @@
         <v>1.326182713580325</v>
       </c>
       <c r="H6" t="n">
-        <v>0.4506801536040676</v>
+        <v>0.4366794751211818</v>
       </c>
       <c r="I6" t="n">
-        <v>0.2411630505177842</v>
+        <v>0.2375726862388713</v>
       </c>
       <c r="J6" t="n">
-        <v>0.3081567958781482</v>
+        <v>0.3257478386399469</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -1264,13 +1264,13 @@
         <v>0.6509078176668402</v>
       </c>
       <c r="Q6" t="n">
-        <v>2.65</v>
+        <v>2.88</v>
       </c>
       <c r="R6" t="n">
-        <v>3.3</v>
+        <v>3.38</v>
       </c>
       <c r="S6" t="n">
-        <v>2.33</v>
+        <v>2.13</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
@@ -1278,10 +1278,10 @@
         </is>
       </c>
       <c r="U6" t="n">
-        <v>0.4873574956151483</v>
+        <v>0.6164489008949536</v>
       </c>
       <c r="V6" t="n">
-        <v>1.650332228575254</v>
+        <v>1.798402496872085</v>
       </c>
       <c r="W6" t="inlineStr">
         <is>
@@ -1327,13 +1327,13 @@
         <v>1.071958582850389</v>
       </c>
       <c r="H7" t="n">
-        <v>0.4985534468391626</v>
+        <v>0.4996365557124051</v>
       </c>
       <c r="I7" t="n">
-        <v>0.2602563765398065</v>
+        <v>0.2593023275514719</v>
       </c>
       <c r="J7" t="n">
-        <v>0.241190176621031</v>
+        <v>0.2410611167361231</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -1360,10 +1360,10 @@
         <v>0.5329508602473002</v>
       </c>
       <c r="Q7" t="n">
-        <v>1.83</v>
+        <v>1.82</v>
       </c>
       <c r="R7" t="n">
-        <v>3.33</v>
+        <v>3.35</v>
       </c>
       <c r="S7" t="n">
         <v>3.8</v>
@@ -1377,7 +1377,7 @@
         <v>-0.06793162825432464</v>
       </c>
       <c r="V7" t="n">
-        <v>1.034508541491024</v>
+        <v>1.03563599414073</v>
       </c>
       <c r="W7" t="inlineStr">
         <is>
@@ -1423,13 +1423,13 @@
         <v>1.609501646597387</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2014382694120476</v>
+        <v>0.201931620697129</v>
       </c>
       <c r="I8" t="n">
-        <v>0.2565033082290326</v>
+        <v>0.2568360396464877</v>
       </c>
       <c r="J8" t="n">
-        <v>0.5420584223589199</v>
+        <v>0.5412323396563834</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -1456,10 +1456,10 @@
         <v>0.4326093754136387</v>
       </c>
       <c r="Q8" t="n">
-        <v>3.98</v>
+        <v>3.95</v>
       </c>
       <c r="R8" t="n">
-        <v>3.47</v>
+        <v>3.45</v>
       </c>
       <c r="S8" t="n">
         <v>1.76</v>
@@ -1473,7 +1473,7 @@
         <v>0.005211002203980852</v>
       </c>
       <c r="V8" t="n">
-        <v>1.113394361113964</v>
+        <v>1.116991920800162</v>
       </c>
       <c r="W8" t="inlineStr">
         <is>
@@ -1590,13 +1590,13 @@
         <v>1.306897846560767</v>
       </c>
       <c r="H10" t="n">
-        <v>0.6164395991768743</v>
+        <v>0.6156427069908121</v>
       </c>
       <c r="I10" t="n">
-        <v>0.2083930590145646</v>
+        <v>0.2081097195706315</v>
       </c>
       <c r="J10" t="n">
-        <v>0.1751673418085612</v>
+        <v>0.1762475734385567</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1629,7 +1629,7 @@
         <v>4.05</v>
       </c>
       <c r="S10" t="n">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
@@ -1637,10 +1637,10 @@
         </is>
       </c>
       <c r="U10" t="n">
-        <v>0.1995011379144342</v>
+        <v>0.1795094522825271</v>
       </c>
       <c r="V10" t="n">
-        <v>1.329076878121241</v>
+        <v>1.310257544424538</v>
       </c>
       <c r="W10" t="inlineStr">
         <is>
@@ -1686,13 +1686,13 @@
         <v>0.7403710307211662</v>
       </c>
       <c r="H11" t="n">
-        <v>0.6449614567710117</v>
+        <v>0.648850750464105</v>
       </c>
       <c r="I11" t="n">
-        <v>0.2095448577541949</v>
+        <v>0.2081044785699966</v>
       </c>
       <c r="J11" t="n">
-        <v>0.1454936854747935</v>
+        <v>0.1430447709658985</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1719,13 +1719,13 @@
         <v>0.4599427603142682</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.49</v>
+        <v>1.47</v>
       </c>
       <c r="R11" t="n">
-        <v>4.05</v>
+        <v>4.1</v>
       </c>
       <c r="S11" t="n">
-        <v>5.25</v>
+        <v>5.4</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
@@ -1733,10 +1733,10 @@
         </is>
       </c>
       <c r="U11" t="n">
-        <v>0.01989015121477355</v>
+        <v>0.006200350527326925</v>
       </c>
       <c r="V11" t="n">
-        <v>1.130579553774913</v>
+        <v>1.116238152258944</v>
       </c>
       <c r="W11" t="inlineStr">
         <is>
@@ -1974,13 +1974,13 @@
         <v>0.7459017889013188</v>
       </c>
       <c r="H14" t="n">
-        <v>0.7641387855868687</v>
+        <v>0.7709071247944488</v>
       </c>
       <c r="I14" t="n">
-        <v>0.1394989152886915</v>
+        <v>0.1376578292905821</v>
       </c>
       <c r="J14" t="n">
-        <v>0.09636229912443983</v>
+        <v>0.09143504591496912</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -2007,13 +2007,13 @@
         <v>0.5035111033622247</v>
       </c>
       <c r="Q14" t="n">
-        <v>1.33</v>
+        <v>1.3</v>
       </c>
       <c r="R14" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="S14" t="n">
-        <v>6.75</v>
+        <v>7.25</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
@@ -2021,10 +2021,10 @@
         </is>
       </c>
       <c r="U14" t="n">
-        <v>0.1111311096148815</v>
+        <v>0.08606800187920749</v>
       </c>
       <c r="V14" t="n">
-        <v>1.205813961060761</v>
+        <v>1.182706316972872</v>
       </c>
       <c r="W14" t="inlineStr">
         <is>
@@ -2237,13 +2237,13 @@
         <v>1.509315576065982</v>
       </c>
       <c r="H17" t="n">
-        <v>0.3741914589951574</v>
+        <v>0.3655960268161452</v>
       </c>
       <c r="I17" t="n">
-        <v>0.2696105173830409</v>
+        <v>0.2691914073904897</v>
       </c>
       <c r="J17" t="n">
-        <v>0.3561980236218015</v>
+        <v>0.365212565793365</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -2270,13 +2270,13 @@
         <v>0.6165787364946821</v>
       </c>
       <c r="Q17" t="n">
-        <v>2.55</v>
+        <v>2.67</v>
       </c>
       <c r="R17" t="n">
         <v>3.12</v>
       </c>
       <c r="S17" t="n">
-        <v>2.67</v>
+        <v>2.53</v>
       </c>
       <c r="T17" t="inlineStr">
         <is>
@@ -2284,10 +2284,10 @@
         </is>
       </c>
       <c r="U17" t="n">
-        <v>-0.01141624062580793</v>
+        <v>0.03510534805062471</v>
       </c>
       <c r="V17" t="n">
-        <v>1.074789764320383</v>
+        <v>1.128576988905159</v>
       </c>
       <c r="W17" t="inlineStr">
         <is>
@@ -2500,13 +2500,13 @@
         <v>1.541288913531921</v>
       </c>
       <c r="H20" t="n">
-        <v>0.4514170763615597</v>
+        <v>0.4575652893519966</v>
       </c>
       <c r="I20" t="n">
-        <v>0.2395548890600154</v>
+        <v>0.2386642738865024</v>
       </c>
       <c r="J20" t="n">
-        <v>0.3090280345784251</v>
+        <v>0.3037704367615012</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -2533,13 +2533,13 @@
         <v>0.6948602572676411</v>
       </c>
       <c r="Q20" t="n">
-        <v>2.25</v>
+        <v>2.18</v>
       </c>
       <c r="R20" t="n">
-        <v>3.28</v>
+        <v>3.3</v>
       </c>
       <c r="S20" t="n">
-        <v>2.57</v>
+        <v>2.65</v>
       </c>
       <c r="T20" t="inlineStr">
         <is>
@@ -2547,10 +2547,10 @@
         </is>
       </c>
       <c r="U20" t="n">
-        <v>0.1529722419439956</v>
+        <v>0.1171019944168492</v>
       </c>
       <c r="V20" t="n">
-        <v>1.312575366448333</v>
+        <v>1.272495785836011</v>
       </c>
       <c r="W20" t="inlineStr">
         <is>
@@ -2788,13 +2788,13 @@
         <v>1.258903593920413</v>
       </c>
       <c r="H23" t="n">
-        <v>0.3902030896943928</v>
+        <v>0.4016170187773654</v>
       </c>
       <c r="I23" t="n">
-        <v>0.2632199425257202</v>
+        <v>0.2635538618679668</v>
       </c>
       <c r="J23" t="n">
-        <v>0.3465769677798869</v>
+        <v>0.3348291193546677</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -2821,13 +2821,13 @@
         <v>0.576945687615827</v>
       </c>
       <c r="Q23" t="n">
-        <v>2.83</v>
+        <v>2.65</v>
       </c>
       <c r="R23" t="n">
         <v>3.3</v>
       </c>
       <c r="S23" t="n">
-        <v>2.3</v>
+        <v>2.45</v>
       </c>
       <c r="T23" t="inlineStr">
         <is>
@@ -2835,10 +2835,10 @@
         </is>
       </c>
       <c r="U23" t="n">
-        <v>0.2921018385534442</v>
+        <v>0.2099186827443911</v>
       </c>
       <c r="V23" t="n">
-        <v>1.409902507577649</v>
+        <v>1.317059473205963</v>
       </c>
       <c r="W23" t="inlineStr">
         <is>
@@ -2884,13 +2884,13 @@
         <v>1.337395419164045</v>
       </c>
       <c r="H24" t="n">
-        <v>0.3634928172953928</v>
+        <v>0.3626771830498831</v>
       </c>
       <c r="I24" t="n">
-        <v>0.2674023828448891</v>
+        <v>0.2689024191660137</v>
       </c>
       <c r="J24" t="n">
-        <v>0.369104799859718</v>
+        <v>0.3684203977841031</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -2917,13 +2917,13 @@
         <v>0.584803544793031</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.03</v>
+        <v>3.05</v>
       </c>
       <c r="R24" t="n">
-        <v>3.23</v>
+        <v>3.2</v>
       </c>
       <c r="S24" t="n">
-        <v>2.22</v>
+        <v>2.23</v>
       </c>
       <c r="T24" t="inlineStr">
         <is>
@@ -2931,10 +2931,10 @@
         </is>
       </c>
       <c r="U24" t="n">
-        <v>0.2854034317825553</v>
+        <v>0.2938879428834302</v>
       </c>
       <c r="V24" t="n">
-        <v>1.401193828718883</v>
+        <v>1.408784345662726</v>
       </c>
       <c r="W24" t="inlineStr">
         <is>
@@ -2980,13 +2980,13 @@
         <v>2.11736404323407</v>
       </c>
       <c r="H25" t="n">
-        <v>0.3145395999434535</v>
+        <v>0.3138516456563984</v>
       </c>
       <c r="I25" t="n">
-        <v>0.2272380356515361</v>
+        <v>0.2281077910244806</v>
       </c>
       <c r="J25" t="n">
-        <v>0.4582223644050104</v>
+        <v>0.4580405633191209</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -3013,10 +3013,10 @@
         <v>0.7179591329146391</v>
       </c>
       <c r="Q25" t="n">
-        <v>2.87</v>
+        <v>2.88</v>
       </c>
       <c r="R25" t="n">
-        <v>3.78</v>
+        <v>3.75</v>
       </c>
       <c r="S25" t="n">
         <v>2.1</v>
@@ -3030,7 +3030,7 @@
         <v>0.006405968415735597</v>
       </c>
       <c r="V25" t="n">
-        <v>1.096150003023462</v>
+        <v>1.097062379062709</v>
       </c>
       <c r="W25" t="inlineStr">
         <is>
@@ -3076,13 +3076,13 @@
         <v>2.16032619526544</v>
       </c>
       <c r="H26" t="n">
-        <v>0.2359769798817941</v>
+        <v>0.2361935659580168</v>
       </c>
       <c r="I26" t="n">
-        <v>0.2068268507105566</v>
+        <v>0.2059334331461383</v>
       </c>
       <c r="J26" t="n">
-        <v>0.5571961694076493</v>
+        <v>0.557873000895845</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -3112,7 +3112,7 @@
         <v>4.75</v>
       </c>
       <c r="R26" t="n">
-        <v>4.5</v>
+        <v>4.55</v>
       </c>
       <c r="S26" t="n">
         <v>1.52</v>
@@ -3126,7 +3126,7 @@
         <v>0.3248912284480898</v>
       </c>
       <c r="V26" t="n">
-        <v>1.4449837082197</v>
+        <v>1.441748320604442</v>
       </c>
       <c r="W26" t="inlineStr">
         <is>
@@ -3172,13 +3172,13 @@
         <v>2.109890993669715</v>
       </c>
       <c r="H27" t="n">
-        <v>0.3553937966639609</v>
+        <v>0.3538535859278235</v>
       </c>
       <c r="I27" t="n">
-        <v>0.2308534403214916</v>
+        <v>0.2320996851552005</v>
       </c>
       <c r="J27" t="n">
-        <v>0.4137527630145476</v>
+        <v>0.4140467289169762</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -3205,10 +3205,10 @@
         <v>0.7011060068226381</v>
       </c>
       <c r="Q27" t="n">
-        <v>2.18</v>
+        <v>2.2</v>
       </c>
       <c r="R27" t="n">
-        <v>3.68</v>
+        <v>3.65</v>
       </c>
       <c r="S27" t="n">
         <v>2.77</v>
@@ -3222,7 +3222,7 @@
         <v>0.3759909882085071</v>
       </c>
       <c r="V27" t="n">
-        <v>1.501846770495773</v>
+        <v>1.499181930744323</v>
       </c>
       <c r="W27" t="inlineStr">
         <is>
@@ -3364,13 +3364,13 @@
         <v>4.091636529830818</v>
       </c>
       <c r="H29" t="n">
-        <v>0.07763878760763415</v>
+        <v>0.07647913985268912</v>
       </c>
       <c r="I29" t="n">
-        <v>0.1024341486337306</v>
+        <v>0.1005325965579631</v>
       </c>
       <c r="J29" t="n">
-        <v>0.8199270637586351</v>
+        <v>0.8229882635893477</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -3397,13 +3397,13 @@
         <v>0.7015799731548024</v>
       </c>
       <c r="Q29" t="n">
-        <v>10</v>
+        <v>10.25</v>
       </c>
       <c r="R29" t="n">
-        <v>7.75</v>
+        <v>8</v>
       </c>
       <c r="S29" t="n">
-        <v>1.16</v>
+        <v>1.15</v>
       </c>
       <c r="T29" t="inlineStr">
         <is>
@@ -3411,10 +3411,10 @@
         </is>
       </c>
       <c r="U29" t="n">
-        <v>-0.01427446236032115</v>
+        <v>-0.02277209630549082</v>
       </c>
       <c r="V29" t="n">
-        <v>1.075526340234439</v>
+        <v>1.067256190156291</v>
       </c>
       <c r="W29" t="inlineStr">
         <is>
@@ -3460,13 +3460,13 @@
         <v>1.278946641111108</v>
       </c>
       <c r="H30" t="n">
-        <v>0.4628024512933257</v>
+        <v>0.4510295008491559</v>
       </c>
       <c r="I30" t="n">
-        <v>0.2588869954239827</v>
+        <v>0.2623414822368209</v>
       </c>
       <c r="J30" t="n">
-        <v>0.2783105532826916</v>
+        <v>0.2866290169140232</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -3493,13 +3493,13 @@
         <v>0.5853904950683293</v>
       </c>
       <c r="Q30" t="n">
-        <v>1.88</v>
+        <v>1.98</v>
       </c>
       <c r="R30" t="n">
-        <v>3.23</v>
+        <v>3.15</v>
       </c>
       <c r="S30" t="n">
-        <v>3.35</v>
+        <v>3.15</v>
       </c>
       <c r="T30" t="inlineStr">
         <is>
@@ -3507,10 +3507,10 @@
         </is>
       </c>
       <c r="U30" t="n">
-        <v>-0.01249697908110758</v>
+        <v>-0.07145238331507131</v>
       </c>
       <c r="V30" t="n">
-        <v>1.125773074936952</v>
+        <v>1.058517485109803</v>
       </c>
       <c r="W30" t="inlineStr">
         <is>
@@ -4032,13 +4032,13 @@
         <v>1.867601730563736</v>
       </c>
       <c r="H37" t="n">
-        <v>0.2882211162554782</v>
+        <v>0.2871945054024257</v>
       </c>
       <c r="I37" t="n">
-        <v>0.2497766782329458</v>
+        <v>0.2506653921421936</v>
       </c>
       <c r="J37" t="n">
-        <v>0.4620022055115761</v>
+        <v>0.4621401024553807</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -4065,10 +4065,10 @@
         <v>0.6047993974448378</v>
       </c>
       <c r="Q37" t="n">
-        <v>2.83</v>
+        <v>2.85</v>
       </c>
       <c r="R37" t="n">
-        <v>3.4</v>
+        <v>3.38</v>
       </c>
       <c r="S37" t="n">
         <v>2.25</v>
@@ -4082,7 +4082,7 @@
         <v>0.1631910623050006</v>
       </c>
       <c r="V37" t="n">
-        <v>1.270110400580108</v>
+        <v>1.269250387858607</v>
       </c>
       <c r="W37" t="inlineStr">
         <is>
@@ -4128,13 +4128,13 @@
         <v>1.739432984348578</v>
       </c>
       <c r="H38" t="n">
-        <v>0.5272823352564746</v>
+        <v>0.5279836481308295</v>
       </c>
       <c r="I38" t="n">
-        <v>0.2151947581392757</v>
+        <v>0.2154787465624713</v>
       </c>
       <c r="J38" t="n">
-        <v>0.2575229066042498</v>
+        <v>0.2565376053066992</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
@@ -4167,7 +4167,7 @@
         <v>4.05</v>
       </c>
       <c r="S38" t="n">
-        <v>4.25</v>
+        <v>4.3</v>
       </c>
       <c r="T38" t="inlineStr">
         <is>
@@ -4175,10 +4175,10 @@
         </is>
       </c>
       <c r="U38" t="n">
-        <v>0.2731634282565141</v>
+        <v>0.2881418215301199</v>
       </c>
       <c r="V38" t="n">
-        <v>1.390248369353416</v>
+        <v>1.403079904693197</v>
       </c>
       <c r="W38" t="inlineStr">
         <is>
@@ -4224,13 +4224,13 @@
         <v>1.34184830221176</v>
       </c>
       <c r="H39" t="n">
-        <v>0.4077760090530064</v>
+        <v>0.4026569522658787</v>
       </c>
       <c r="I39" t="n">
-        <v>0.2522895275822308</v>
+        <v>0.2526432760540198</v>
       </c>
       <c r="J39" t="n">
-        <v>0.3399344633647627</v>
+        <v>0.3446997716801016</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -4257,13 +4257,13 @@
         <v>0.6148596020833412</v>
       </c>
       <c r="Q39" t="n">
-        <v>2.68</v>
+        <v>2.77</v>
       </c>
       <c r="R39" t="n">
         <v>3.42</v>
       </c>
       <c r="S39" t="n">
-        <v>2.35</v>
+        <v>2.3</v>
       </c>
       <c r="T39" t="inlineStr">
         <is>
@@ -4271,10 +4271,10 @@
         </is>
       </c>
       <c r="U39" t="n">
-        <v>0.2691428094585586</v>
+        <v>0.311763276940376</v>
       </c>
       <c r="V39" t="n">
-        <v>1.384715908510908</v>
+        <v>1.42744912306252</v>
       </c>
       <c r="W39" t="inlineStr">
         <is>
@@ -4320,13 +4320,13 @@
         <v>1.642979463599926</v>
       </c>
       <c r="H40" t="n">
-        <v>0.3585809255499413</v>
+        <v>0.3607328521714681</v>
       </c>
       <c r="I40" t="n">
-        <v>0.25129967915506</v>
+        <v>0.2514075663123865</v>
       </c>
       <c r="J40" t="n">
-        <v>0.3901193952949987</v>
+        <v>0.3878595815161454</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -4353,13 +4353,13 @@
         <v>0.6432708745489725</v>
       </c>
       <c r="Q40" t="n">
-        <v>2.63</v>
+        <v>2.6</v>
       </c>
       <c r="R40" t="n">
         <v>3.45</v>
       </c>
       <c r="S40" t="n">
-        <v>2.37</v>
+        <v>2.4</v>
       </c>
       <c r="T40" t="inlineStr">
         <is>
@@ -4367,10 +4367,10 @@
         </is>
       </c>
       <c r="U40" t="n">
-        <v>-0.02959500600719667</v>
+        <v>-0.04066426449380645</v>
       </c>
       <c r="V40" t="n">
-        <v>1.059705676703192</v>
+        <v>1.046766835146808</v>
       </c>
       <c r="W40" t="inlineStr">
         <is>
@@ -4416,13 +4416,13 @@
         <v>1.816159781941692</v>
       </c>
       <c r="H41" t="n">
-        <v>0.2570834246396049</v>
+        <v>0.2572523415681667</v>
       </c>
       <c r="I41" t="n">
-        <v>0.2439821309418515</v>
+        <v>0.2448852933535652</v>
       </c>
       <c r="J41" t="n">
-        <v>0.4989344444185437</v>
+        <v>0.4978623650782682</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -4452,10 +4452,10 @@
         <v>4.05</v>
       </c>
       <c r="R41" t="n">
-        <v>3.6</v>
+        <v>3.58</v>
       </c>
       <c r="S41" t="n">
-        <v>1.77</v>
+        <v>1.78</v>
       </c>
       <c r="T41" t="inlineStr">
         <is>
@@ -4466,7 +4466,7 @@
         <v>0.1646609052072994</v>
       </c>
       <c r="V41" t="n">
-        <v>1.269088023408038</v>
+        <v>1.267198748405859</v>
       </c>
       <c r="W41" t="inlineStr">
         <is>
@@ -4608,13 +4608,13 @@
         <v>1.613835703805611</v>
       </c>
       <c r="H43" t="n">
-        <v>0.2036774011183924</v>
+        <v>0.2063634430609084</v>
       </c>
       <c r="I43" t="n">
-        <v>0.2682603793988715</v>
+        <v>0.26966234875527</v>
       </c>
       <c r="J43" t="n">
-        <v>0.5280622194827358</v>
+        <v>0.5239742081838216</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
@@ -4641,13 +4641,13 @@
         <v>0.4573326878990664</v>
       </c>
       <c r="Q43" t="n">
-        <v>4.15</v>
+        <v>4.05</v>
       </c>
       <c r="R43" t="n">
-        <v>3.15</v>
+        <v>3.12</v>
       </c>
       <c r="S43" t="n">
-        <v>1.78</v>
+        <v>1.81</v>
       </c>
       <c r="T43" t="inlineStr">
         <is>
@@ -4655,10 +4655,10 @@
         </is>
       </c>
       <c r="U43" t="n">
-        <v>-0.01277875874542511</v>
+        <v>0.00385980150043852</v>
       </c>
       <c r="V43" t="n">
-        <v>1.105906879961252</v>
+        <v>1.124235228894895</v>
       </c>
       <c r="W43" t="inlineStr">
         <is>
@@ -4704,13 +4704,13 @@
         <v>0.6984852279550878</v>
       </c>
       <c r="H44" t="n">
-        <v>0.6603809715201751</v>
+        <v>0.6588468411429533</v>
       </c>
       <c r="I44" t="n">
-        <v>0.205682011857071</v>
+        <v>0.2059309173718862</v>
       </c>
       <c r="J44" t="n">
-        <v>0.1339370166227539</v>
+        <v>0.1352222414851603</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -4737,13 +4737,13 @@
         <v>0.4302673558662803</v>
       </c>
       <c r="Q44" t="n">
-        <v>1.39</v>
+        <v>1.4</v>
       </c>
       <c r="R44" t="n">
         <v>4.65</v>
       </c>
       <c r="S44" t="n">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="T44" t="inlineStr">
         <is>
@@ -4754,7 +4754,7 @@
         <v>-0.006000991545592194</v>
       </c>
       <c r="V44" t="n">
-        <v>1.081793352329117</v>
+        <v>1.079074864448754</v>
       </c>
       <c r="W44" t="inlineStr">
         <is>
@@ -4800,13 +4800,13 @@
         <v>0.6525267046466084</v>
       </c>
       <c r="H45" t="n">
-        <v>0.8395114742348266</v>
+        <v>0.8386190624411948</v>
       </c>
       <c r="I45" t="n">
-        <v>0.1074465067284379</v>
+        <v>0.1073175388305195</v>
       </c>
       <c r="J45" t="n">
-        <v>0.05304201903673553</v>
+        <v>0.05406339872828569</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
@@ -4839,7 +4839,7 @@
         <v>7.75</v>
       </c>
       <c r="S45" t="n">
-        <v>14.75</v>
+        <v>14.25</v>
       </c>
       <c r="T45" t="inlineStr">
         <is>
@@ -4850,7 +4850,7 @@
         <v>-0.03718984470798536</v>
       </c>
       <c r="V45" t="n">
-        <v>1.049160757558206</v>
+        <v>1.051451117725419</v>
       </c>
       <c r="W45" t="inlineStr">
         <is>
@@ -4896,13 +4896,13 @@
         <v>1.669079606418681</v>
       </c>
       <c r="H46" t="n">
-        <v>0.6562688951096317</v>
+        <v>0.6548659963006653</v>
       </c>
       <c r="I46" t="n">
-        <v>0.1688178055510744</v>
+        <v>0.1690288237117528</v>
       </c>
       <c r="J46" t="n">
-        <v>0.1749132993392939</v>
+        <v>0.1761051799875817</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
@@ -4929,13 +4929,13 @@
         <v>0.7828628545575615</v>
       </c>
       <c r="Q46" t="n">
-        <v>1.48</v>
+        <v>1.49</v>
       </c>
       <c r="R46" t="n">
         <v>4.75</v>
       </c>
       <c r="S46" t="n">
-        <v>4.85</v>
+        <v>4.8</v>
       </c>
       <c r="T46" t="inlineStr">
         <is>
@@ -4943,10 +4943,10 @@
         </is>
       </c>
       <c r="U46" t="n">
-        <v>0.02712990490408584</v>
+        <v>0.03406997182911353</v>
       </c>
       <c r="V46" t="n">
-        <v>1.122023929055304</v>
+        <v>1.127136878071534</v>
       </c>
       <c r="W46" t="inlineStr">
         <is>
@@ -4992,13 +4992,13 @@
         <v>0.6401931479937157</v>
       </c>
       <c r="H47" t="n">
-        <v>0.8186038226791237</v>
+        <v>0.8146526621225523</v>
       </c>
       <c r="I47" t="n">
-        <v>0.1227207654112213</v>
+        <v>0.1249248932118969</v>
       </c>
       <c r="J47" t="n">
-        <v>0.05867541190965522</v>
+        <v>0.06042244466555097</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
@@ -5025,13 +5025,13 @@
         <v>0.4312886156726625</v>
       </c>
       <c r="Q47" t="n">
-        <v>1.05</v>
+        <v>1.06</v>
       </c>
       <c r="R47" t="n">
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="S47" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="T47" t="inlineStr">
         <is>
@@ -5039,10 +5039,10 @@
         </is>
       </c>
       <c r="U47" t="n">
-        <v>0.8983869847782044</v>
+        <v>0.7401880693800207</v>
       </c>
       <c r="V47" t="n">
-        <v>2.06788582270483</v>
+        <v>1.894805122542774</v>
       </c>
       <c r="W47" t="inlineStr">
         <is>
@@ -5088,13 +5088,13 @@
         <v>1.122130451557203</v>
       </c>
       <c r="H48" t="n">
-        <v>0.617658793695226</v>
+        <v>0.6205984655606609</v>
       </c>
       <c r="I48" t="n">
-        <v>0.1993292969365545</v>
+        <v>0.1991554261006111</v>
       </c>
       <c r="J48" t="n">
-        <v>0.1830119093682194</v>
+        <v>0.1802461083387279</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
@@ -5121,13 +5121,13 @@
         <v>0.6237414999623524</v>
       </c>
       <c r="Q48" t="n">
-        <v>1.66</v>
+        <v>1.64</v>
       </c>
       <c r="R48" t="n">
         <v>4.05</v>
       </c>
       <c r="S48" t="n">
-        <v>4.15</v>
+        <v>4.25</v>
       </c>
       <c r="T48" t="inlineStr">
         <is>
@@ -5135,10 +5135,10 @@
         </is>
       </c>
       <c r="U48" t="n">
-        <v>0.1334375634174001</v>
+        <v>0.1197816891593591</v>
       </c>
       <c r="V48" t="n">
-        <v>1.235772324832596</v>
+        <v>1.222761063375407</v>
       </c>
       <c r="W48" t="inlineStr">
         <is>
@@ -5422,13 +5422,13 @@
         <v>1.11264099148167</v>
       </c>
       <c r="H52" t="n">
-        <v>0.4841126219674445</v>
+        <v>0.4803788043011803</v>
       </c>
       <c r="I52" t="n">
-        <v>0.2555822614866745</v>
+        <v>0.2563071412520317</v>
       </c>
       <c r="J52" t="n">
-        <v>0.260305116545881</v>
+        <v>0.263314054446788</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -5455,13 +5455,13 @@
         <v>0.5397465778429353</v>
       </c>
       <c r="Q52" t="n">
-        <v>1.91</v>
+        <v>1.94</v>
       </c>
       <c r="R52" t="n">
-        <v>3.55</v>
+        <v>3.53</v>
       </c>
       <c r="S52" t="n">
-        <v>3.53</v>
+        <v>3.45</v>
       </c>
       <c r="T52" t="inlineStr">
         <is>
@@ -5469,10 +5469,10 @@
         </is>
       </c>
       <c r="U52" t="n">
-        <v>-0.06935445747800495</v>
+        <v>-0.05473698822373285</v>
       </c>
       <c r="V52" t="n">
-        <v>1.013041612979514</v>
+        <v>1.029018143939741</v>
       </c>
       <c r="W52" t="inlineStr">
         <is>
@@ -5518,13 +5518,13 @@
         <v>1.529136542215973</v>
       </c>
       <c r="H53" t="n">
-        <v>0.3476949077166279</v>
+        <v>0.3450140909904484</v>
       </c>
       <c r="I53" t="n">
-        <v>0.2604458696801017</v>
+        <v>0.2606020765315394</v>
       </c>
       <c r="J53" t="n">
-        <v>0.3918592226032703</v>
+        <v>0.394383832478012</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -5551,13 +5551,13 @@
         <v>0.6284429767793762</v>
       </c>
       <c r="Q53" t="n">
-        <v>3.07</v>
+        <v>3.12</v>
       </c>
       <c r="R53" t="n">
-        <v>3.28</v>
+        <v>3.27</v>
       </c>
       <c r="S53" t="n">
-        <v>2.18</v>
+        <v>2.15</v>
       </c>
       <c r="T53" t="inlineStr">
         <is>
@@ -5565,10 +5565,10 @@
         </is>
       </c>
       <c r="U53" t="n">
-        <v>0.2168483559556409</v>
+        <v>0.2366667330884691</v>
       </c>
       <c r="V53" t="n">
-        <v>1.325545214327768</v>
+        <v>1.349746917287028</v>
       </c>
       <c r="W53" t="inlineStr">
         <is>
@@ -5710,13 +5710,13 @@
         <v>1.427558893552563</v>
       </c>
       <c r="H55" t="n">
-        <v>0.5844085925793456</v>
+        <v>0.5884338750138116</v>
       </c>
       <c r="I55" t="n">
-        <v>0.2090441961508707</v>
+        <v>0.2077994676938826</v>
       </c>
       <c r="J55" t="n">
-        <v>0.2065472112697838</v>
+        <v>0.2037666572923059</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
@@ -5743,13 +5743,13 @@
         <v>0.6893569696047046</v>
       </c>
       <c r="Q55" t="n">
-        <v>1.56</v>
+        <v>1.54</v>
       </c>
       <c r="R55" t="n">
-        <v>4.15</v>
+        <v>4.2</v>
       </c>
       <c r="S55" t="n">
-        <v>4.85</v>
+        <v>5</v>
       </c>
       <c r="T55" t="inlineStr">
         <is>
@@ -5757,10 +5757,10 @@
         </is>
       </c>
       <c r="U55" t="n">
-        <v>0.08453816809205472</v>
+        <v>0.118080585661912</v>
       </c>
       <c r="V55" t="n">
-        <v>1.180167389885801</v>
+        <v>1.215852134711136</v>
       </c>
       <c r="W55" t="inlineStr">
         <is>
@@ -5902,13 +5902,13 @@
         <v>1.768893310395192</v>
       </c>
       <c r="H57" t="n">
-        <v>0.6557815228140289</v>
+        <v>0.6670833285928683</v>
       </c>
       <c r="I57" t="n">
-        <v>0.1618550034864507</v>
+        <v>0.1631442062324047</v>
       </c>
       <c r="J57" t="n">
-        <v>0.1823634736995204</v>
+        <v>0.169772465174727</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
@@ -5935,13 +5935,13 @@
         <v>0.7874684227946003</v>
       </c>
       <c r="Q57" t="n">
-        <v>1.27</v>
+        <v>1.25</v>
       </c>
       <c r="R57" t="n">
         <v>5.6</v>
       </c>
       <c r="S57" t="n">
-        <v>5.75</v>
+        <v>7</v>
       </c>
       <c r="T57" t="inlineStr">
         <is>
@@ -5949,10 +5949,10 @@
         </is>
       </c>
       <c r="U57" t="n">
-        <v>0.2198992730762395</v>
+        <v>0.485094767223248</v>
       </c>
       <c r="V57" t="n">
-        <v>1.390546159945527</v>
+        <v>1.665427703243214</v>
       </c>
       <c r="W57" t="inlineStr">
         <is>
@@ -5998,13 +5998,13 @@
         <v>1.411562315208403</v>
       </c>
       <c r="H58" t="n">
-        <v>0.6848498312407429</v>
+        <v>0.6838066333099266</v>
       </c>
       <c r="I58" t="n">
-        <v>0.1632685428552959</v>
+        <v>0.1630326894100678</v>
       </c>
       <c r="J58" t="n">
-        <v>0.151881625903961</v>
+        <v>0.1531606772800054</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
@@ -6037,7 +6037,7 @@
         <v>5.75</v>
       </c>
       <c r="S58" t="n">
-        <v>6.9</v>
+        <v>6.75</v>
       </c>
       <c r="T58" t="inlineStr">
         <is>
@@ -6045,10 +6045,10 @@
         </is>
       </c>
       <c r="U58" t="n">
-        <v>0.1769090604254822</v>
+        <v>0.151324080851015</v>
       </c>
       <c r="V58" t="n">
-        <v>1.280561028957938</v>
+        <v>1.256430713773993</v>
       </c>
       <c r="W58" t="inlineStr">
         <is>
@@ -6428,13 +6428,13 @@
         <v>1.267735705596107</v>
       </c>
       <c r="H63" t="n">
-        <v>0.3871767943875938</v>
+        <v>0.3879651593083796</v>
       </c>
       <c r="I63" t="n">
-        <v>0.2637691963598924</v>
+        <v>0.2643097894484312</v>
       </c>
       <c r="J63" t="n">
-        <v>0.3490540092525139</v>
+        <v>0.3477250512431893</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -6467,7 +6467,7 @@
         <v>3.5</v>
       </c>
       <c r="S63" t="n">
-        <v>2.57</v>
+        <v>2.6</v>
       </c>
       <c r="T63" t="inlineStr">
         <is>
@@ -6478,7 +6478,7 @@
         <v>-0.05773353692045224</v>
       </c>
       <c r="V63" t="n">
-        <v>1.028470662847109</v>
+        <v>1.024240193841963</v>
       </c>
       <c r="W63" t="inlineStr">
         <is>
@@ -6620,13 +6620,13 @@
         <v>1.768677962550518</v>
       </c>
       <c r="H65" t="n">
-        <v>0.3351926848105896</v>
+        <v>0.3363776908280009</v>
       </c>
       <c r="I65" t="n">
-        <v>0.2605573656327125</v>
+        <v>0.2609578695852443</v>
       </c>
       <c r="J65" t="n">
-        <v>0.4042499495566981</v>
+        <v>0.402664439586755</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
@@ -6653,13 +6653,13 @@
         <v>0.6515954800796417</v>
       </c>
       <c r="Q65" t="n">
-        <v>2.72</v>
+        <v>2.7</v>
       </c>
       <c r="R65" t="n">
-        <v>3.18</v>
+        <v>3.17</v>
       </c>
       <c r="S65" t="n">
-        <v>2.45</v>
+        <v>2.47</v>
       </c>
       <c r="T65" t="inlineStr">
         <is>
@@ -6667,10 +6667,10 @@
         </is>
       </c>
       <c r="U65" t="n">
-        <v>0.06362558036865673</v>
+        <v>0.07230823816758458</v>
       </c>
       <c r="V65" t="n">
-        <v>1.159645159204515</v>
+        <v>1.169551672285884</v>
       </c>
       <c r="W65" t="inlineStr">
         <is>
@@ -6954,13 +6954,13 @@
         <v>1.523965627828707</v>
       </c>
       <c r="H69" t="n">
-        <v>0.2924266152569004</v>
+        <v>0.2892484885230557</v>
       </c>
       <c r="I69" t="n">
-        <v>0.2667927711945851</v>
+        <v>0.2667127154849229</v>
       </c>
       <c r="J69" t="n">
-        <v>0.4407806135485146</v>
+        <v>0.4440387959920215</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -6987,13 +6987,13 @@
         <v>0.5650680958204189</v>
       </c>
       <c r="Q69" t="n">
-        <v>3.4</v>
+        <v>3.48</v>
       </c>
       <c r="R69" t="n">
         <v>3.3</v>
       </c>
       <c r="S69" t="n">
-        <v>2.03</v>
+        <v>2</v>
       </c>
       <c r="T69" t="inlineStr">
         <is>
@@ -7001,14 +7001,14 @@
         </is>
       </c>
       <c r="U69" t="n">
-        <v>0.07086672243593584</v>
+        <v>0.09606358649325197</v>
       </c>
       <c r="V69" t="n">
-        <v>1.166986421045387</v>
+        <v>1.195133074718609</v>
       </c>
       <c r="W69" t="inlineStr">
         <is>
-          <t>Pas de valeur</t>
+          <t>PARI VALUE</t>
         </is>
       </c>
       <c r="X69" t="inlineStr">
@@ -7050,13 +7050,13 @@
         <v>1.336616924815223</v>
       </c>
       <c r="H70" t="n">
-        <v>0.3684347049803396</v>
+        <v>0.3668931670451754</v>
       </c>
       <c r="I70" t="n">
-        <v>0.2756944229118428</v>
+        <v>0.2713044609164587</v>
       </c>
       <c r="J70" t="n">
-        <v>0.3558708721078176</v>
+        <v>0.3618023720383659</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -7083,13 +7083,13 @@
         <v>0.545531836322639</v>
       </c>
       <c r="Q70" t="n">
-        <v>2.48</v>
+        <v>2.5</v>
       </c>
       <c r="R70" t="n">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
       <c r="S70" t="n">
-        <v>2.67</v>
+        <v>2.58</v>
       </c>
       <c r="T70" t="inlineStr">
         <is>
@@ -7097,10 +7097,10 @@
         </is>
       </c>
       <c r="U70" t="n">
-        <v>-0.01686393502099315</v>
+        <v>-0.05000335294163372</v>
       </c>
       <c r="V70" t="n">
-        <v>1.07187160763255</v>
+        <v>1.036092185333001</v>
       </c>
       <c r="W70" t="inlineStr">
         <is>
@@ -7146,13 +7146,13 @@
         <v>1.368315802227365</v>
       </c>
       <c r="H71" t="n">
-        <v>0.2497539289071898</v>
+        <v>0.2490123519273592</v>
       </c>
       <c r="I71" t="n">
-        <v>0.2792914535068446</v>
+        <v>0.2803825366425882</v>
       </c>
       <c r="J71" t="n">
-        <v>0.4709546175859657</v>
+        <v>0.4706051114300527</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -7179,10 +7179,10 @@
         <v>0.4706324666789738</v>
       </c>
       <c r="Q71" t="n">
-        <v>3.98</v>
+        <v>4</v>
       </c>
       <c r="R71" t="n">
-        <v>3.28</v>
+        <v>3.25</v>
       </c>
       <c r="S71" t="n">
         <v>1.88</v>
@@ -7193,10 +7193,10 @@
         </is>
       </c>
       <c r="U71" t="n">
-        <v>0.06896520831136255</v>
+        <v>0.07433689277523881</v>
       </c>
       <c r="V71" t="n">
-        <v>1.163086765177241</v>
+        <v>1.170605215000189</v>
       </c>
       <c r="W71" t="inlineStr">
         <is>
@@ -7242,13 +7242,13 @@
         <v>1.013619913753882</v>
       </c>
       <c r="H72" t="n">
-        <v>0.5661858587164007</v>
+        <v>0.5665423877353174</v>
       </c>
       <c r="I72" t="n">
-        <v>0.2396549356510249</v>
+        <v>0.2392016344698308</v>
       </c>
       <c r="J72" t="n">
-        <v>0.1941592056325745</v>
+        <v>0.1942559777948519</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -7278,7 +7278,7 @@
         <v>1.52</v>
       </c>
       <c r="R72" t="n">
-        <v>3.93</v>
+        <v>3.95</v>
       </c>
       <c r="S72" t="n">
         <v>5.6</v>
@@ -7292,7 +7292,7 @@
         <v>0.2579248397181069</v>
       </c>
       <c r="V72" t="n">
-        <v>1.37229422347426</v>
+        <v>1.3706735517962</v>
       </c>
       <c r="W72" t="inlineStr">
         <is>
@@ -7338,13 +7338,13 @@
         <v>1.610986105612227</v>
       </c>
       <c r="H73" t="n">
-        <v>0.5079921563290901</v>
+        <v>0.5082861979877756</v>
       </c>
       <c r="I73" t="n">
-        <v>0.2187722437034678</v>
+        <v>0.2182988181397981</v>
       </c>
       <c r="J73" t="n">
-        <v>0.2732355999674421</v>
+        <v>0.2734149838724264</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
@@ -7374,7 +7374,7 @@
         <v>1.94</v>
       </c>
       <c r="R73" t="n">
-        <v>3.83</v>
+        <v>3.85</v>
       </c>
       <c r="S73" t="n">
         <v>3.18</v>
@@ -7388,7 +7388,7 @@
         <v>0.0544410684111063</v>
       </c>
       <c r="V73" t="n">
-        <v>1.150422549481312</v>
+        <v>1.148992362551861</v>
       </c>
       <c r="W73" t="inlineStr">
         <is>
@@ -7434,13 +7434,13 @@
         <v>1.567579328799631</v>
       </c>
       <c r="H74" t="n">
-        <v>0.5093202293765956</v>
+        <v>0.5100489355869083</v>
       </c>
       <c r="I74" t="n">
-        <v>0.2322423959841554</v>
+        <v>0.2318411981829721</v>
       </c>
       <c r="J74" t="n">
-        <v>0.258437374639249</v>
+        <v>0.2581098662301197</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -7467,7 +7467,7 @@
         <v>0.6733258878586383</v>
       </c>
       <c r="Q74" t="n">
-        <v>1.69</v>
+        <v>1.68</v>
       </c>
       <c r="R74" t="n">
         <v>4</v>
@@ -7484,7 +7484,7 @@
         <v>0.5764783098007162</v>
       </c>
       <c r="V74" t="n">
-        <v>1.648677247005392</v>
+        <v>1.654229791066397</v>
       </c>
       <c r="W74" t="inlineStr">
         <is>
@@ -7530,13 +7530,13 @@
         <v>1.618079317628398</v>
       </c>
       <c r="H75" t="n">
-        <v>0.4176928842061265</v>
+        <v>0.413744993839997</v>
       </c>
       <c r="I75" t="n">
-        <v>0.2577052329435578</v>
+        <v>0.257771719087045</v>
       </c>
       <c r="J75" t="n">
-        <v>0.3246018828503156</v>
+        <v>0.328483287072958</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
@@ -7563,13 +7563,13 @@
         <v>0.6609433151648293</v>
       </c>
       <c r="Q75" t="n">
-        <v>2.08</v>
+        <v>2.12</v>
       </c>
       <c r="R75" t="n">
         <v>3.15</v>
       </c>
       <c r="S75" t="n">
-        <v>3.1</v>
+        <v>3.02</v>
       </c>
       <c r="T75" t="inlineStr">
         <is>
@@ -7577,14 +7577,14 @@
         </is>
       </c>
       <c r="U75" t="n">
-        <v>0.1203199451413177</v>
+        <v>0.09140846268605785</v>
       </c>
       <c r="V75" t="n">
-        <v>1.255666014373454</v>
+        <v>1.222687720321703</v>
       </c>
       <c r="W75" t="inlineStr">
         <is>
-          <t>Ecart suspect</t>
+          <t>Pas de valeur</t>
         </is>
       </c>
       <c r="X75" t="inlineStr">
@@ -7818,13 +7818,13 @@
         <v>1.054941555353019</v>
       </c>
       <c r="H78" t="n">
-        <v>0.546080348201736</v>
+        <v>0.5452602994467879</v>
       </c>
       <c r="I78" t="n">
-        <v>0.2378351727371213</v>
+        <v>0.238929722022673</v>
       </c>
       <c r="J78" t="n">
-        <v>0.2160844790611429</v>
+        <v>0.2158099785305392</v>
       </c>
       <c r="K78" t="inlineStr">
         <is>
@@ -7854,7 +7854,7 @@
         <v>1.59</v>
       </c>
       <c r="R78" t="n">
-        <v>4.05</v>
+        <v>4</v>
       </c>
       <c r="S78" t="n">
         <v>4.75</v>
@@ -7868,7 +7868,7 @@
         <v>0.1323064557438824</v>
       </c>
       <c r="V78" t="n">
-        <v>1.230104572392964</v>
+        <v>1.23359934540452</v>
       </c>
       <c r="W78" t="inlineStr">
         <is>
@@ -7914,13 +7914,13 @@
         <v>2.037331410174504</v>
       </c>
       <c r="H79" t="n">
-        <v>0.3152438824044571</v>
+        <v>0.3086431366980612</v>
       </c>
       <c r="I79" t="n">
-        <v>0.236897270335737</v>
+        <v>0.2380756636838965</v>
       </c>
       <c r="J79" t="n">
-        <v>0.4478588472598058</v>
+        <v>0.4532811996180423</v>
       </c>
       <c r="K79" t="inlineStr">
         <is>
@@ -7929,7 +7929,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>Faible</t>
+          <t>Moyenne</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
@@ -7947,24 +7947,24 @@
         <v>0.6489241778337835</v>
       </c>
       <c r="Q79" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="R79" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="S79" t="n">
         <v>2.43</v>
       </c>
-      <c r="R79" t="n">
-        <v>3.58</v>
-      </c>
-      <c r="S79" t="n">
-        <v>2.5</v>
-      </c>
       <c r="T79" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
       <c r="U79" t="n">
-        <v>0.3225797988422339</v>
+        <v>0.2855475644746515</v>
       </c>
       <c r="V79" t="n">
-        <v>1.442739139694815</v>
+        <v>1.401295916447371</v>
       </c>
       <c r="W79" t="inlineStr">
         <is>
@@ -8106,13 +8106,13 @@
         <v>0.9939750569230624</v>
       </c>
       <c r="H81" t="n">
-        <v>0.6053560665447039</v>
+        <v>0.6111275863238642</v>
       </c>
       <c r="I81" t="n">
-        <v>0.2182778382128666</v>
+        <v>0.2168676430606303</v>
       </c>
       <c r="J81" t="n">
-        <v>0.1763660952424296</v>
+        <v>0.1720047706155056</v>
       </c>
       <c r="K81" t="inlineStr">
         <is>
@@ -8139,13 +8139,13 @@
         <v>0.5536122953975022</v>
       </c>
       <c r="Q81" t="n">
-        <v>1.56</v>
+        <v>1.53</v>
       </c>
       <c r="R81" t="n">
-        <v>4</v>
+        <v>4.05</v>
       </c>
       <c r="S81" t="n">
-        <v>5</v>
+        <v>5.25</v>
       </c>
       <c r="T81" t="inlineStr">
         <is>
@@ -8153,10 +8153,10 @@
         </is>
       </c>
       <c r="U81" t="n">
-        <v>-0.02785781503622309</v>
+        <v>-0.0465528570547572</v>
       </c>
       <c r="V81" t="n">
-        <v>1.060632050518172</v>
+        <v>1.040196094533891</v>
       </c>
       <c r="W81" t="inlineStr">
         <is>
@@ -8273,13 +8273,13 @@
         <v>1.912431955956947</v>
       </c>
       <c r="H83" t="n">
-        <v>0.2818933743778043</v>
+        <v>0.2825838862537052</v>
       </c>
       <c r="I83" t="n">
-        <v>0.2324589583894952</v>
+        <v>0.233131833143186</v>
       </c>
       <c r="J83" t="n">
-        <v>0.4856476672327006</v>
+        <v>0.4842842806031089</v>
       </c>
       <c r="K83" t="inlineStr">
         <is>
@@ -8306,13 +8306,13 @@
         <v>0.6780798948880914</v>
       </c>
       <c r="Q83" t="n">
-        <v>3.75</v>
+        <v>3.73</v>
       </c>
       <c r="R83" t="n">
-        <v>3.8</v>
+        <v>3.78</v>
       </c>
       <c r="S83" t="n">
-        <v>1.78</v>
+        <v>1.79</v>
       </c>
       <c r="T83" t="inlineStr">
         <is>
@@ -8320,10 +8320,10 @@
         </is>
       </c>
       <c r="U83" t="n">
-        <v>0.1981325552964233</v>
+        <v>0.1917425150015091</v>
       </c>
       <c r="V83" t="n">
-        <v>1.307908232746015</v>
+        <v>1.300555753706785</v>
       </c>
       <c r="W83" t="inlineStr">
         <is>
@@ -8369,13 +8369,13 @@
         <v>1.559880014539196</v>
       </c>
       <c r="H84" t="n">
-        <v>0.1891619977052077</v>
+        <v>0.1890718988665879</v>
       </c>
       <c r="I84" t="n">
-        <v>0.2456703159351602</v>
+        <v>0.2461232288890273</v>
       </c>
       <c r="J84" t="n">
-        <v>0.565167686359632</v>
+        <v>0.5648048722443847</v>
       </c>
       <c r="K84" t="inlineStr">
         <is>
@@ -8405,7 +8405,7 @@
         <v>6</v>
       </c>
       <c r="R84" t="n">
-        <v>3.95</v>
+        <v>3.93</v>
       </c>
       <c r="S84" t="n">
         <v>1.49</v>
@@ -8419,7 +8419,7 @@
         <v>0.3533303009981377</v>
       </c>
       <c r="V84" t="n">
-        <v>1.476445686039242</v>
+        <v>1.478189275179575</v>
       </c>
       <c r="W84" t="inlineStr">
         <is>
@@ -8536,13 +8536,13 @@
         <v>1.749070691683812</v>
       </c>
       <c r="H86" t="n">
-        <v>0.4772579361640552</v>
+        <v>0.4703053404823286</v>
       </c>
       <c r="I86" t="n">
-        <v>0.2312694749860071</v>
+        <v>0.2318460427335339</v>
       </c>
       <c r="J86" t="n">
-        <v>0.2914725888499377</v>
+        <v>0.2978486167841373</v>
       </c>
       <c r="K86" t="inlineStr">
         <is>
@@ -8569,13 +8569,13 @@
         <v>0.7520466936701869</v>
       </c>
       <c r="Q86" t="n">
-        <v>2.12</v>
+        <v>2.2</v>
       </c>
       <c r="R86" t="n">
         <v>3.45</v>
       </c>
       <c r="S86" t="n">
-        <v>3.03</v>
+        <v>2.92</v>
       </c>
       <c r="T86" t="inlineStr">
         <is>
@@ -8583,10 +8583,10 @@
         </is>
       </c>
       <c r="U86" t="n">
-        <v>0.1074755802109986</v>
+        <v>0.1492671115397155</v>
       </c>
       <c r="V86" t="n">
-        <v>1.208905047981686</v>
+        <v>1.24909967074416</v>
       </c>
       <c r="W86" t="inlineStr">
         <is>
@@ -9087,13 +9087,13 @@
         <v>1.172842116194884</v>
       </c>
       <c r="H92" t="n">
-        <v>0.561128576051344</v>
+        <v>0.5626817573286196</v>
       </c>
       <c r="I92" t="n">
-        <v>0.2266550593521447</v>
+        <v>0.2272171630524921</v>
       </c>
       <c r="J92" t="n">
-        <v>0.2122163645965112</v>
+        <v>0.2101010796188883</v>
       </c>
       <c r="K92" t="inlineStr">
         <is>
@@ -9126,7 +9126,7 @@
         <v>4.2</v>
       </c>
       <c r="S92" t="n">
-        <v>5.1</v>
+        <v>5.25</v>
       </c>
       <c r="T92" t="inlineStr">
         <is>
@@ -9134,10 +9134,10 @@
         </is>
       </c>
       <c r="U92" t="n">
-        <v>0.2489133650538371</v>
+        <v>0.2856461110848323</v>
       </c>
       <c r="V92" t="n">
-        <v>1.363898828193469</v>
+        <v>1.39681100038916</v>
       </c>
       <c r="W92" t="inlineStr">
         <is>
@@ -9183,13 +9183,13 @@
         <v>1.712704896346409</v>
       </c>
       <c r="H93" t="n">
-        <v>0.3945396440631941</v>
+        <v>0.39439954914394</v>
       </c>
       <c r="I93" t="n">
-        <v>0.2582950814008343</v>
+        <v>0.2595519108926334</v>
       </c>
       <c r="J93" t="n">
-        <v>0.3471652745359715</v>
+        <v>0.3460485399634265</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -9219,10 +9219,10 @@
         <v>2.25</v>
       </c>
       <c r="R93" t="n">
-        <v>3.2</v>
+        <v>3.17</v>
       </c>
       <c r="S93" t="n">
-        <v>3</v>
+        <v>3.02</v>
       </c>
       <c r="T93" t="inlineStr">
         <is>
@@ -9230,10 +9230,10 @@
         </is>
       </c>
       <c r="U93" t="n">
-        <v>0.1657941949865296</v>
+        <v>0.1735661562864399</v>
       </c>
       <c r="V93" t="n">
-        <v>1.271039504256147</v>
+        <v>1.280393167283978</v>
       </c>
       <c r="W93" t="inlineStr">
         <is>
@@ -9471,13 +9471,13 @@
         <v>1.578568129405063</v>
       </c>
       <c r="H96" t="n">
-        <v>0.3690228014926289</v>
+        <v>0.366443813744595</v>
       </c>
       <c r="I96" t="n">
-        <v>0.2432301786716001</v>
+        <v>0.2429576940387355</v>
       </c>
       <c r="J96" t="n">
-        <v>0.387747019835771</v>
+        <v>0.3905984922166695</v>
       </c>
       <c r="K96" t="inlineStr">
         <is>
@@ -9504,13 +9504,13 @@
         <v>0.6729792714700736</v>
       </c>
       <c r="Q96" t="n">
-        <v>3.15</v>
+        <v>3.2</v>
       </c>
       <c r="R96" t="n">
         <v>3.53</v>
       </c>
       <c r="S96" t="n">
-        <v>2.05</v>
+        <v>2.02</v>
       </c>
       <c r="T96" t="inlineStr">
         <is>
@@ -9518,10 +9518,10 @@
         </is>
       </c>
       <c r="U96" t="n">
-        <v>0.4061915044018494</v>
+        <v>0.4285120044717201</v>
       </c>
       <c r="V96" t="n">
-        <v>1.530711610540274</v>
+        <v>1.558271783690354</v>
       </c>
       <c r="W96" t="inlineStr">
         <is>
@@ -9830,13 +9830,13 @@
         <v>2.456568352541854</v>
       </c>
       <c r="H100" t="n">
-        <v>0.3153854595295835</v>
+        <v>0.3129504330693437</v>
       </c>
       <c r="I100" t="n">
-        <v>0.2221495333613384</v>
+        <v>0.2231921667236118</v>
       </c>
       <c r="J100" t="n">
-        <v>0.4624650071090782</v>
+        <v>0.4638574002070445</v>
       </c>
       <c r="K100" t="inlineStr">
         <is>
@@ -9863,13 +9863,13 @@
         <v>0.7272349907651137</v>
       </c>
       <c r="Q100" t="n">
-        <v>2.37</v>
+        <v>2.4</v>
       </c>
       <c r="R100" t="n">
-        <v>3.68</v>
+        <v>3.65</v>
       </c>
       <c r="S100" t="n">
-        <v>2.6</v>
+        <v>2.58</v>
       </c>
       <c r="T100" t="inlineStr">
         <is>
@@ -9877,10 +9877,10 @@
         </is>
       </c>
       <c r="U100" t="n">
-        <v>0.4774284182919459</v>
+        <v>0.4660635843050849</v>
       </c>
       <c r="V100" t="n">
-        <v>1.59310433127599</v>
+        <v>1.580762782110838</v>
       </c>
       <c r="W100" t="inlineStr">
         <is>
@@ -10068,13 +10068,13 @@
         <v>1.48417037089417</v>
       </c>
       <c r="H103" t="n">
-        <v>0.4664907897836355</v>
+        <v>0.4329040979634901</v>
       </c>
       <c r="I103" t="n">
-        <v>0.2278023084471008</v>
+        <v>0.2533453277974168</v>
       </c>
       <c r="J103" t="n">
-        <v>0.3057069017692637</v>
+        <v>0.3137505742390931</v>
       </c>
       <c r="K103" t="inlineStr">
         <is>
@@ -10083,7 +10083,7 @@
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>Moyenne</t>
+          <t>Faible</t>
         </is>
       </c>
       <c r="M103" t="inlineStr">
@@ -10100,9 +10100,34 @@
       <c r="P103" t="n">
         <v>0.6561499962820434</v>
       </c>
+      <c r="Q103" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="R103" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="S103" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U103" t="n">
+        <v>0.02627973752399804</v>
+      </c>
+      <c r="V103" t="n">
+        <v>1.168220524842779</v>
+      </c>
       <c r="W103" t="inlineStr">
         <is>
-          <t>Pas de cote</t>
+          <t>Pas de valeur</t>
+        </is>
+      </c>
+      <c r="X103" t="inlineStr">
+        <is>
+          <t>Betclic</t>
         </is>
       </c>
     </row>
@@ -10210,13 +10235,13 @@
         <v>1.430353886066146</v>
       </c>
       <c r="H105" t="n">
-        <v>0.4216292406861701</v>
+        <v>0.4847345683706593</v>
       </c>
       <c r="I105" t="n">
-        <v>0.2433947650600129</v>
+        <v>0.2458537329107767</v>
       </c>
       <c r="J105" t="n">
-        <v>0.3349759942538171</v>
+        <v>0.2694116987185641</v>
       </c>
       <c r="K105" t="inlineStr">
         <is>
@@ -10225,7 +10250,7 @@
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>Faible</t>
+          <t>Moyenne</t>
         </is>
       </c>
       <c r="M105" t="inlineStr">
@@ -10242,9 +10267,34 @@
       <c r="P105" t="n">
         <v>0.6138174288447785</v>
       </c>
+      <c r="Q105" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="R105" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="S105" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U105" t="n">
+        <v>0.4403967752914133</v>
+      </c>
+      <c r="V105" t="n">
+        <v>1.643268391074807</v>
+      </c>
       <c r="W105" t="inlineStr">
         <is>
-          <t>Pas de cote</t>
+          <t>Ecart suspect</t>
+        </is>
+      </c>
+      <c r="X105" t="inlineStr">
+        <is>
+          <t>Betclic</t>
         </is>
       </c>
     </row>
@@ -10281,13 +10331,13 @@
         <v>1.24404783964945</v>
       </c>
       <c r="H106" t="n">
-        <v>0.5169046793321698</v>
+        <v>0.4983022202529153</v>
       </c>
       <c r="I106" t="n">
-        <v>0.230514390352963</v>
+        <v>0.2470665890124874</v>
       </c>
       <c r="J106" t="n">
-        <v>0.2525809303148668</v>
+        <v>0.2546311907345971</v>
       </c>
       <c r="K106" t="inlineStr">
         <is>
@@ -10313,9 +10363,34 @@
       <c r="P106" t="n">
         <v>0.6034477764651902</v>
       </c>
+      <c r="Q106" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="R106" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="S106" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U106" t="n">
+        <v>-0.05406443682212925</v>
+      </c>
+      <c r="V106" t="n">
+        <v>1.07755875897766</v>
+      </c>
       <c r="W106" t="inlineStr">
         <is>
-          <t>Pas de cote</t>
+          <t>Pas de valeur</t>
+        </is>
+      </c>
+      <c r="X106" t="inlineStr">
+        <is>
+          <t>Betclic</t>
         </is>
       </c>
     </row>
@@ -10423,13 +10498,13 @@
         <v>1.829096938422859</v>
       </c>
       <c r="H108" t="n">
-        <v>0.3307015210891077</v>
+        <v>0.2956599318448822</v>
       </c>
       <c r="I108" t="n">
-        <v>0.2285804287124483</v>
+        <v>0.2426942808129804</v>
       </c>
       <c r="J108" t="n">
-        <v>0.4407180501984441</v>
+        <v>0.4616457873421376</v>
       </c>
       <c r="K108" t="inlineStr">
         <is>
@@ -10438,7 +10513,7 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>Faible</t>
+          <t>Moyenne</t>
         </is>
       </c>
       <c r="M108" t="inlineStr">
@@ -10455,9 +10530,34 @@
       <c r="P108" t="n">
         <v>0.6656689788642458</v>
       </c>
+      <c r="Q108" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="R108" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="S108" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U108" t="n">
+        <v>0.1144641260702928</v>
+      </c>
+      <c r="V108" t="n">
+        <v>1.268911151030682</v>
+      </c>
       <c r="W108" t="inlineStr">
         <is>
-          <t>Pas de cote</t>
+          <t>Ecart suspect</t>
+        </is>
+      </c>
+      <c r="X108" t="inlineStr">
+        <is>
+          <t>Betclic</t>
         </is>
       </c>
     </row>
@@ -10494,13 +10594,13 @@
         <v>1.491975066709752</v>
       </c>
       <c r="H109" t="n">
-        <v>0.5030238591313618</v>
+        <v>0.5050889932187048</v>
       </c>
       <c r="I109" t="n">
-        <v>0.2215093513669412</v>
+        <v>0.2231207709864433</v>
       </c>
       <c r="J109" t="n">
-        <v>0.275466789501697</v>
+        <v>0.2717902357948519</v>
       </c>
       <c r="K109" t="inlineStr">
         <is>
@@ -10527,13 +10627,13 @@
         <v>0.7024078926980601</v>
       </c>
       <c r="Q109" t="n">
-        <v>2.1</v>
+        <v>2.08</v>
       </c>
       <c r="R109" t="n">
-        <v>3.78</v>
+        <v>3.73</v>
       </c>
       <c r="S109" t="n">
-        <v>2.95</v>
+        <v>3.02</v>
       </c>
       <c r="T109" t="inlineStr">
         <is>
@@ -10541,10 +10641,10 @@
         </is>
       </c>
       <c r="U109" t="n">
-        <v>0.1865374176540455</v>
+        <v>0.1752370612954357</v>
       </c>
       <c r="V109" t="n">
-        <v>1.281132679450696</v>
+        <v>1.269246122863136</v>
       </c>
       <c r="W109" t="inlineStr">
         <is>
@@ -10590,13 +10690,13 @@
         <v>0.8388993159386002</v>
       </c>
       <c r="H110" t="n">
-        <v>0.6720887358983385</v>
+        <v>0.6697708939688178</v>
       </c>
       <c r="I110" t="n">
-        <v>0.1974018801223755</v>
+        <v>0.1989615836614025</v>
       </c>
       <c r="J110" t="n">
-        <v>0.1305093839792862</v>
+        <v>0.1312675223697797</v>
       </c>
       <c r="K110" t="inlineStr">
         <is>
@@ -10626,10 +10726,10 @@
         <v>1.23</v>
       </c>
       <c r="R110" t="n">
-        <v>5.9</v>
+        <v>5.75</v>
       </c>
       <c r="S110" t="n">
-        <v>10.75</v>
+        <v>10.5</v>
       </c>
       <c r="T110" t="inlineStr">
         <is>
@@ -10637,10 +10737,10 @@
         </is>
       </c>
       <c r="U110" t="n">
-        <v>0.8761714696343508</v>
+        <v>0.8325395749916913</v>
       </c>
       <c r="V110" t="n">
-        <v>2.017865401154752</v>
+        <v>1.983099686515778</v>
       </c>
       <c r="W110" t="inlineStr">
         <is>
@@ -10686,13 +10786,13 @@
         <v>2.846947581180713</v>
       </c>
       <c r="H111" t="n">
-        <v>0.3966771018146482</v>
+        <v>0.3944686353189382</v>
       </c>
       <c r="I111" t="n">
-        <v>0.2059720404337906</v>
+        <v>0.2066689407529982</v>
       </c>
       <c r="J111" t="n">
-        <v>0.3973508577515614</v>
+        <v>0.3988624239280636</v>
       </c>
       <c r="K111" t="inlineStr">
         <is>
@@ -10719,13 +10819,13 @@
         <v>0.8485437689991057</v>
       </c>
       <c r="Q111" t="n">
-        <v>1.95</v>
+        <v>1.97</v>
       </c>
       <c r="R111" t="n">
-        <v>3.95</v>
+        <v>3.93</v>
       </c>
       <c r="S111" t="n">
-        <v>3.18</v>
+        <v>3.15</v>
       </c>
       <c r="T111" t="inlineStr">
         <is>
@@ -10733,10 +10833,10 @@
         </is>
       </c>
       <c r="U111" t="n">
-        <v>0.6016115811288711</v>
+        <v>0.586502037910674</v>
       </c>
       <c r="V111" t="n">
-        <v>1.730461999342083</v>
+        <v>1.712672510299925</v>
       </c>
       <c r="W111" t="inlineStr">
         <is>
@@ -10782,13 +10882,13 @@
         <v>1.641562094661614</v>
       </c>
       <c r="H112" t="n">
-        <v>0.4429635312805151</v>
+        <v>0.4404661584494168</v>
       </c>
       <c r="I112" t="n">
-        <v>0.2425587281573245</v>
+        <v>0.2434056481609665</v>
       </c>
       <c r="J112" t="n">
-        <v>0.3144777405621603</v>
+        <v>0.3161281933896165</v>
       </c>
       <c r="K112" t="inlineStr">
         <is>
@@ -10815,13 +10915,13 @@
         <v>0.6931786695436087</v>
       </c>
       <c r="Q112" t="n">
-        <v>2.13</v>
+        <v>2.15</v>
       </c>
       <c r="R112" t="n">
-        <v>3.5</v>
+        <v>3.47</v>
       </c>
       <c r="S112" t="n">
-        <v>3.07</v>
+        <v>3.03</v>
       </c>
       <c r="T112" t="inlineStr">
         <is>
@@ -10829,10 +10929,10 @@
         </is>
       </c>
       <c r="U112" t="n">
-        <v>0.005764684538395404</v>
+        <v>-0.007339741318782456</v>
       </c>
       <c r="V112" t="n">
-        <v>1.087161977610017</v>
+        <v>1.075382331140717</v>
       </c>
       <c r="W112" t="inlineStr">
         <is>
@@ -10840,6 +10940,674 @@
         </is>
       </c>
       <c r="X112" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Feyenoord</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>2.151149444380951</v>
+      </c>
+      <c r="G113" t="n">
+        <v>1.728280072399264</v>
+      </c>
+      <c r="H113" t="n">
+        <v>0.3721800080718713</v>
+      </c>
+      <c r="I113" t="n">
+        <v>0.221043500660688</v>
+      </c>
+      <c r="J113" t="n">
+        <v>0.4067764912674406</v>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Victoire Como</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>Inter-champ.</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>2 - 1</t>
+        </is>
+      </c>
+      <c r="N113" t="n">
+        <v>0.9007128221379019</v>
+      </c>
+      <c r="O113" t="n">
+        <v>0.7436877051214856</v>
+      </c>
+      <c r="P113" t="n">
+        <v>0.7282572103198369</v>
+      </c>
+      <c r="Q113" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="R113" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="S113" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U113" t="n">
+        <v>0.6569872632742242</v>
+      </c>
+      <c r="V113" t="n">
+        <v>1.789515192374834</v>
+      </c>
+      <c r="W113" t="inlineStr">
+        <is>
+          <t>Ecart suspect</t>
+        </is>
+      </c>
+      <c r="X113" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Portsmouth</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Sheffield Utd</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>1.762628517226536</v>
+      </c>
+      <c r="G114" t="n">
+        <v>1.669211441991185</v>
+      </c>
+      <c r="H114" t="n">
+        <v>0.4049151912302197</v>
+      </c>
+      <c r="I114" t="n">
+        <v>0.2288220538274281</v>
+      </c>
+      <c r="J114" t="n">
+        <v>0.3662627549423524</v>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Victoire Portsmouth</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N114" t="n">
+        <v>0.8586318092515689</v>
+      </c>
+      <c r="O114" t="n">
+        <v>0.6663603295388084</v>
+      </c>
+      <c r="P114" t="n">
+        <v>0.6742402870041125</v>
+      </c>
+      <c r="W114" t="inlineStr">
+        <is>
+          <t>Pas de cote</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Norwich</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Southampton</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>2.035968695462377</v>
+      </c>
+      <c r="G115" t="n">
+        <v>2.417343213892737</v>
+      </c>
+      <c r="H115" t="n">
+        <v>0.3329388101210415</v>
+      </c>
+      <c r="I115" t="n">
+        <v>0.1948075938445686</v>
+      </c>
+      <c r="J115" t="n">
+        <v>0.47225359603439</v>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Victoire Southampton</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>2 - 2</t>
+        </is>
+      </c>
+      <c r="N115" t="n">
+        <v>0.9376659912213764</v>
+      </c>
+      <c r="O115" t="n">
+        <v>0.8210920582778795</v>
+      </c>
+      <c r="P115" t="n">
+        <v>0.7930689179936222</v>
+      </c>
+      <c r="W115" t="inlineStr">
+        <is>
+          <t>Pas de cote</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>QPR</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Derby County</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>2.026882234322699</v>
+      </c>
+      <c r="G116" t="n">
+        <v>1.622009710986557</v>
+      </c>
+      <c r="H116" t="n">
+        <v>0.4725030703360488</v>
+      </c>
+      <c r="I116" t="n">
+        <v>0.2170190295872018</v>
+      </c>
+      <c r="J116" t="n">
+        <v>0.3104779000767495</v>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Victoire QPR</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N116" t="n">
+        <v>0.8807457063050608</v>
+      </c>
+      <c r="O116" t="n">
+        <v>0.7058128488496682</v>
+      </c>
+      <c r="P116" t="n">
+        <v>0.6984826316052337</v>
+      </c>
+      <c r="W116" t="inlineStr">
+        <is>
+          <t>Pas de cote</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Lincoln City</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>West Ham</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>1.49105461098188</v>
+      </c>
+      <c r="G117" t="n">
+        <v>2.020759301948158</v>
+      </c>
+      <c r="H117" t="n">
+        <v>0.2832896083763405</v>
+      </c>
+      <c r="I117" t="n">
+        <v>0.2185981394705664</v>
+      </c>
+      <c r="J117" t="n">
+        <v>0.4981122521530933</v>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>Victoire West Ham</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N117" t="n">
+        <v>0.8671522188577089</v>
+      </c>
+      <c r="O117" t="n">
+        <v>0.6813292828113284</v>
+      </c>
+      <c r="P117" t="n">
+        <v>0.6739501928737288</v>
+      </c>
+      <c r="W117" t="inlineStr">
+        <is>
+          <t>Pas de cote</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Roma</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Real Madrid</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>1.712606582738095</v>
+      </c>
+      <c r="G118" t="n">
+        <v>1.278122006324338</v>
+      </c>
+      <c r="H118" t="n">
+        <v>0.3680757434738996</v>
+      </c>
+      <c r="I118" t="n">
+        <v>0.2385034849789181</v>
+      </c>
+      <c r="J118" t="n">
+        <v>0.3934207715471821</v>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>Victoire Real Madrid</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>Inter-champ.</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N118" t="n">
+        <v>0.8016621405353836</v>
+      </c>
+      <c r="O118" t="n">
+        <v>0.5747286477684252</v>
+      </c>
+      <c r="P118" t="n">
+        <v>0.5934955268083245</v>
+      </c>
+      <c r="Q118" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="R118" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="S118" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="T118" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U118" t="n">
+        <v>0.6737312917365996</v>
+      </c>
+      <c r="V118" t="n">
+        <v>1.80966723831707</v>
+      </c>
+      <c r="W118" t="inlineStr">
+        <is>
+          <t>Ecart suspect</t>
+        </is>
+      </c>
+      <c r="X118" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Manchester City</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>1.950986740415254</v>
+      </c>
+      <c r="G119" t="n">
+        <v>1.436401073617317</v>
+      </c>
+      <c r="H119" t="n">
+        <v>0.4561722853790539</v>
+      </c>
+      <c r="I119" t="n">
+        <v>0.2321784258386375</v>
+      </c>
+      <c r="J119" t="n">
+        <v>0.3116492887823086</v>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>Victoire Manchester City</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>Inter-champ.</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>1 - 1</t>
+        </is>
+      </c>
+      <c r="N119" t="n">
+        <v>0.8536133570631234</v>
+      </c>
+      <c r="O119" t="n">
+        <v>0.6578185496552342</v>
+      </c>
+      <c r="P119" t="n">
+        <v>0.6557745798914788</v>
+      </c>
+      <c r="Q119" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="R119" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="S119" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="T119" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U119" t="n">
+        <v>0.09762153779073457</v>
+      </c>
+      <c r="V119" t="n">
+        <v>1.183057949514344</v>
+      </c>
+      <c r="W119" t="inlineStr">
+        <is>
+          <t>Pas de valeur</t>
+        </is>
+      </c>
+      <c r="X119" t="inlineStr">
+        <is>
+          <t>Betclic</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Real Betis</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Porto</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>0.7593921974108753</v>
+      </c>
+      <c r="G120" t="n">
+        <v>2.018315688628648</v>
+      </c>
+      <c r="H120" t="n">
+        <v>0.2848532124814295</v>
+      </c>
+      <c r="I120" t="n">
+        <v>0.2326914089632512</v>
+      </c>
+      <c r="J120" t="n">
+        <v>0.4824553785553194</v>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Victoire Porto</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>Inter-champ.</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>0 - 2</t>
+        </is>
+      </c>
+      <c r="N120" t="n">
+        <v>0.7670028167029931</v>
+      </c>
+      <c r="O120" t="n">
+        <v>0.5252112891956778</v>
+      </c>
+      <c r="P120" t="n">
+        <v>0.4632564832637176</v>
+      </c>
+      <c r="Q120" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="R120" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="S120" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="T120" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U120" t="n">
+        <v>1.065692710278863</v>
+      </c>
+      <c r="V120" t="n">
+        <v>2.231900953058705</v>
+      </c>
+      <c r="W120" t="inlineStr">
+        <is>
+          <t>Ecart suspect</t>
+        </is>
+      </c>
+      <c r="X120" t="inlineStr">
         <is>
           <t>Betclic</t>
         </is>
@@ -10856,7 +11624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K112"/>
+  <dimension ref="A1:K120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10868,7 +11636,7 @@
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
     <col width="29" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -10950,26 +11718,9 @@
           <t>Bragantino - Mirassol</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>12 (pas de nul)</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>0.7618961130020734</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1.215532286212915</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1.312514899255404</v>
-      </c>
-      <c r="I2" t="n">
-        <v>-0.07389067590585663</v>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Cote insuffisante</t>
+          <t>Aucune selection a ce seuil</t>
         </is>
       </c>
     </row>
@@ -11000,16 +11751,16 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.7436188211217682</v>
+        <v>0.7421200660485252</v>
       </c>
       <c r="G3" t="n">
-        <v>1.270396975425331</v>
+        <v>1.276470588235294</v>
       </c>
       <c r="H3" t="n">
-        <v>1.344774999765974</v>
+        <v>1.347490851884084</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.0553088987775554</v>
+        <v>-0.05270556274982363</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -11098,16 +11849,16 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.7588369494822158</v>
+        <v>0.7624273137611287</v>
       </c>
       <c r="G6" t="n">
-        <v>1.239859437751004</v>
+        <v>1.224431137724551</v>
       </c>
       <c r="H6" t="n">
-        <v>1.317806151482659</v>
+        <v>1.311600439741465</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.05914884647029295</v>
+        <v>-0.06646025677918799</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -11142,16 +11893,16 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.7397436234601936</v>
+        <v>0.7406976724485281</v>
       </c>
       <c r="G7" t="n">
-        <v>1.235168738898757</v>
+        <v>1.230604982206406</v>
       </c>
       <c r="H7" t="n">
-        <v>1.351819695751404</v>
+        <v>1.350078496526518</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.08629180150227578</v>
+        <v>-0.08849375397615289</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -11186,16 +11937,16 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.7434966917709676</v>
+        <v>0.7431639603535124</v>
       </c>
       <c r="G8" t="n">
-        <v>1.220348432055749</v>
+        <v>1.217513134851138</v>
       </c>
       <c r="H8" t="n">
-        <v>1.344995897181541</v>
+        <v>1.345598082453183</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.09267497795866309</v>
+        <v>-0.095188116921608</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -11480,16 +12231,16 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.7303894826169589</v>
+        <v>0.7308085926095103</v>
       </c>
       <c r="G17" t="n">
-        <v>1.304310344827586</v>
+        <v>1.299057692307692</v>
       </c>
       <c r="H17" t="n">
-        <v>1.369132529697767</v>
+        <v>1.368347348557142</v>
       </c>
       <c r="I17" t="n">
-        <v>-0.04734544206943214</v>
+        <v>-0.05063747616605729</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -11693,16 +12444,16 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.7367800574742798</v>
+        <v>0.7364461381320331</v>
       </c>
       <c r="G23" t="n">
-        <v>1.268810916179337</v>
+        <v>1.273039215686275</v>
       </c>
       <c r="H23" t="n">
-        <v>1.357257148663947</v>
+        <v>1.357872556079201</v>
       </c>
       <c r="I23" t="n">
-        <v>-0.06516542025339433</v>
+        <v>-0.06247518591721068</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -11737,16 +12488,16 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.7325976171551107</v>
+        <v>0.7310975808339861</v>
       </c>
       <c r="G24" t="n">
-        <v>1.281257142857143</v>
+        <v>1.288162878787879</v>
       </c>
       <c r="H24" t="n">
-        <v>1.365005804800854</v>
+        <v>1.367806468268256</v>
       </c>
       <c r="I24" t="n">
-        <v>-0.06135407017989181</v>
+        <v>-0.05822723559803855</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -11781,16 +12532,16 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>0.7727619643484639</v>
+        <v>0.7718922089755194</v>
       </c>
       <c r="G25" t="n">
-        <v>1.212676056338028</v>
+        <v>1.214457831325301</v>
       </c>
       <c r="H25" t="n">
-        <v>1.294059550204605</v>
+        <v>1.2955176751003</v>
       </c>
       <c r="I25" t="n">
-        <v>-0.06289006858587676</v>
+        <v>-0.06256946187069456</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -11852,16 +12603,16 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>0.7691465596785085</v>
+        <v>0.7679003148447996</v>
       </c>
       <c r="G27" t="n">
-        <v>1.219919191919192</v>
+        <v>1.226156941649899</v>
       </c>
       <c r="H27" t="n">
-        <v>1.3001423297245</v>
+        <v>1.302252363579393</v>
       </c>
       <c r="I27" t="n">
-        <v>-0.06170335044956721</v>
+        <v>-0.0584336984579058</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -11950,16 +12701,16 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0.7411130045760173</v>
+        <v>0.7376585177631791</v>
       </c>
       <c r="G30" t="n">
-        <v>1.204206500956023</v>
+        <v>1.215789473684211</v>
       </c>
       <c r="H30" t="n">
-        <v>1.349321889948604</v>
+        <v>1.355640822846221</v>
       </c>
       <c r="I30" t="n">
-        <v>-0.1075469019465092</v>
+        <v>-0.1031625389300296</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -12173,16 +12924,16 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>0.7117788837445219</v>
+        <v>0.7128054945975744</v>
       </c>
       <c r="G37" t="n">
-        <v>1.353982300884956</v>
+        <v>1.350799289520426</v>
       </c>
       <c r="H37" t="n">
-        <v>1.404930692435277</v>
+        <v>1.402907255315934</v>
       </c>
       <c r="I37" t="n">
-        <v>-0.03626398926626684</v>
+        <v>-0.03714284433134041</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -12244,16 +12995,16 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>0.7477104724177691</v>
+        <v>0.7473567239459802</v>
       </c>
       <c r="G39" t="n">
-        <v>1.252087475149106</v>
+        <v>1.256607495069033</v>
       </c>
       <c r="H39" t="n">
-        <v>1.337416067968711</v>
+        <v>1.338049110898588</v>
       </c>
       <c r="I39" t="n">
-        <v>-0.06380108244789051</v>
+        <v>-0.06086593919924277</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -12288,16 +13039,16 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>0.74870032084494</v>
+        <v>0.7485924336876135</v>
       </c>
       <c r="G40" t="n">
-        <v>1.24662</v>
+        <v>1.248</v>
       </c>
       <c r="H40" t="n">
-        <v>1.335647884952764</v>
+        <v>1.335840378554104</v>
       </c>
       <c r="I40" t="n">
-        <v>-0.0666552060282809</v>
+        <v>-0.06575664275785831</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -12332,16 +13083,16 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>0.7560178690581486</v>
+        <v>0.7551147066464349</v>
       </c>
       <c r="G41" t="n">
-        <v>1.231701030927835</v>
+        <v>1.236535162950257</v>
       </c>
       <c r="H41" t="n">
-        <v>1.322720058516349</v>
+        <v>1.32430211092184</v>
       </c>
       <c r="I41" t="n">
-        <v>-0.06881201128121328</v>
+        <v>-0.066274113170815</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -12403,16 +13154,16 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>0.7317396206011282</v>
+        <v>0.7303376512447299</v>
       </c>
       <c r="G43" t="n">
-        <v>1.245699831365936</v>
+        <v>1.250938566552901</v>
       </c>
       <c r="H43" t="n">
-        <v>1.366606333518601</v>
+        <v>1.369229695738237</v>
       </c>
       <c r="I43" t="n">
-        <v>-0.08847207801340085</v>
+        <v>-0.08639246545230506</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
@@ -12450,13 +13201,13 @@
         <v>0.7364086038126073</v>
       </c>
       <c r="G44" t="n">
-        <v>1.247736239173774</v>
+        <v>1.250879631681409</v>
       </c>
       <c r="H44" t="n">
         <v>1.35794176605583</v>
       </c>
       <c r="I44" t="n">
-        <v>-0.08115629818364745</v>
+        <v>-0.0788414768958654</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -12680,16 +13431,16 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>0.7444177385133255</v>
+        <v>0.7436928587479683</v>
       </c>
       <c r="G52" t="n">
-        <v>1.239393382352941</v>
+        <v>1.241743970315399</v>
       </c>
       <c r="H52" t="n">
-        <v>1.343331772288362</v>
+        <v>1.34464112198621</v>
       </c>
       <c r="I52" t="n">
-        <v>-0.07737358118044213</v>
+        <v>-0.07652387688308881</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -12724,16 +13475,16 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>0.7395541303198983</v>
+        <v>0.7393979234684604</v>
       </c>
       <c r="G53" t="n">
-        <v>1.274780952380952</v>
+        <v>1.272865275142315</v>
       </c>
       <c r="H53" t="n">
-        <v>1.352166067367434</v>
+        <v>1.352451728981162</v>
       </c>
       <c r="I53" t="n">
-        <v>-0.05723048141353315</v>
+        <v>-0.05884605870466164</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -13014,13 +13765,13 @@
         <v>0.7436987278148628</v>
       </c>
       <c r="G63" t="n">
-        <v>1.231926471990655</v>
+        <v>1.237014757714755</v>
       </c>
       <c r="H63" t="n">
         <v>1.34463051044635</v>
       </c>
       <c r="I63" t="n">
-        <v>-0.08381785001909758</v>
+        <v>-0.08003369839932595</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -13082,16 +13833,16 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>0.7394426343672877</v>
+        <v>0.7390421304147559</v>
       </c>
       <c r="G65" t="n">
-        <v>1.288974854932302</v>
+        <v>1.289941972920696</v>
       </c>
       <c r="H65" t="n">
-        <v>1.352369952072971</v>
+        <v>1.353102832498592</v>
       </c>
       <c r="I65" t="n">
-        <v>-0.04687703763566609</v>
+        <v>-0.04667853622127516</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
@@ -13224,16 +13975,16 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>0.733207228805415</v>
+        <v>0.7332872845150772</v>
       </c>
       <c r="G69" t="n">
-        <v>1.271086556169429</v>
+        <v>1.27007299270073</v>
       </c>
       <c r="H69" t="n">
-        <v>1.36387089585745</v>
+        <v>1.363721996981442</v>
       </c>
       <c r="I69" t="n">
-        <v>-0.06803014857919454</v>
+        <v>-0.06867162404654426</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -13268,16 +14019,16 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>0.7243055770881572</v>
+        <v>0.7286955390835413</v>
       </c>
       <c r="G70" t="n">
-        <v>1.285747572815534</v>
+        <v>1.269685039370079</v>
       </c>
       <c r="H70" t="n">
-        <v>1.380632748984463</v>
+        <v>1.372315248776835</v>
       </c>
       <c r="I70" t="n">
-        <v>-0.06872586228214728</v>
+        <v>-0.07478617576991287</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -13312,16 +14063,16 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>0.7207085464931555</v>
+        <v>0.7196174633574119</v>
       </c>
       <c r="G71" t="n">
-        <v>1.276860068259386</v>
+        <v>1.27891156462585</v>
       </c>
       <c r="H71" t="n">
-        <v>1.387523437686189</v>
+        <v>1.389627199059969</v>
       </c>
       <c r="I71" t="n">
-        <v>-0.07975603612962667</v>
+        <v>-0.07967290400548666</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -13359,13 +14110,13 @@
         <v>0.7538174238186578</v>
       </c>
       <c r="G72" t="n">
-        <v>1.216021591439419</v>
+        <v>1.217459404075821</v>
       </c>
       <c r="H72" t="n">
         <v>1.326581169926055</v>
       </c>
       <c r="I72" t="n">
-        <v>-0.08334173663327271</v>
+        <v>-0.08225788841576609</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -13400,16 +14151,16 @@
         </is>
       </c>
       <c r="F73" t="n">
-        <v>0.7812277562965322</v>
+        <v>0.781701181860202</v>
       </c>
       <c r="G73" t="n">
         <v>1.204921875</v>
       </c>
       <c r="H73" t="n">
-        <v>1.280036445121425</v>
+        <v>1.279261210300739</v>
       </c>
       <c r="I73" t="n">
-        <v>-0.05868158708113946</v>
+        <v>-0.0581111462632895</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
@@ -13444,16 +14195,16 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>0.7677576040158446</v>
+        <v>0.768158801817028</v>
       </c>
       <c r="G74" t="n">
-        <v>1.25660091047041</v>
+        <v>1.251063829787234</v>
       </c>
       <c r="H74" t="n">
-        <v>1.302494426325946</v>
+        <v>1.30181415305607</v>
       </c>
       <c r="I74" t="n">
-        <v>-0.03523509577310946</v>
+        <v>-0.03898430751401605</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -13488,16 +14239,16 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>0.7422947670564422</v>
+        <v>0.742228280912955</v>
       </c>
       <c r="G75" t="n">
-        <v>1.244787644787645</v>
+        <v>1.245603112840467</v>
       </c>
       <c r="H75" t="n">
-        <v>1.347173716400405</v>
+        <v>1.347294391383175</v>
       </c>
       <c r="I75" t="n">
-        <v>-0.07600064517761806</v>
+        <v>-0.07547814285659471</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
@@ -13589,13 +14340,13 @@
         <v>0.7567423739018653</v>
       </c>
       <c r="G78" t="n">
-        <v>1.216392958928378</v>
+        <v>1.212946931415357</v>
       </c>
       <c r="H78" t="n">
         <v>1.321453686865539</v>
       </c>
       <c r="I78" t="n">
-        <v>-0.07950390466302515</v>
+        <v>-0.08211165970376</v>
       </c>
       <c r="K78" t="inlineStr">
         <is>
@@ -13630,16 +14381,16 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>0.763102729664263</v>
+        <v>0.7619243363161035</v>
       </c>
       <c r="G79" t="n">
-        <v>1.232251521298174</v>
+        <v>1.237090909090909</v>
       </c>
       <c r="H79" t="n">
-        <v>1.310439553059865</v>
+        <v>1.312466280884254</v>
       </c>
       <c r="I79" t="n">
-        <v>-0.05966550046442243</v>
+        <v>-0.05743033012822385</v>
       </c>
       <c r="K79" t="inlineStr">
         <is>
@@ -13772,16 +14523,16 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>0.7675410416105048</v>
+        <v>0.766868166856814</v>
       </c>
       <c r="G83" t="n">
-        <v>1.207052441229656</v>
+        <v>1.209547101449275</v>
       </c>
       <c r="H83" t="n">
-        <v>1.302861926316975</v>
+        <v>1.304005099205944</v>
       </c>
       <c r="I83" t="n">
-        <v>-0.07353771198008685</v>
+        <v>-0.07243683158462133</v>
       </c>
       <c r="K83" t="inlineStr">
         <is>
@@ -13819,13 +14570,13 @@
         <v>0.7154791223096694</v>
       </c>
       <c r="G84" t="n">
-        <v>1.281118683806446</v>
+        <v>1.279607548079736</v>
       </c>
       <c r="H84" t="n">
         <v>1.397664821821574</v>
       </c>
       <c r="I84" t="n">
-        <v>-0.08338632853564532</v>
+        <v>-0.08446751459908231</v>
       </c>
       <c r="K84" t="inlineStr">
         <is>
@@ -13887,16 +14638,16 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>0.7687305250139929</v>
+        <v>0.768153957266466</v>
       </c>
       <c r="G86" t="n">
-        <v>1.247300970873787</v>
+        <v>1.2546875</v>
       </c>
       <c r="H86" t="n">
-        <v>1.300845962870796</v>
+        <v>1.30182236326501</v>
       </c>
       <c r="I86" t="n">
-        <v>-0.04116166980973102</v>
+        <v>-0.03620683174223105</v>
       </c>
       <c r="K86" t="inlineStr">
         <is>
@@ -14127,16 +14878,16 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>0.7417049185991655</v>
+        <v>0.7404480891073666</v>
       </c>
       <c r="G93" t="n">
-        <v>1.285714285714286</v>
+        <v>1.289373814041746</v>
       </c>
       <c r="H93" t="n">
-        <v>1.348245070140115</v>
+        <v>1.350533568403872</v>
       </c>
       <c r="I93" t="n">
-        <v>-0.04637939037250138</v>
+        <v>-0.04528562324771235</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -14259,16 +15010,16 @@
         </is>
       </c>
       <c r="F96" t="n">
-        <v>0.7567698213284</v>
+        <v>0.7570423059612645</v>
       </c>
       <c r="G96" t="n">
-        <v>1.241826923076923</v>
+        <v>1.238314176245211</v>
       </c>
       <c r="H96" t="n">
-        <v>1.321405758814014</v>
+        <v>1.320930141057621</v>
       </c>
       <c r="I96" t="n">
-        <v>-0.06022286130228016</v>
+        <v>-0.06254378051080189</v>
       </c>
       <c r="K96" t="inlineStr">
         <is>
@@ -14418,16 +15169,16 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>0.7778504666386616</v>
+        <v>0.7768078332763881</v>
       </c>
       <c r="G100" t="n">
-        <v>1.239839034205231</v>
+        <v>1.243373493975904</v>
       </c>
       <c r="H100" t="n">
-        <v>1.285594137805582</v>
+        <v>1.287319665382674</v>
       </c>
       <c r="I100" t="n">
-        <v>-0.0355906286866331</v>
+        <v>-0.03413773019128608</v>
       </c>
       <c r="K100" t="inlineStr">
         <is>
@@ -14510,9 +15261,26 @@
           <t>Millwall - Swansea</t>
         </is>
       </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>0.7466546722025831</v>
+      </c>
+      <c r="G103" t="n">
+        <v>1.218255578093306</v>
+      </c>
+      <c r="H103" t="n">
+        <v>1.339307228936323</v>
+      </c>
+      <c r="I103" t="n">
+        <v>-0.09038378067977393</v>
+      </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Aucune selection a ce seuil</t>
+          <t>Cote insuffisante</t>
         </is>
       </c>
     </row>
@@ -14678,16 +15446,16 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>0.724533210498303</v>
+        <v>0.7282097642051482</v>
       </c>
       <c r="G109" t="n">
-        <v>1.35</v>
+        <v>1.335352839931153</v>
       </c>
       <c r="H109" t="n">
-        <v>1.380198982614258</v>
+        <v>1.373230694168891</v>
       </c>
       <c r="I109" t="n">
-        <v>-0.02188016582729091</v>
+        <v>-0.02758302330305995</v>
       </c>
       <c r="K109" t="inlineStr">
         <is>
@@ -14725,13 +15493,13 @@
         <v>0.7331233133372206</v>
       </c>
       <c r="G110" t="n">
-        <v>1.268245422025781</v>
+        <v>1.260467888501898</v>
       </c>
       <c r="H110" t="n">
         <v>1.36402700856414</v>
       </c>
       <c r="I110" t="n">
-        <v>-0.07021971407969774</v>
+        <v>-0.0759216052263183</v>
       </c>
       <c r="K110" t="inlineStr">
         <is>
@@ -14766,16 +15534,16 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>0.7940279595662096</v>
+        <v>0.7933310592470019</v>
       </c>
       <c r="G111" t="n">
-        <v>1.208771929824561</v>
+        <v>1.21201171875</v>
       </c>
       <c r="H111" t="n">
-        <v>1.259401495819261</v>
+        <v>1.260507814920495</v>
       </c>
       <c r="I111" t="n">
-        <v>-0.04020129098049419</v>
+        <v>-0.03847345934428303</v>
       </c>
       <c r="K111" t="inlineStr">
         <is>
@@ -14810,20 +15578,307 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>0.7574412718426754</v>
+        <v>0.7565943518390333</v>
       </c>
       <c r="G112" t="n">
-        <v>1.257519230769231</v>
+        <v>1.257625482625483</v>
       </c>
       <c r="H112" t="n">
-        <v>1.320234369546878</v>
+        <v>1.321712219459909</v>
       </c>
       <c r="I112" t="n">
-        <v>-0.04750303447953108</v>
+        <v>-0.04848766311672148</v>
       </c>
       <c r="K112" t="inlineStr">
         <is>
           <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Feyenoord - Como</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>0.7789564993393119</v>
+      </c>
+      <c r="G113" t="n">
+        <v>1.206672932330827</v>
+      </c>
+      <c r="H113" t="n">
+        <v>1.283768735286464</v>
+      </c>
+      <c r="I113" t="n">
+        <v>-0.06005427678407649</v>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Portsmouth - Sheffield Utd</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Norwich - Southampton</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>QPR - Derby County</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Lincoln City - West Ham</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>Aucune selection a ce seuil</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Roma - Real Madrid</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>0.7614965150210817</v>
+      </c>
+      <c r="G118" t="n">
+        <v>1.209534450651769</v>
+      </c>
+      <c r="H118" t="n">
+        <v>1.313203646076194</v>
+      </c>
+      <c r="I118" t="n">
+        <v>-0.07894373103073926</v>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Manchester City - Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>12 (pas de nul)</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>0.7678215741613624</v>
+      </c>
+      <c r="G119" t="n">
+        <v>1.222348178137652</v>
+      </c>
+      <c r="H119" t="n">
+        <v>1.302385910544686</v>
+      </c>
+      <c r="I119" t="n">
+        <v>-0.06145469768907463</v>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>Cote insuffisante</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Real Betis - Porto</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>N2 (ne perd pas exterieur)</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>0.7151467875185705</v>
+      </c>
+      <c r="G120" t="n">
+        <v>1.654887218045113</v>
+      </c>
+      <c r="H120" t="n">
+        <v>1.398314328544799</v>
+      </c>
+      <c r="I120" t="n">
+        <v>0.1834872776905065</v>
+      </c>
+      <c r="J120" t="n">
+        <v>3.502268647077694</v>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>RETENU</t>
         </is>
       </c>
     </row>

</xml_diff>